<commit_message>
Add ensembl ids from sce_pb
</commit_message>
<xml_diff>
--- a/processed-data/21_Xenium/02_xenium_compile_custom/ERC_Xenium_select_custom_probes.xlsx
+++ b/processed-data/21_Xenium/02_xenium_compile_custom/ERC_Xenium_select_custom_probes.xlsx
@@ -351,41 +351,46 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:G101"/>
+  <dimension ref="A1:H101"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <sheetData>
     <row r="1" s="1" customFormat="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
+          <t>gene_id</t>
+        </is>
+      </c>
+      <c r="B1" s="1" t="inlineStr">
+        <is>
           <t>gene_name</t>
         </is>
       </c>
-      <c r="B1" s="1" t="inlineStr">
+      <c r="C1" s="1" t="inlineStr">
         <is>
           <t>in_base</t>
         </is>
       </c>
-      <c r="C1" s="1" t="inlineStr">
+      <c r="D1" s="1" t="inlineStr">
         <is>
           <t>n_goal</t>
         </is>
       </c>
-      <c r="D1" s="1" t="inlineStr">
+      <c r="E1" s="1" t="inlineStr">
         <is>
           <t>goals</t>
         </is>
       </c>
-      <c r="E1" s="1" t="inlineStr">
+      <c r="F1" s="1" t="inlineStr">
         <is>
           <t>targets</t>
         </is>
       </c>
-      <c r="F1" s="1" t="inlineStr">
+      <c r="G1" s="1" t="inlineStr">
         <is>
           <t>notes</t>
         </is>
       </c>
-      <c r="G1" s="1" t="inlineStr">
+      <c r="H1" s="1" t="inlineStr">
         <is>
           <t>yesprobe</t>
         </is>
@@ -394,3100 +399,3600 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
+          <t>ENSG00000181409</t>
+        </is>
+      </c>
+      <c r="B2" t="inlineStr">
+        <is>
           <t>AATK</t>
         </is>
       </c>
-      <c r="B2" t="b">
-        <v>0</v>
-      </c>
-      <c r="C2">
-        <v>1</v>
-      </c>
-      <c r="D2" t="inlineStr">
+      <c r="C2" t="b">
+        <v>0</v>
+      </c>
+      <c r="D2">
+        <v>1</v>
+      </c>
+      <c r="E2" t="inlineStr">
         <is>
           <t>Marker - cell type specific</t>
         </is>
       </c>
-      <c r="E2" t="inlineStr">
+      <c r="F2" t="inlineStr">
         <is>
           <t>OPC.5</t>
         </is>
       </c>
-      <c r="F2" t="inlineStr">
+      <c r="G2" t="inlineStr">
         <is>
           <t>OPC.5 specific Enrich genes t= 6.2</t>
         </is>
       </c>
-      <c r="G2" t="b">
+      <c r="H2" t="b">
         <v>1</v>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
+          <t>ENSG00000141338</t>
+        </is>
+      </c>
+      <c r="B3" t="inlineStr">
+        <is>
           <t>ABCA8</t>
         </is>
       </c>
-      <c r="B3" t="b">
-        <v>0</v>
-      </c>
-      <c r="C3">
-        <v>1</v>
-      </c>
-      <c r="D3" t="inlineStr">
+      <c r="C3" t="b">
+        <v>0</v>
+      </c>
+      <c r="D3">
+        <v>1</v>
+      </c>
+      <c r="E3" t="inlineStr">
         <is>
           <t>DEG - mediation</t>
         </is>
       </c>
-      <c r="E3" t="inlineStr">
+      <c r="F3" t="inlineStr">
         <is>
           <t>Astro.2</t>
         </is>
       </c>
-      <c r="F3" t="inlineStr">
+      <c r="G3" t="inlineStr">
         <is>
           <t>mediation gene: mediator Astro.2</t>
         </is>
       </c>
-      <c r="G3" t="b">
+      <c r="H3" t="b">
         <v>1</v>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
+          <t>ENSG00000069122</t>
+        </is>
+      </c>
+      <c r="B4" t="inlineStr">
+        <is>
           <t>ADGRF5</t>
         </is>
       </c>
-      <c r="B4" t="b">
-        <v>0</v>
-      </c>
-      <c r="C4">
-        <v>1</v>
-      </c>
-      <c r="D4" t="inlineStr">
+      <c r="C4" t="b">
+        <v>0</v>
+      </c>
+      <c r="D4">
+        <v>1</v>
+      </c>
+      <c r="E4" t="inlineStr">
         <is>
           <t>Marker - cell type specific</t>
         </is>
       </c>
-      <c r="E4" t="inlineStr">
+      <c r="F4" t="inlineStr">
         <is>
           <t>Oligo.5</t>
         </is>
       </c>
-      <c r="F4" t="inlineStr">
+      <c r="G4" t="inlineStr">
         <is>
           <t>Oligo.5 specific Enrich genes t= 10.4</t>
         </is>
       </c>
-      <c r="G4" t="b">
+      <c r="H4" t="b">
         <v>1</v>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
+          <t>ENSG00000043591</t>
+        </is>
+      </c>
+      <c r="B5" t="inlineStr">
+        <is>
           <t>ADRB1</t>
         </is>
       </c>
-      <c r="B5" t="b">
-        <v>0</v>
-      </c>
-      <c r="C5">
-        <v>1</v>
-      </c>
-      <c r="D5" t="inlineStr">
+      <c r="C5" t="b">
+        <v>0</v>
+      </c>
+      <c r="D5">
+        <v>1</v>
+      </c>
+      <c r="E5" t="inlineStr">
         <is>
           <t>Lit - NE receptors</t>
         </is>
       </c>
-      <c r="E5" t="inlineStr">
+      <c r="F5" t="inlineStr">
         <is>
           <t>Oligo, Astro</t>
         </is>
       </c>
-      <c r="F5" t="inlineStr">
+      <c r="G5" t="inlineStr">
         <is>
           <t>NA</t>
         </is>
       </c>
-      <c r="G5" t="b">
+      <c r="H5" t="b">
         <v>1</v>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
+          <t>ENSG00000163947</t>
+        </is>
+      </c>
+      <c r="B6" t="inlineStr">
+        <is>
           <t>ARHGEF3</t>
         </is>
       </c>
-      <c r="B6" t="b">
-        <v>0</v>
-      </c>
-      <c r="C6">
-        <v>1</v>
-      </c>
-      <c r="D6" t="inlineStr">
+      <c r="C6" t="b">
+        <v>0</v>
+      </c>
+      <c r="D6">
+        <v>1</v>
+      </c>
+      <c r="E6" t="inlineStr">
         <is>
           <t>Marker - cell type specific</t>
         </is>
       </c>
-      <c r="E6" t="inlineStr">
+      <c r="F6" t="inlineStr">
         <is>
           <t>Oligo.5</t>
         </is>
       </c>
-      <c r="F6" t="inlineStr">
+      <c r="G6" t="inlineStr">
         <is>
           <t>Oligo.5 specific MR genes - Oligo.5/Oligo.2: 2.851, Oligo.5 specific Enrich genes t= 12.26</t>
         </is>
       </c>
-      <c r="G6" t="b">
+      <c r="H6" t="b">
         <v>1</v>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
+          <t>ENSG00000206190</t>
+        </is>
+      </c>
+      <c r="B7" t="inlineStr">
+        <is>
           <t>ATP10A</t>
         </is>
       </c>
-      <c r="B7" t="b">
-        <v>0</v>
-      </c>
-      <c r="C7">
-        <v>1</v>
-      </c>
-      <c r="D7" t="inlineStr">
+      <c r="C7" t="b">
+        <v>0</v>
+      </c>
+      <c r="D7">
+        <v>1</v>
+      </c>
+      <c r="E7" t="inlineStr">
         <is>
           <t>DEG - ancestry</t>
         </is>
       </c>
-      <c r="E7" t="inlineStr">
-        <is>
-          <t>Oligo.3</t>
-        </is>
-      </c>
       <c r="F7" t="inlineStr">
         <is>
+          <t>Oligo.3</t>
+        </is>
+      </c>
+      <c r="G7" t="inlineStr">
+        <is>
           <t>DEG carrier top: Oligo.3 EA_up</t>
         </is>
       </c>
-      <c r="G7" t="b">
+      <c r="H7" t="b">
         <v>1</v>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
+          <t>ENSG00000064787</t>
+        </is>
+      </c>
+      <c r="B8" t="inlineStr">
+        <is>
           <t>BCAS1</t>
         </is>
       </c>
-      <c r="B8" t="b">
-        <v>0</v>
-      </c>
-      <c r="C8">
+      <c r="C8" t="b">
+        <v>0</v>
+      </c>
+      <c r="D8">
         <v>2</v>
       </c>
-      <c r="D8" t="inlineStr">
+      <c r="E8" t="inlineStr">
         <is>
           <t>Marker - cell type specific, Marker - SpD</t>
         </is>
       </c>
-      <c r="E8" t="inlineStr">
+      <c r="F8" t="inlineStr">
         <is>
           <t>Astro.3, WM.uf~Sp09D07</t>
         </is>
       </c>
-      <c r="F8" t="inlineStr">
+      <c r="G8" t="inlineStr">
         <is>
           <t>Astro.3 specific Enrich genes t= 8.31, SpD Enrich gene t=5.88</t>
         </is>
       </c>
-      <c r="G8" t="b">
+      <c r="H8" t="b">
         <v>1</v>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
+          <t>ENSG00000153162</t>
+        </is>
+      </c>
+      <c r="B9" t="inlineStr">
+        <is>
           <t>BMP6</t>
         </is>
       </c>
-      <c r="B9" t="b">
-        <v>0</v>
-      </c>
-      <c r="C9">
-        <v>1</v>
-      </c>
-      <c r="D9" t="inlineStr">
+      <c r="C9" t="b">
+        <v>0</v>
+      </c>
+      <c r="D9">
+        <v>1</v>
+      </c>
+      <c r="E9" t="inlineStr">
         <is>
           <t>DEG - ancestry</t>
         </is>
       </c>
-      <c r="E9" t="inlineStr">
-        <is>
-          <t>Oligo.3</t>
-        </is>
-      </c>
       <c r="F9" t="inlineStr">
         <is>
+          <t>Oligo.3</t>
+        </is>
+      </c>
+      <c r="G9" t="inlineStr">
+        <is>
           <t>DEG Ancestry op: Oligo.3 AA_down-EA_up*</t>
         </is>
       </c>
-      <c r="G9" t="b">
+      <c r="H9" t="b">
         <v>1</v>
       </c>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
+          <t>ENSG00000134508</t>
+        </is>
+      </c>
+      <c r="B10" t="inlineStr">
+        <is>
           <t>CABLES1</t>
         </is>
       </c>
-      <c r="B10" t="b">
-        <v>0</v>
-      </c>
-      <c r="C10">
-        <v>1</v>
-      </c>
-      <c r="D10" t="inlineStr">
+      <c r="C10" t="b">
+        <v>0</v>
+      </c>
+      <c r="D10">
+        <v>1</v>
+      </c>
+      <c r="E10" t="inlineStr">
         <is>
           <t>MOFA - Factor3</t>
         </is>
       </c>
-      <c r="E10" t="inlineStr">
-        <is>
-          <t>Oligo.3</t>
-        </is>
-      </c>
       <c r="F10" t="inlineStr">
         <is>
+          <t>Oligo.3</t>
+        </is>
+      </c>
+      <c r="G10" t="inlineStr">
+        <is>
           <t>MOFA Oligo.3 Factor3+</t>
         </is>
       </c>
-      <c r="G10" t="b">
+      <c r="H10" t="b">
         <v>1</v>
       </c>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
+          <t>ENSG00000160200</t>
+        </is>
+      </c>
+      <c r="B11" t="inlineStr">
+        <is>
           <t>CBS</t>
         </is>
       </c>
-      <c r="B11" t="b">
-        <v>0</v>
-      </c>
-      <c r="C11">
-        <v>1</v>
-      </c>
-      <c r="D11" t="inlineStr">
+      <c r="C11" t="b">
+        <v>0</v>
+      </c>
+      <c r="D11">
+        <v>1</v>
+      </c>
+      <c r="E11" t="inlineStr">
         <is>
           <t>DEG - ancestry</t>
         </is>
       </c>
-      <c r="E11" t="inlineStr">
-        <is>
-          <t>Oligo.3</t>
-        </is>
-      </c>
       <c r="F11" t="inlineStr">
         <is>
+          <t>Oligo.3</t>
+        </is>
+      </c>
+      <c r="G11" t="inlineStr">
+        <is>
           <t>DEG Ancestry op: Oligo.3 AA_up*-EA_down</t>
         </is>
       </c>
-      <c r="G11" t="b">
+      <c r="H11" t="b">
         <v>1</v>
       </c>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
+          <t>ENSG00000071991</t>
+        </is>
+      </c>
+      <c r="B12" t="inlineStr">
+        <is>
           <t>CDH19</t>
         </is>
       </c>
-      <c r="B12" t="b">
-        <v>0</v>
-      </c>
-      <c r="C12">
-        <v>1</v>
-      </c>
-      <c r="D12" t="inlineStr">
+      <c r="C12" t="b">
+        <v>0</v>
+      </c>
+      <c r="D12">
+        <v>1</v>
+      </c>
+      <c r="E12" t="inlineStr">
         <is>
           <t>MOFA - Factor3</t>
         </is>
       </c>
-      <c r="E12" t="inlineStr">
-        <is>
-          <t>Oligo.3</t>
-        </is>
-      </c>
       <c r="F12" t="inlineStr">
         <is>
+          <t>Oligo.3</t>
+        </is>
+      </c>
+      <c r="G12" t="inlineStr">
+        <is>
           <t>MOFA Oligo.3 Factor3-</t>
         </is>
       </c>
-      <c r="G12" t="b">
+      <c r="H12" t="b">
         <v>1</v>
       </c>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
+          <t>ENSG00000134389</t>
+        </is>
+      </c>
+      <c r="B13" t="inlineStr">
+        <is>
           <t>CFHR5</t>
         </is>
       </c>
-      <c r="B13" t="b">
-        <v>0</v>
-      </c>
-      <c r="C13">
-        <v>1</v>
-      </c>
-      <c r="D13" t="inlineStr">
+      <c r="C13" t="b">
+        <v>0</v>
+      </c>
+      <c r="D13">
+        <v>1</v>
+      </c>
+      <c r="E13" t="inlineStr">
         <is>
           <t>Marker - SpD</t>
         </is>
       </c>
-      <c r="E13" t="inlineStr">
+      <c r="F13" t="inlineStr">
         <is>
           <t>WM.uf_Sp09D07-WM_Sp09D06</t>
         </is>
       </c>
-      <c r="F13" t="inlineStr">
+      <c r="G13" t="inlineStr">
         <is>
           <t>SpD pw gene t=8.23</t>
         </is>
       </c>
-      <c r="G13" t="b">
+      <c r="H13" t="b">
         <v>1</v>
       </c>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
+          <t>ENSG00000133019</t>
+        </is>
+      </c>
+      <c r="B14" t="inlineStr">
+        <is>
           <t>CHRM3</t>
         </is>
       </c>
-      <c r="B14" t="b">
-        <v>0</v>
-      </c>
-      <c r="C14">
-        <v>1</v>
-      </c>
-      <c r="D14" t="inlineStr">
+      <c r="C14" t="b">
+        <v>0</v>
+      </c>
+      <c r="D14">
+        <v>1</v>
+      </c>
+      <c r="E14" t="inlineStr">
         <is>
           <t>DEG - mediation</t>
         </is>
       </c>
-      <c r="E14" t="inlineStr">
+      <c r="F14" t="inlineStr">
         <is>
           <t>Astro.3</t>
         </is>
       </c>
-      <c r="F14" t="inlineStr">
+      <c r="G14" t="inlineStr">
         <is>
           <t>mediation gene: mediator Astro.3</t>
         </is>
       </c>
-      <c r="G14" t="b">
+      <c r="H14" t="b">
         <v>1</v>
       </c>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
+          <t>ENSG00000171310</t>
+        </is>
+      </c>
+      <c r="B15" t="inlineStr">
+        <is>
           <t>CHST11</t>
         </is>
       </c>
-      <c r="B15" t="b">
-        <v>0</v>
-      </c>
-      <c r="C15">
-        <v>1</v>
-      </c>
-      <c r="D15" t="inlineStr">
+      <c r="C15" t="b">
+        <v>0</v>
+      </c>
+      <c r="D15">
+        <v>1</v>
+      </c>
+      <c r="E15" t="inlineStr">
         <is>
           <t>DEG - carrier</t>
         </is>
       </c>
-      <c r="E15" t="inlineStr">
-        <is>
-          <t>Oligo.3</t>
-        </is>
-      </c>
       <c r="F15" t="inlineStr">
         <is>
+          <t>Oligo.3</t>
+        </is>
+      </c>
+      <c r="G15" t="inlineStr">
+        <is>
           <t>DEG carrier top: Oligo.3 up</t>
         </is>
       </c>
-      <c r="G15" t="b">
+      <c r="H15" t="b">
         <v>1</v>
       </c>
     </row>
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
+          <t>ENSG00000174469</t>
+        </is>
+      </c>
+      <c r="B16" t="inlineStr">
+        <is>
           <t>CNTNAP2</t>
         </is>
       </c>
-      <c r="B16" t="b">
-        <v>0</v>
-      </c>
-      <c r="C16">
-        <v>1</v>
-      </c>
-      <c r="D16" t="inlineStr">
+      <c r="C16" t="b">
+        <v>0</v>
+      </c>
+      <c r="D16">
+        <v>1</v>
+      </c>
+      <c r="E16" t="inlineStr">
         <is>
           <t>Marker - cell type specific</t>
         </is>
       </c>
-      <c r="E16" t="inlineStr">
-        <is>
-          <t>Oligo.3</t>
-        </is>
-      </c>
       <c r="F16" t="inlineStr">
         <is>
+          <t>Oligo.3</t>
+        </is>
+      </c>
+      <c r="G16" t="inlineStr">
+        <is>
           <t>Oligo.3 specific MR genes - Oligo.3/Oligo.2: 1.055</t>
         </is>
       </c>
-      <c r="G16" t="b">
+      <c r="H16" t="b">
         <v>1</v>
       </c>
     </row>
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
+          <t>ENSG00000084636</t>
+        </is>
+      </c>
+      <c r="B17" t="inlineStr">
+        <is>
           <t>COL16A1</t>
         </is>
       </c>
-      <c r="B17" t="b">
-        <v>0</v>
-      </c>
-      <c r="C17">
-        <v>1</v>
-      </c>
-      <c r="D17" t="inlineStr">
+      <c r="C17" t="b">
+        <v>0</v>
+      </c>
+      <c r="D17">
+        <v>1</v>
+      </c>
+      <c r="E17" t="inlineStr">
         <is>
           <t>Marker - cell type specific</t>
         </is>
       </c>
-      <c r="E17" t="inlineStr">
+      <c r="F17" t="inlineStr">
         <is>
           <t>Astro.3</t>
         </is>
       </c>
-      <c r="F17" t="inlineStr">
+      <c r="G17" t="inlineStr">
         <is>
           <t>Astro.3 specific MR genes - Astro.3/Astro.2: 1.061</t>
         </is>
       </c>
-      <c r="G17" t="b">
+      <c r="H17" t="b">
         <v>1</v>
       </c>
     </row>
     <row r="18">
       <c r="A18" t="inlineStr">
         <is>
+          <t>ENSG00000124749</t>
+        </is>
+      </c>
+      <c r="B18" t="inlineStr">
+        <is>
           <t>COL21A1</t>
         </is>
       </c>
-      <c r="B18" t="b">
-        <v>0</v>
-      </c>
-      <c r="C18">
-        <v>1</v>
-      </c>
-      <c r="D18" t="inlineStr">
+      <c r="C18" t="b">
+        <v>0</v>
+      </c>
+      <c r="D18">
+        <v>1</v>
+      </c>
+      <c r="E18" t="inlineStr">
         <is>
           <t>DEG - carrier</t>
         </is>
       </c>
-      <c r="E18" t="inlineStr">
-        <is>
-          <t>Oligo.3</t>
-        </is>
-      </c>
       <c r="F18" t="inlineStr">
         <is>
+          <t>Oligo.3</t>
+        </is>
+      </c>
+      <c r="G18" t="inlineStr">
+        <is>
           <t>DEG carrier top: Oligo.3 up</t>
         </is>
       </c>
-      <c r="G18" t="b">
+      <c r="H18" t="b">
         <v>1</v>
       </c>
     </row>
     <row r="19">
       <c r="A19" t="inlineStr">
         <is>
+          <t>ENSG00000172428</t>
+        </is>
+      </c>
+      <c r="B19" t="inlineStr">
+        <is>
           <t>COPS9</t>
         </is>
       </c>
-      <c r="B19" t="b">
-        <v>0</v>
-      </c>
-      <c r="C19">
-        <v>1</v>
-      </c>
-      <c r="D19" t="inlineStr">
+      <c r="C19" t="b">
+        <v>0</v>
+      </c>
+      <c r="D19">
+        <v>1</v>
+      </c>
+      <c r="E19" t="inlineStr">
         <is>
           <t>Marker - SpD</t>
         </is>
       </c>
-      <c r="E19" t="inlineStr">
+      <c r="F19" t="inlineStr">
         <is>
           <t>LD~Sp09D02</t>
         </is>
       </c>
-      <c r="F19" t="inlineStr">
+      <c r="G19" t="inlineStr">
         <is>
           <t>SpD MeanRatio gene: LD~Sp09D02/Inhib~Sp09D09: 1.112</t>
         </is>
       </c>
-      <c r="G19" t="b">
+      <c r="H19" t="b">
         <v>1</v>
       </c>
     </row>
     <row r="20">
       <c r="A20" t="inlineStr">
         <is>
+          <t>ENSG00000157851</t>
+        </is>
+      </c>
+      <c r="B20" t="inlineStr">
+        <is>
           <t>DPYSL5</t>
         </is>
       </c>
-      <c r="B20" t="b">
-        <v>0</v>
-      </c>
-      <c r="C20">
-        <v>1</v>
-      </c>
-      <c r="D20" t="inlineStr">
+      <c r="C20" t="b">
+        <v>0</v>
+      </c>
+      <c r="D20">
+        <v>1</v>
+      </c>
+      <c r="E20" t="inlineStr">
         <is>
           <t>Marker - cell type global</t>
         </is>
       </c>
-      <c r="E20" t="inlineStr">
+      <c r="F20" t="inlineStr">
         <is>
           <t>Oligo.2</t>
         </is>
       </c>
-      <c r="F20" t="inlineStr">
+      <c r="G20" t="inlineStr">
         <is>
           <t>globl MR genes -  Oligo.2/Oligo.1: 1.557</t>
         </is>
       </c>
-      <c r="G20" t="b">
+      <c r="H20" t="b">
         <v>1</v>
       </c>
     </row>
     <row r="21">
       <c r="A21" t="inlineStr">
         <is>
+          <t>ENSG00000004975</t>
+        </is>
+      </c>
+      <c r="B21" t="inlineStr">
+        <is>
           <t>DVL2</t>
         </is>
       </c>
-      <c r="B21" t="b">
-        <v>0</v>
-      </c>
-      <c r="C21">
-        <v>1</v>
-      </c>
-      <c r="D21" t="inlineStr">
+      <c r="C21" t="b">
+        <v>0</v>
+      </c>
+      <c r="D21">
+        <v>1</v>
+      </c>
+      <c r="E21" t="inlineStr">
         <is>
           <t>DEG - ancestry</t>
         </is>
       </c>
-      <c r="E21" t="inlineStr">
-        <is>
-          <t>Oligo.3</t>
-        </is>
-      </c>
       <c r="F21" t="inlineStr">
         <is>
+          <t>Oligo.3</t>
+        </is>
+      </c>
+      <c r="G21" t="inlineStr">
+        <is>
           <t>DEG Ancestry op: Oligo.3 AA_up-EA_down*</t>
         </is>
       </c>
-      <c r="G21" t="b">
+      <c r="H21" t="b">
         <v>1</v>
       </c>
     </row>
     <row r="22">
       <c r="A22" t="inlineStr">
         <is>
+          <t>ENSG00000171617</t>
+        </is>
+      </c>
+      <c r="B22" t="inlineStr">
+        <is>
           <t>ENC1</t>
         </is>
       </c>
-      <c r="B22" t="b">
-        <v>0</v>
-      </c>
-      <c r="C22">
-        <v>1</v>
-      </c>
-      <c r="D22" t="inlineStr">
+      <c r="C22" t="b">
+        <v>0</v>
+      </c>
+      <c r="D22">
+        <v>1</v>
+      </c>
+      <c r="E22" t="inlineStr">
         <is>
           <t>DEG - mediation</t>
         </is>
       </c>
-      <c r="E22" t="inlineStr">
-        <is>
-          <t>Oligo.3</t>
-        </is>
-      </c>
       <c r="F22" t="inlineStr">
         <is>
+          <t>Oligo.3</t>
+        </is>
+      </c>
+      <c r="G22" t="inlineStr">
+        <is>
           <t>mediation gene: outcome Oligo.3</t>
         </is>
       </c>
-      <c r="G22" t="b">
+      <c r="H22" t="b">
         <v>1</v>
       </c>
     </row>
     <row r="23">
       <c r="A23" t="inlineStr">
         <is>
+          <t>ENSG00000178568</t>
+        </is>
+      </c>
+      <c r="B23" t="inlineStr">
+        <is>
           <t>ERBB4</t>
         </is>
       </c>
-      <c r="B23" t="b">
-        <v>0</v>
-      </c>
-      <c r="C23">
-        <v>1</v>
-      </c>
-      <c r="D23" t="inlineStr">
+      <c r="C23" t="b">
+        <v>0</v>
+      </c>
+      <c r="D23">
+        <v>1</v>
+      </c>
+      <c r="E23" t="inlineStr">
         <is>
           <t>Marker - cell type specific</t>
         </is>
       </c>
-      <c r="E23" t="inlineStr">
+      <c r="F23" t="inlineStr">
         <is>
           <t>Oligo.1</t>
         </is>
       </c>
-      <c r="F23" t="inlineStr">
+      <c r="G23" t="inlineStr">
         <is>
           <t>Oligo.1 specific Enrich genes t= 5.58</t>
         </is>
       </c>
-      <c r="G23" t="b">
+      <c r="H23" t="b">
         <v>1</v>
       </c>
     </row>
     <row r="24">
       <c r="A24" t="inlineStr">
         <is>
+          <t>ENSG00000182473</t>
+        </is>
+      </c>
+      <c r="B24" t="inlineStr">
+        <is>
           <t>EXOC7</t>
         </is>
       </c>
-      <c r="B24" t="b">
-        <v>0</v>
-      </c>
-      <c r="C24">
-        <v>1</v>
-      </c>
-      <c r="D24" t="inlineStr">
+      <c r="C24" t="b">
+        <v>0</v>
+      </c>
+      <c r="D24">
+        <v>1</v>
+      </c>
+      <c r="E24" t="inlineStr">
         <is>
           <t>Marker - cell type specific</t>
         </is>
       </c>
-      <c r="E24" t="inlineStr">
+      <c r="F24" t="inlineStr">
         <is>
           <t>OPC.5</t>
         </is>
       </c>
-      <c r="F24" t="inlineStr">
+      <c r="G24" t="inlineStr">
         <is>
           <t>OPC.5 specific Enrich genes t= 7.33</t>
         </is>
       </c>
-      <c r="G24" t="b">
+      <c r="H24" t="b">
         <v>1</v>
       </c>
     </row>
     <row r="25">
       <c r="A25" t="inlineStr">
         <is>
+          <t>ENSG00000144369</t>
+        </is>
+      </c>
+      <c r="B25" t="inlineStr">
+        <is>
           <t>FAM171B</t>
         </is>
       </c>
-      <c r="B25" t="b">
-        <v>0</v>
-      </c>
-      <c r="C25">
-        <v>1</v>
-      </c>
-      <c r="D25" t="inlineStr">
+      <c r="C25" t="b">
+        <v>0</v>
+      </c>
+      <c r="D25">
+        <v>1</v>
+      </c>
+      <c r="E25" t="inlineStr">
         <is>
           <t>Marker - cell type specific</t>
         </is>
       </c>
-      <c r="E25" t="inlineStr">
+      <c r="F25" t="inlineStr">
         <is>
           <t>Astro.1</t>
         </is>
       </c>
-      <c r="F25" t="inlineStr">
+      <c r="G25" t="inlineStr">
         <is>
           <t>Astro.1 specific Enrich genes t= 8.3</t>
         </is>
       </c>
-      <c r="G25" t="b">
+      <c r="H25" t="b">
         <v>1</v>
       </c>
     </row>
     <row r="26">
       <c r="A26" t="inlineStr">
         <is>
+          <t>ENSG00000182263</t>
+        </is>
+      </c>
+      <c r="B26" t="inlineStr">
+        <is>
           <t>FIGN</t>
         </is>
       </c>
-      <c r="B26" t="b">
-        <v>0</v>
-      </c>
-      <c r="C26">
-        <v>1</v>
-      </c>
-      <c r="D26" t="inlineStr">
+      <c r="C26" t="b">
+        <v>0</v>
+      </c>
+      <c r="D26">
+        <v>1</v>
+      </c>
+      <c r="E26" t="inlineStr">
         <is>
           <t>Marker - cell type specific</t>
         </is>
       </c>
-      <c r="E26" t="inlineStr">
+      <c r="F26" t="inlineStr">
         <is>
           <t>Oligo.1</t>
         </is>
       </c>
-      <c r="F26" t="inlineStr">
+      <c r="G26" t="inlineStr">
         <is>
           <t>Oligo.1 specific MR genes - Oligo.1/Oligo.4: 1.143</t>
         </is>
       </c>
-      <c r="G26" t="b">
+      <c r="H26" t="b">
         <v>1</v>
       </c>
     </row>
     <row r="27">
       <c r="A27" t="inlineStr">
         <is>
+          <t>ENSG00000170345</t>
+        </is>
+      </c>
+      <c r="B27" t="inlineStr">
+        <is>
           <t>FOS</t>
         </is>
       </c>
-      <c r="B27" t="b">
-        <v>0</v>
-      </c>
-      <c r="C27">
-        <v>1</v>
-      </c>
-      <c r="D27" t="inlineStr">
+      <c r="C27" t="b">
+        <v>0</v>
+      </c>
+      <c r="D27">
+        <v>1</v>
+      </c>
+      <c r="E27" t="inlineStr">
         <is>
           <t>DEG - carrier</t>
         </is>
       </c>
-      <c r="E27" t="inlineStr">
-        <is>
-          <t>Oligo.3</t>
-        </is>
-      </c>
       <c r="F27" t="inlineStr">
         <is>
+          <t>Oligo.3</t>
+        </is>
+      </c>
+      <c r="G27" t="inlineStr">
+        <is>
           <t>DEG carrier top: Oligo.3 up, DEG of interest: Oligo.3 up</t>
         </is>
       </c>
-      <c r="G27" t="b">
+      <c r="H27" t="b">
         <v>1</v>
       </c>
     </row>
     <row r="28">
       <c r="A28" t="inlineStr">
         <is>
+          <t>ENSG00000177283</t>
+        </is>
+      </c>
+      <c r="B28" t="inlineStr">
+        <is>
           <t>FZD8</t>
         </is>
       </c>
-      <c r="B28" t="b">
-        <v>0</v>
-      </c>
-      <c r="C28">
-        <v>1</v>
-      </c>
-      <c r="D28" t="inlineStr">
+      <c r="C28" t="b">
+        <v>0</v>
+      </c>
+      <c r="D28">
+        <v>1</v>
+      </c>
+      <c r="E28" t="inlineStr">
         <is>
           <t>DEG - mediation</t>
         </is>
       </c>
-      <c r="E28" t="inlineStr">
+      <c r="F28" t="inlineStr">
         <is>
           <t>Astro.2</t>
         </is>
       </c>
-      <c r="F28" t="inlineStr">
+      <c r="G28" t="inlineStr">
         <is>
           <t>mediation gene: mediator Astro.2</t>
         </is>
       </c>
-      <c r="G28" t="b">
+      <c r="H28" t="b">
         <v>1</v>
       </c>
     </row>
     <row r="29">
       <c r="A29" t="inlineStr">
         <is>
+          <t>ENSG00000147533</t>
+        </is>
+      </c>
+      <c r="B29" t="inlineStr">
+        <is>
           <t>GOLGA7</t>
         </is>
       </c>
-      <c r="B29" t="b">
-        <v>0</v>
-      </c>
-      <c r="C29">
-        <v>1</v>
-      </c>
-      <c r="D29" t="inlineStr">
+      <c r="C29" t="b">
+        <v>0</v>
+      </c>
+      <c r="D29">
+        <v>1</v>
+      </c>
+      <c r="E29" t="inlineStr">
         <is>
           <t>Marker - cell type specific</t>
         </is>
       </c>
-      <c r="E29" t="inlineStr">
+      <c r="F29" t="inlineStr">
         <is>
           <t>Oligo.1</t>
         </is>
       </c>
-      <c r="F29" t="inlineStr">
+      <c r="G29" t="inlineStr">
         <is>
           <t>Oligo.1 specific Enrich genes t= 5.54</t>
         </is>
       </c>
-      <c r="G29" t="b">
+      <c r="H29" t="b">
         <v>1</v>
       </c>
     </row>
     <row r="30">
       <c r="A30" t="inlineStr">
         <is>
+          <t>ENSG00000235984</t>
+        </is>
+      </c>
+      <c r="B30" t="inlineStr">
+        <is>
           <t>GPC5-AS1</t>
         </is>
       </c>
-      <c r="B30" t="b">
-        <v>0</v>
-      </c>
-      <c r="C30">
-        <v>1</v>
-      </c>
-      <c r="D30" t="inlineStr">
+      <c r="C30" t="b">
+        <v>0</v>
+      </c>
+      <c r="D30">
+        <v>1</v>
+      </c>
+      <c r="E30" t="inlineStr">
         <is>
           <t>Marker - cell type specific</t>
         </is>
       </c>
-      <c r="E30" t="inlineStr">
+      <c r="F30" t="inlineStr">
         <is>
           <t>Excit.L5.2</t>
         </is>
       </c>
-      <c r="F30" t="inlineStr">
+      <c r="G30" t="inlineStr">
         <is>
           <t>Excit.L5.2 specific MR genes - Excit.L5.2/Excit.L5.1: 13.028</t>
         </is>
       </c>
-      <c r="G30" t="b">
+      <c r="H30" t="b">
         <v>1</v>
       </c>
     </row>
     <row r="31">
       <c r="A31" t="inlineStr">
         <is>
+          <t>ENSG00000183098</t>
+        </is>
+      </c>
+      <c r="B31" t="inlineStr">
+        <is>
           <t>GPC6</t>
         </is>
       </c>
-      <c r="B31" t="b">
-        <v>0</v>
-      </c>
-      <c r="C31">
-        <v>1</v>
-      </c>
-      <c r="D31" t="inlineStr">
+      <c r="C31" t="b">
+        <v>0</v>
+      </c>
+      <c r="D31">
+        <v>1</v>
+      </c>
+      <c r="E31" t="inlineStr">
         <is>
           <t>MOFA - Factor3</t>
         </is>
       </c>
-      <c r="E31" t="inlineStr">
-        <is>
-          <t>Oligo.3</t>
-        </is>
-      </c>
       <c r="F31" t="inlineStr">
         <is>
+          <t>Oligo.3</t>
+        </is>
+      </c>
+      <c r="G31" t="inlineStr">
+        <is>
           <t>MOFA Oligo.3 Factor3+</t>
         </is>
       </c>
-      <c r="G31" t="b">
+      <c r="H31" t="b">
         <v>1</v>
       </c>
     </row>
     <row r="32">
       <c r="A32" t="inlineStr">
         <is>
+          <t>ENSG00000150625</t>
+        </is>
+      </c>
+      <c r="B32" t="inlineStr">
+        <is>
           <t>GPM6A</t>
         </is>
       </c>
-      <c r="B32" t="b">
-        <v>0</v>
-      </c>
-      <c r="C32">
+      <c r="C32" t="b">
+        <v>0</v>
+      </c>
+      <c r="D32">
         <v>2</v>
       </c>
-      <c r="D32" t="inlineStr">
+      <c r="E32" t="inlineStr">
         <is>
           <t>DEG - mediation, Marker - cell type specific</t>
         </is>
       </c>
-      <c r="E32" t="inlineStr">
-        <is>
-          <t>Oligo.3</t>
-        </is>
-      </c>
       <c r="F32" t="inlineStr">
         <is>
+          <t>Oligo.3</t>
+        </is>
+      </c>
+      <c r="G32" t="inlineStr">
+        <is>
           <t>Oligo.3 specific Enrich genes t= 9.66, mediation gene: outcome Oligo.3</t>
         </is>
       </c>
-      <c r="G32" t="b">
+      <c r="H32" t="b">
         <v>1</v>
       </c>
     </row>
     <row r="33">
       <c r="A33" t="inlineStr">
         <is>
+          <t>ENSG00000174948</t>
+        </is>
+      </c>
+      <c r="B33" t="inlineStr">
+        <is>
           <t>GPR149</t>
         </is>
       </c>
-      <c r="B33" t="b">
-        <v>0</v>
-      </c>
-      <c r="C33">
-        <v>1</v>
-      </c>
-      <c r="D33" t="inlineStr">
+      <c r="C33" t="b">
+        <v>0</v>
+      </c>
+      <c r="D33">
+        <v>1</v>
+      </c>
+      <c r="E33" t="inlineStr">
         <is>
           <t>DEG - carrier</t>
         </is>
       </c>
-      <c r="E33" t="inlineStr">
+      <c r="F33" t="inlineStr">
         <is>
           <t>Excit.L2_5.1</t>
         </is>
       </c>
-      <c r="F33" t="inlineStr">
+      <c r="G33" t="inlineStr">
         <is>
           <t>DEG carrier top:  Excit.L2_5.1 down</t>
         </is>
       </c>
-      <c r="G33" t="b">
+      <c r="H33" t="b">
         <v>1</v>
       </c>
     </row>
     <row r="34">
       <c r="A34" t="inlineStr">
         <is>
+          <t>ENSG00000244734</t>
+        </is>
+      </c>
+      <c r="B34" t="inlineStr">
+        <is>
           <t>HBB</t>
         </is>
       </c>
-      <c r="B34" t="b">
-        <v>0</v>
-      </c>
-      <c r="C34">
-        <v>1</v>
-      </c>
-      <c r="D34" t="inlineStr">
+      <c r="C34" t="b">
+        <v>0</v>
+      </c>
+      <c r="D34">
+        <v>1</v>
+      </c>
+      <c r="E34" t="inlineStr">
         <is>
           <t>DEG - ancestry</t>
         </is>
       </c>
-      <c r="E34" t="inlineStr">
-        <is>
-          <t>Oligo.3</t>
-        </is>
-      </c>
       <c r="F34" t="inlineStr">
         <is>
+          <t>Oligo.3</t>
+        </is>
+      </c>
+      <c r="G34" t="inlineStr">
+        <is>
           <t>DEG carrier top: Oligo.3 AA_down</t>
         </is>
       </c>
-      <c r="G34" t="b">
+      <c r="H34" t="b">
         <v>1</v>
       </c>
     </row>
     <row r="35">
       <c r="A35" t="inlineStr">
         <is>
+          <t>ENSG00000148357</t>
+        </is>
+      </c>
+      <c r="B35" t="inlineStr">
+        <is>
           <t>HMCN2</t>
         </is>
       </c>
-      <c r="B35" t="b">
-        <v>0</v>
-      </c>
-      <c r="C35">
-        <v>1</v>
-      </c>
-      <c r="D35" t="inlineStr">
+      <c r="C35" t="b">
+        <v>0</v>
+      </c>
+      <c r="D35">
+        <v>1</v>
+      </c>
+      <c r="E35" t="inlineStr">
         <is>
           <t>Marker - cell type specific</t>
         </is>
       </c>
-      <c r="E35" t="inlineStr">
+      <c r="F35" t="inlineStr">
         <is>
           <t>Excit.L5.2</t>
         </is>
       </c>
-      <c r="F35" t="inlineStr">
+      <c r="G35" t="inlineStr">
         <is>
           <t>Excit.L5.2 specific MR genes - Excit.L5.2/Excit.L6b: 13.871</t>
         </is>
       </c>
-      <c r="G35" t="b">
+      <c r="H35" t="b">
         <v>1</v>
       </c>
     </row>
     <row r="36">
       <c r="A36" t="inlineStr">
         <is>
+          <t>ENSG00000233429</t>
+        </is>
+      </c>
+      <c r="B36" t="inlineStr">
+        <is>
           <t>HOTAIRM1</t>
         </is>
       </c>
-      <c r="B36" t="b">
-        <v>0</v>
-      </c>
-      <c r="C36">
-        <v>1</v>
-      </c>
-      <c r="D36" t="inlineStr">
+      <c r="C36" t="b">
+        <v>0</v>
+      </c>
+      <c r="D36">
+        <v>1</v>
+      </c>
+      <c r="E36" t="inlineStr">
         <is>
           <t>Marker - cell type specific</t>
         </is>
       </c>
-      <c r="E36" t="inlineStr">
+      <c r="F36" t="inlineStr">
         <is>
           <t>Excit.L5.2</t>
         </is>
       </c>
-      <c r="F36" t="inlineStr">
+      <c r="G36" t="inlineStr">
         <is>
           <t>Excit.L5.2 specific Enrich genes t= 16.54</t>
         </is>
       </c>
-      <c r="G36" t="b">
+      <c r="H36" t="b">
         <v>1</v>
       </c>
     </row>
     <row r="37">
       <c r="A37" t="inlineStr">
         <is>
+          <t>ENSG00000185811</t>
+        </is>
+      </c>
+      <c r="B37" t="inlineStr">
+        <is>
           <t>IKZF1</t>
         </is>
       </c>
-      <c r="B37" t="b">
-        <v>0</v>
-      </c>
-      <c r="C37">
-        <v>1</v>
-      </c>
-      <c r="D37" t="inlineStr">
+      <c r="C37" t="b">
+        <v>0</v>
+      </c>
+      <c r="D37">
+        <v>1</v>
+      </c>
+      <c r="E37" t="inlineStr">
         <is>
           <t>DEG - carrier</t>
         </is>
       </c>
-      <c r="E37" t="inlineStr">
-        <is>
-          <t>Oligo.3</t>
-        </is>
-      </c>
       <c r="F37" t="inlineStr">
         <is>
+          <t>Oligo.3</t>
+        </is>
+      </c>
+      <c r="G37" t="inlineStr">
+        <is>
           <t>DEG carrier top: Oligo.3 up</t>
         </is>
       </c>
-      <c r="G37" t="b">
+      <c r="H37" t="b">
         <v>1</v>
       </c>
     </row>
     <row r="38">
       <c r="A38" t="inlineStr">
         <is>
+          <t>ENSG00000134352</t>
+        </is>
+      </c>
+      <c r="B38" t="inlineStr">
+        <is>
           <t>IL6ST</t>
         </is>
       </c>
-      <c r="B38" t="b">
-        <v>0</v>
-      </c>
-      <c r="C38">
-        <v>1</v>
-      </c>
-      <c r="D38" t="inlineStr">
+      <c r="C38" t="b">
+        <v>0</v>
+      </c>
+      <c r="D38">
+        <v>1</v>
+      </c>
+      <c r="E38" t="inlineStr">
         <is>
           <t>DEG - mediation</t>
         </is>
       </c>
-      <c r="E38" t="inlineStr">
+      <c r="F38" t="inlineStr">
         <is>
           <t>Astro.3</t>
         </is>
       </c>
-      <c r="F38" t="inlineStr">
+      <c r="G38" t="inlineStr">
         <is>
           <t>mediation gene: mediator Astro.3</t>
         </is>
       </c>
-      <c r="G38" t="b">
+      <c r="H38" t="b">
         <v>1</v>
       </c>
     </row>
     <row r="39">
       <c r="A39" t="inlineStr">
         <is>
+          <t>ENSG00000138448</t>
+        </is>
+      </c>
+      <c r="B39" t="inlineStr">
+        <is>
           <t>ITGAV</t>
         </is>
       </c>
-      <c r="B39" t="b">
-        <v>0</v>
-      </c>
-      <c r="C39">
-        <v>1</v>
-      </c>
-      <c r="D39" t="inlineStr">
+      <c r="C39" t="b">
+        <v>0</v>
+      </c>
+      <c r="D39">
+        <v>1</v>
+      </c>
+      <c r="E39" t="inlineStr">
         <is>
           <t>Marker - cell type specific</t>
         </is>
       </c>
-      <c r="E39" t="inlineStr">
+      <c r="F39" t="inlineStr">
         <is>
           <t>Oligo.2</t>
         </is>
       </c>
-      <c r="F39" t="inlineStr">
+      <c r="G39" t="inlineStr">
         <is>
           <t>Oligo.2 specific MR genes - Oligo.2/Oligo.1: 1.663</t>
         </is>
       </c>
-      <c r="G39" t="b">
+      <c r="H39" t="b">
         <v>1</v>
       </c>
     </row>
     <row r="40">
       <c r="A40" t="inlineStr">
         <is>
+          <t>ENSG00000108773</t>
+        </is>
+      </c>
+      <c r="B40" t="inlineStr">
+        <is>
           <t>KAT2A</t>
         </is>
       </c>
-      <c r="B40" t="b">
-        <v>0</v>
-      </c>
-      <c r="C40">
-        <v>1</v>
-      </c>
-      <c r="D40" t="inlineStr">
+      <c r="C40" t="b">
+        <v>0</v>
+      </c>
+      <c r="D40">
+        <v>1</v>
+      </c>
+      <c r="E40" t="inlineStr">
         <is>
           <t>DEG - ancestry</t>
         </is>
       </c>
-      <c r="E40" t="inlineStr">
-        <is>
-          <t>Oligo.3</t>
-        </is>
-      </c>
       <c r="F40" t="inlineStr">
         <is>
+          <t>Oligo.3</t>
+        </is>
+      </c>
+      <c r="G40" t="inlineStr">
+        <is>
           <t>DEG Ancestry op: Oligo.3 AA_up*-EA_down</t>
         </is>
       </c>
-      <c r="G40" t="b">
+      <c r="H40" t="b">
         <v>1</v>
       </c>
     </row>
     <row r="41">
       <c r="A41" t="inlineStr">
         <is>
+          <t>ENSG00000184408</t>
+        </is>
+      </c>
+      <c r="B41" t="inlineStr">
+        <is>
           <t>KCND2</t>
         </is>
       </c>
-      <c r="B41" t="b">
-        <v>0</v>
-      </c>
-      <c r="C41">
-        <v>1</v>
-      </c>
-      <c r="D41" t="inlineStr">
+      <c r="C41" t="b">
+        <v>0</v>
+      </c>
+      <c r="D41">
+        <v>1</v>
+      </c>
+      <c r="E41" t="inlineStr">
         <is>
           <t>Marker - cell type specific</t>
         </is>
       </c>
-      <c r="E41" t="inlineStr">
-        <is>
-          <t>Oligo.3</t>
-        </is>
-      </c>
       <c r="F41" t="inlineStr">
         <is>
+          <t>Oligo.3</t>
+        </is>
+      </c>
+      <c r="G41" t="inlineStr">
+        <is>
           <t>Oligo.3 specific Enrich genes t= 9.2</t>
         </is>
       </c>
-      <c r="G41" t="b">
+      <c r="H41" t="b">
         <v>1</v>
       </c>
     </row>
     <row r="42">
       <c r="A42" t="inlineStr">
         <is>
+          <t>ENSG00000162989</t>
+        </is>
+      </c>
+      <c r="B42" t="inlineStr">
+        <is>
           <t>KCNJ3</t>
         </is>
       </c>
-      <c r="B42" t="b">
-        <v>0</v>
-      </c>
-      <c r="C42">
-        <v>1</v>
-      </c>
-      <c r="D42" t="inlineStr">
+      <c r="C42" t="b">
+        <v>0</v>
+      </c>
+      <c r="D42">
+        <v>1</v>
+      </c>
+      <c r="E42" t="inlineStr">
         <is>
           <t>Marker - cell type specific</t>
         </is>
       </c>
-      <c r="E42" t="inlineStr">
-        <is>
-          <t>Oligo.3</t>
-        </is>
-      </c>
       <c r="F42" t="inlineStr">
         <is>
+          <t>Oligo.3</t>
+        </is>
+      </c>
+      <c r="G42" t="inlineStr">
+        <is>
           <t>Oligo.3 specific Enrich genes t= 9.5</t>
         </is>
       </c>
-      <c r="G42" t="b">
+      <c r="H42" t="b">
         <v>1</v>
       </c>
     </row>
     <row r="43">
       <c r="A43" t="inlineStr">
         <is>
+          <t>ENSG00000234665</t>
+        </is>
+      </c>
+      <c r="B43" t="inlineStr">
+        <is>
           <t>LERFS</t>
         </is>
       </c>
-      <c r="B43" t="b">
-        <v>0</v>
-      </c>
-      <c r="C43">
-        <v>1</v>
-      </c>
-      <c r="D43" t="inlineStr">
+      <c r="C43" t="b">
+        <v>0</v>
+      </c>
+      <c r="D43">
+        <v>1</v>
+      </c>
+      <c r="E43" t="inlineStr">
         <is>
           <t>DEG - carrier</t>
         </is>
       </c>
-      <c r="E43" t="inlineStr">
-        <is>
-          <t>Oligo.3</t>
-        </is>
-      </c>
       <c r="F43" t="inlineStr">
         <is>
+          <t>Oligo.3</t>
+        </is>
+      </c>
+      <c r="G43" t="inlineStr">
+        <is>
           <t>DEG carrier top: Oligo.3 down</t>
         </is>
       </c>
-      <c r="G43" t="b">
+      <c r="H43" t="b">
         <v>1</v>
       </c>
     </row>
     <row r="44">
       <c r="A44" t="inlineStr">
         <is>
+          <t>ENSG00000231023</t>
+        </is>
+      </c>
+      <c r="B44" t="inlineStr">
+        <is>
           <t>LINC00326</t>
         </is>
       </c>
-      <c r="B44" t="b">
-        <v>0</v>
-      </c>
-      <c r="C44">
-        <v>1</v>
-      </c>
-      <c r="D44" t="inlineStr">
+      <c r="C44" t="b">
+        <v>0</v>
+      </c>
+      <c r="D44">
+        <v>1</v>
+      </c>
+      <c r="E44" t="inlineStr">
         <is>
           <t>DEG - carrier</t>
         </is>
       </c>
-      <c r="E44" t="inlineStr">
+      <c r="F44" t="inlineStr">
         <is>
           <t>Excit.L2_5.1</t>
         </is>
       </c>
-      <c r="F44" t="inlineStr">
+      <c r="G44" t="inlineStr">
         <is>
           <t>DEG carrier top:  Excit.L2_5.1 up</t>
         </is>
       </c>
-      <c r="G44" t="b">
+      <c r="H44" t="b">
         <v>1</v>
       </c>
     </row>
     <row r="45">
       <c r="A45" t="inlineStr">
         <is>
+          <t>ENSG00000233237</t>
+        </is>
+      </c>
+      <c r="B45" t="inlineStr">
+        <is>
           <t>LINC00472</t>
         </is>
       </c>
-      <c r="B45" t="b">
-        <v>0</v>
-      </c>
-      <c r="C45">
-        <v>1</v>
-      </c>
-      <c r="D45" t="inlineStr">
+      <c r="C45" t="b">
+        <v>0</v>
+      </c>
+      <c r="D45">
+        <v>1</v>
+      </c>
+      <c r="E45" t="inlineStr">
         <is>
           <t>DEG - ancestry</t>
         </is>
       </c>
-      <c r="E45" t="inlineStr">
-        <is>
-          <t>Oligo.3</t>
-        </is>
-      </c>
       <c r="F45" t="inlineStr">
         <is>
+          <t>Oligo.3</t>
+        </is>
+      </c>
+      <c r="G45" t="inlineStr">
+        <is>
           <t>DEG Ancestry op: Oligo.3 AA_down-EA_up*</t>
         </is>
       </c>
-      <c r="G45" t="b">
+      <c r="H45" t="b">
         <v>1</v>
       </c>
     </row>
     <row r="46">
       <c r="A46" t="inlineStr">
         <is>
+          <t>ENSG00000257585</t>
+        </is>
+      </c>
+      <c r="B46" t="inlineStr">
+        <is>
           <t>LINC00609</t>
         </is>
       </c>
-      <c r="B46" t="b">
-        <v>0</v>
-      </c>
-      <c r="C46">
-        <v>1</v>
-      </c>
-      <c r="D46" t="inlineStr">
+      <c r="C46" t="b">
+        <v>0</v>
+      </c>
+      <c r="D46">
+        <v>1</v>
+      </c>
+      <c r="E46" t="inlineStr">
         <is>
           <t>Marker - cell type specific</t>
         </is>
       </c>
-      <c r="E46" t="inlineStr">
+      <c r="F46" t="inlineStr">
         <is>
           <t>Oligo.2</t>
         </is>
       </c>
-      <c r="F46" t="inlineStr">
+      <c r="G46" t="inlineStr">
         <is>
           <t>Oligo.2 specific Enrich genes t= 10.42</t>
         </is>
       </c>
-      <c r="G46" t="b">
+      <c r="H46" t="b">
         <v>1</v>
       </c>
     </row>
     <row r="47">
       <c r="A47" t="inlineStr">
         <is>
+          <t>ENSG00000281186</t>
+        </is>
+      </c>
+      <c r="B47" t="inlineStr">
+        <is>
           <t>LINC00706</t>
         </is>
       </c>
-      <c r="B47" t="b">
-        <v>0</v>
-      </c>
-      <c r="C47">
-        <v>1</v>
-      </c>
-      <c r="D47" t="inlineStr">
+      <c r="C47" t="b">
+        <v>0</v>
+      </c>
+      <c r="D47">
+        <v>1</v>
+      </c>
+      <c r="E47" t="inlineStr">
         <is>
           <t>DEG - ancestry</t>
         </is>
       </c>
-      <c r="E47" t="inlineStr">
-        <is>
-          <t>Oligo.3</t>
-        </is>
-      </c>
       <c r="F47" t="inlineStr">
         <is>
+          <t>Oligo.3</t>
+        </is>
+      </c>
+      <c r="G47" t="inlineStr">
+        <is>
           <t>DEG carrier top: Oligo.3 AA_down</t>
         </is>
       </c>
-      <c r="G47" t="b">
+      <c r="H47" t="b">
         <v>1</v>
       </c>
     </row>
     <row r="48">
       <c r="A48" t="inlineStr">
         <is>
+          <t>ENSG00000233973</t>
+        </is>
+      </c>
+      <c r="B48" t="inlineStr">
+        <is>
           <t>LINC01360</t>
         </is>
       </c>
-      <c r="B48" t="b">
-        <v>0</v>
-      </c>
-      <c r="C48">
-        <v>1</v>
-      </c>
-      <c r="D48" t="inlineStr">
+      <c r="C48" t="b">
+        <v>0</v>
+      </c>
+      <c r="D48">
+        <v>1</v>
+      </c>
+      <c r="E48" t="inlineStr">
         <is>
           <t>DEG - carrier</t>
         </is>
       </c>
-      <c r="E48" t="inlineStr">
+      <c r="F48" t="inlineStr">
         <is>
           <t>Excit.L5.2</t>
         </is>
       </c>
-      <c r="F48" t="inlineStr">
+      <c r="G48" t="inlineStr">
         <is>
           <t>DEG carrier top:  Excit.L5.2 up</t>
         </is>
       </c>
-      <c r="G48" t="b">
+      <c r="H48" t="b">
         <v>1</v>
       </c>
     </row>
     <row r="49">
       <c r="A49" t="inlineStr">
         <is>
+          <t>ENSG00000238217</t>
+        </is>
+      </c>
+      <c r="B49" t="inlineStr">
+        <is>
           <t>LINC01877</t>
         </is>
       </c>
-      <c r="B49" t="b">
-        <v>0</v>
-      </c>
-      <c r="C49">
+      <c r="C49" t="b">
+        <v>0</v>
+      </c>
+      <c r="D49">
         <v>2</v>
       </c>
-      <c r="D49" t="inlineStr">
+      <c r="E49" t="inlineStr">
         <is>
           <t>Marker - cell type global, Marker - cell type specific</t>
         </is>
       </c>
-      <c r="E49" t="inlineStr">
+      <c r="F49" t="inlineStr">
         <is>
           <t>Oligo.2</t>
         </is>
       </c>
-      <c r="F49" t="inlineStr">
+      <c r="G49" t="inlineStr">
         <is>
           <t>globl MR genes -  Oligo.2/Oligo.1: 1.743, Oligo.2 specific MR genes - Oligo.2/Oligo.1: 1.743</t>
         </is>
       </c>
-      <c r="G49" t="b">
+      <c r="H49" t="b">
         <v>1</v>
       </c>
     </row>
     <row r="50">
       <c r="A50" t="inlineStr">
         <is>
+          <t>ENSG00000254401</t>
+        </is>
+      </c>
+      <c r="B50" t="inlineStr">
+        <is>
           <t>LINC02752</t>
         </is>
       </c>
-      <c r="B50" t="b">
-        <v>0</v>
-      </c>
-      <c r="C50">
-        <v>1</v>
-      </c>
-      <c r="D50" t="inlineStr">
+      <c r="C50" t="b">
+        <v>0</v>
+      </c>
+      <c r="D50">
+        <v>1</v>
+      </c>
+      <c r="E50" t="inlineStr">
         <is>
           <t>Marker - cell type global</t>
         </is>
       </c>
-      <c r="E50" t="inlineStr">
+      <c r="F50" t="inlineStr">
         <is>
           <t>Excit.L5.2</t>
         </is>
       </c>
-      <c r="F50" t="inlineStr">
+      <c r="G50" t="inlineStr">
         <is>
           <t>globl MR genes -  Excit.L5.2/Excit.L2_5.2: 10.797</t>
         </is>
       </c>
-      <c r="G50" t="b">
+      <c r="H50" t="b">
         <v>1</v>
       </c>
     </row>
     <row r="51">
       <c r="A51" t="inlineStr">
         <is>
+          <t>ENSG00000174482</t>
+        </is>
+      </c>
+      <c r="B51" t="inlineStr">
+        <is>
           <t>LINGO2</t>
         </is>
       </c>
-      <c r="B51" t="b">
-        <v>0</v>
-      </c>
-      <c r="C51">
-        <v>1</v>
-      </c>
-      <c r="D51" t="inlineStr">
+      <c r="C51" t="b">
+        <v>0</v>
+      </c>
+      <c r="D51">
+        <v>1</v>
+      </c>
+      <c r="E51" t="inlineStr">
         <is>
           <t>Marker - cell type specific</t>
         </is>
       </c>
-      <c r="E51" t="inlineStr">
-        <is>
-          <t>Oligo.3</t>
-        </is>
-      </c>
       <c r="F51" t="inlineStr">
         <is>
+          <t>Oligo.3</t>
+        </is>
+      </c>
+      <c r="G51" t="inlineStr">
+        <is>
           <t>Oligo.3 specific Enrich genes t= 9.09</t>
         </is>
       </c>
-      <c r="G51" t="b">
+      <c r="H51" t="b">
         <v>1</v>
       </c>
     </row>
     <row r="52">
       <c r="A52" t="inlineStr">
         <is>
+          <t>ENSG00000048540</t>
+        </is>
+      </c>
+      <c r="B52" t="inlineStr">
+        <is>
           <t>LMO3</t>
         </is>
       </c>
-      <c r="B52" t="b">
-        <v>0</v>
-      </c>
-      <c r="C52">
-        <v>1</v>
-      </c>
-      <c r="D52" t="inlineStr">
+      <c r="C52" t="b">
+        <v>0</v>
+      </c>
+      <c r="D52">
+        <v>1</v>
+      </c>
+      <c r="E52" t="inlineStr">
         <is>
           <t>Marker - cell type specific</t>
         </is>
       </c>
-      <c r="E52" t="inlineStr">
+      <c r="F52" t="inlineStr">
         <is>
           <t>Astro.1</t>
         </is>
       </c>
-      <c r="F52" t="inlineStr">
+      <c r="G52" t="inlineStr">
         <is>
           <t>Astro.1 specific Enrich genes t= 8.73</t>
         </is>
       </c>
-      <c r="G52" t="b">
+      <c r="H52" t="b">
         <v>1</v>
       </c>
     </row>
     <row r="53">
       <c r="A53" t="inlineStr">
         <is>
+          <t>ENSG00000235448</t>
+        </is>
+      </c>
+      <c r="B53" t="inlineStr">
+        <is>
           <t>LURAP1L-AS1</t>
         </is>
       </c>
-      <c r="B53" t="b">
-        <v>0</v>
-      </c>
-      <c r="C53">
-        <v>1</v>
-      </c>
-      <c r="D53" t="inlineStr">
+      <c r="C53" t="b">
+        <v>0</v>
+      </c>
+      <c r="D53">
+        <v>1</v>
+      </c>
+      <c r="E53" t="inlineStr">
         <is>
           <t>DEG - carrier</t>
         </is>
       </c>
-      <c r="E53" t="inlineStr">
-        <is>
-          <t>Oligo.3</t>
-        </is>
-      </c>
       <c r="F53" t="inlineStr">
         <is>
+          <t>Oligo.3</t>
+        </is>
+      </c>
+      <c r="G53" t="inlineStr">
+        <is>
           <t>DEG carrier top: Oligo.3 down</t>
         </is>
       </c>
-      <c r="G53" t="b">
+      <c r="H53" t="b">
         <v>1</v>
       </c>
     </row>
     <row r="54">
       <c r="A54" t="inlineStr">
         <is>
+          <t>ENSG00000102316</t>
+        </is>
+      </c>
+      <c r="B54" t="inlineStr">
+        <is>
           <t>MAGED2</t>
         </is>
       </c>
-      <c r="B54" t="b">
-        <v>0</v>
-      </c>
-      <c r="C54">
-        <v>1</v>
-      </c>
-      <c r="D54" t="inlineStr">
+      <c r="C54" t="b">
+        <v>0</v>
+      </c>
+      <c r="D54">
+        <v>1</v>
+      </c>
+      <c r="E54" t="inlineStr">
         <is>
           <t>DEG - ancestry</t>
         </is>
       </c>
-      <c r="E54" t="inlineStr">
-        <is>
-          <t>Oligo.3</t>
-        </is>
-      </c>
       <c r="F54" t="inlineStr">
         <is>
+          <t>Oligo.3</t>
+        </is>
+      </c>
+      <c r="G54" t="inlineStr">
+        <is>
           <t>DEG Ancestry op: Oligo.3 AA_up-EA_down*</t>
         </is>
       </c>
-      <c r="G54" t="b">
+      <c r="H54" t="b">
         <v>1</v>
       </c>
     </row>
     <row r="55">
       <c r="A55" t="inlineStr">
         <is>
+          <t>ENSG00000186868</t>
+        </is>
+      </c>
+      <c r="B55" t="inlineStr">
+        <is>
           <t>MAPT</t>
         </is>
       </c>
-      <c r="B55" t="b">
-        <v>0</v>
-      </c>
-      <c r="C55">
-        <v>1</v>
-      </c>
-      <c r="D55" t="inlineStr">
+      <c r="C55" t="b">
+        <v>0</v>
+      </c>
+      <c r="D55">
+        <v>1</v>
+      </c>
+      <c r="E55" t="inlineStr">
         <is>
           <t>DEG - carrier</t>
         </is>
       </c>
-      <c r="E55" t="inlineStr">
-        <is>
-          <t>Oligo.3</t>
-        </is>
-      </c>
       <c r="F55" t="inlineStr">
         <is>
+          <t>Oligo.3</t>
+        </is>
+      </c>
+      <c r="G55" t="inlineStr">
+        <is>
           <t>DEG of interest: Oligo.3 down</t>
         </is>
       </c>
-      <c r="G55" t="b">
+      <c r="H55" t="b">
         <v>1</v>
       </c>
     </row>
     <row r="56">
       <c r="A56" t="inlineStr">
         <is>
+          <t>ENSG00000197971</t>
+        </is>
+      </c>
+      <c r="B56" t="inlineStr">
+        <is>
           <t>MBP</t>
         </is>
       </c>
-      <c r="B56" t="b">
-        <v>0</v>
-      </c>
-      <c r="C56">
+      <c r="C56" t="b">
+        <v>0</v>
+      </c>
+      <c r="D56">
         <v>3</v>
       </c>
-      <c r="D56" t="inlineStr">
+      <c r="E56" t="inlineStr">
         <is>
           <t>DEG - carrier, DEG - mediation, Marker - SpD</t>
         </is>
       </c>
-      <c r="E56" t="inlineStr">
+      <c r="F56" t="inlineStr">
         <is>
           <t>Oligo.3, WM.uf~Sp09D07</t>
         </is>
       </c>
-      <c r="F56" t="inlineStr">
+      <c r="G56" t="inlineStr">
         <is>
           <t>SpD Enrich gene t=6.53, DEG of interest: Oligo.3 down, mediation gene: outcome Oligo.3</t>
         </is>
       </c>
-      <c r="G56" t="b">
+      <c r="H56" t="b">
         <v>1</v>
       </c>
     </row>
     <row r="57">
       <c r="A57" t="inlineStr">
         <is>
+          <t>ENSG00000214548</t>
+        </is>
+      </c>
+      <c r="B57" t="inlineStr">
+        <is>
           <t>MEG3</t>
         </is>
       </c>
-      <c r="B57" t="b">
-        <v>0</v>
-      </c>
-      <c r="C57">
-        <v>1</v>
-      </c>
-      <c r="D57" t="inlineStr">
+      <c r="C57" t="b">
+        <v>0</v>
+      </c>
+      <c r="D57">
+        <v>1</v>
+      </c>
+      <c r="E57" t="inlineStr">
         <is>
           <t>Marker - cell type specific</t>
         </is>
       </c>
-      <c r="E57" t="inlineStr">
+      <c r="F57" t="inlineStr">
         <is>
           <t>OPC.5</t>
         </is>
       </c>
-      <c r="F57" t="inlineStr">
+      <c r="G57" t="inlineStr">
         <is>
           <t>OPC.5 specific MR genes - OPC.5/OPC.2: 1.019</t>
         </is>
       </c>
-      <c r="G57" t="b">
+      <c r="H57" t="b">
         <v>1</v>
       </c>
     </row>
     <row r="58">
       <c r="A58" t="inlineStr">
         <is>
+          <t>ENSG00000225783</t>
+        </is>
+      </c>
+      <c r="B58" t="inlineStr">
+        <is>
           <t>MIAT</t>
         </is>
       </c>
-      <c r="B58" t="b">
-        <v>0</v>
-      </c>
-      <c r="C58">
-        <v>1</v>
-      </c>
-      <c r="D58" t="inlineStr">
+      <c r="C58" t="b">
+        <v>0</v>
+      </c>
+      <c r="D58">
+        <v>1</v>
+      </c>
+      <c r="E58" t="inlineStr">
         <is>
           <t>DEG - ancestry</t>
         </is>
       </c>
-      <c r="E58" t="inlineStr">
-        <is>
-          <t>Oligo.3</t>
-        </is>
-      </c>
       <c r="F58" t="inlineStr">
         <is>
+          <t>Oligo.3</t>
+        </is>
+      </c>
+      <c r="G58" t="inlineStr">
+        <is>
           <t>DEG carrier top: Oligo.3 AA_up</t>
         </is>
       </c>
-      <c r="G58" t="b">
+      <c r="H58" t="b">
         <v>1</v>
       </c>
     </row>
     <row r="59">
       <c r="A59" t="inlineStr">
         <is>
+          <t>ENSG00000136297</t>
+        </is>
+      </c>
+      <c r="B59" t="inlineStr">
+        <is>
           <t>MMD2</t>
         </is>
       </c>
-      <c r="B59" t="b">
-        <v>0</v>
-      </c>
-      <c r="C59">
-        <v>1</v>
-      </c>
-      <c r="D59" t="inlineStr">
+      <c r="C59" t="b">
+        <v>0</v>
+      </c>
+      <c r="D59">
+        <v>1</v>
+      </c>
+      <c r="E59" t="inlineStr">
         <is>
           <t>Marker - cell type specific</t>
         </is>
       </c>
-      <c r="E59" t="inlineStr">
+      <c r="F59" t="inlineStr">
         <is>
           <t>Astro.2</t>
         </is>
       </c>
-      <c r="F59" t="inlineStr">
+      <c r="G59" t="inlineStr">
         <is>
           <t>Astro.2 specific MR genes - Astro.2/Astro.5: 1.004</t>
         </is>
       </c>
-      <c r="G59" t="b">
+      <c r="H59" t="b">
         <v>1</v>
       </c>
     </row>
     <row r="60">
       <c r="A60" t="inlineStr">
         <is>
+          <t>ENSG00000198938</t>
+        </is>
+      </c>
+      <c r="B60" t="inlineStr">
+        <is>
           <t>MT-CO3</t>
         </is>
       </c>
-      <c r="B60" t="b">
-        <v>0</v>
-      </c>
-      <c r="C60">
-        <v>1</v>
-      </c>
-      <c r="D60" t="inlineStr">
+      <c r="C60" t="b">
+        <v>0</v>
+      </c>
+      <c r="D60">
+        <v>1</v>
+      </c>
+      <c r="E60" t="inlineStr">
         <is>
           <t>Marker - cell type specific</t>
         </is>
       </c>
-      <c r="E60" t="inlineStr">
-        <is>
-          <t>Oligo.3</t>
-        </is>
-      </c>
       <c r="F60" t="inlineStr">
         <is>
+          <t>Oligo.3</t>
+        </is>
+      </c>
+      <c r="G60" t="inlineStr">
+        <is>
           <t>Oligo.3 specific MR genes - Oligo.3/Oligo.4: 1.141</t>
         </is>
       </c>
-      <c r="G60" t="b">
+      <c r="H60" t="b">
         <v>1</v>
       </c>
     </row>
     <row r="61">
       <c r="A61" t="inlineStr">
         <is>
+          <t>ENSG00000198727</t>
+        </is>
+      </c>
+      <c r="B61" t="inlineStr">
+        <is>
           <t>MT-CYB</t>
         </is>
       </c>
-      <c r="B61" t="b">
-        <v>0</v>
-      </c>
-      <c r="C61">
-        <v>1</v>
-      </c>
-      <c r="D61" t="inlineStr">
+      <c r="C61" t="b">
+        <v>0</v>
+      </c>
+      <c r="D61">
+        <v>1</v>
+      </c>
+      <c r="E61" t="inlineStr">
         <is>
           <t>Marker - cell type specific</t>
         </is>
       </c>
-      <c r="E61" t="inlineStr">
+      <c r="F61" t="inlineStr">
         <is>
           <t>Excit.L2_5.1</t>
         </is>
       </c>
-      <c r="F61" t="inlineStr">
+      <c r="G61" t="inlineStr">
         <is>
           <t>Excit.L2_5.1 specific MR genes - Excit.L2_5.1/Excit.L6b: 1.175</t>
         </is>
       </c>
-      <c r="G61" t="b">
+      <c r="H61" t="b">
         <v>1</v>
       </c>
     </row>
     <row r="62">
       <c r="A62" t="inlineStr">
         <is>
+          <t>ENSG00000198888</t>
+        </is>
+      </c>
+      <c r="B62" t="inlineStr">
+        <is>
           <t>MT-ND1</t>
         </is>
       </c>
-      <c r="B62" t="b">
-        <v>0</v>
-      </c>
-      <c r="C62">
-        <v>1</v>
-      </c>
-      <c r="D62" t="inlineStr">
+      <c r="C62" t="b">
+        <v>0</v>
+      </c>
+      <c r="D62">
+        <v>1</v>
+      </c>
+      <c r="E62" t="inlineStr">
         <is>
           <t>Marker - cell type specific</t>
         </is>
       </c>
-      <c r="E62" t="inlineStr">
+      <c r="F62" t="inlineStr">
         <is>
           <t>Excit.L2_5.1</t>
         </is>
       </c>
-      <c r="F62" t="inlineStr">
+      <c r="G62" t="inlineStr">
         <is>
           <t>Excit.L2_5.1 specific MR genes - Excit.L2_5.1/Excit.L6b: 1.201</t>
         </is>
       </c>
-      <c r="G62" t="b">
+      <c r="H62" t="b">
         <v>1</v>
       </c>
     </row>
     <row r="63">
       <c r="A63" t="inlineStr">
         <is>
+          <t>ENSG00000128654</t>
+        </is>
+      </c>
+      <c r="B63" t="inlineStr">
+        <is>
           <t>MTX2</t>
         </is>
       </c>
-      <c r="B63" t="b">
-        <v>0</v>
-      </c>
-      <c r="C63">
-        <v>1</v>
-      </c>
-      <c r="D63" t="inlineStr">
+      <c r="C63" t="b">
+        <v>0</v>
+      </c>
+      <c r="D63">
+        <v>1</v>
+      </c>
+      <c r="E63" t="inlineStr">
         <is>
           <t>Marker - cell type specific</t>
         </is>
       </c>
-      <c r="E63" t="inlineStr">
+      <c r="F63" t="inlineStr">
         <is>
           <t>Oligo.2</t>
         </is>
       </c>
-      <c r="F63" t="inlineStr">
+      <c r="G63" t="inlineStr">
         <is>
           <t>Oligo.2 specific Enrich genes t= 11.38</t>
         </is>
       </c>
-      <c r="G63" t="b">
+      <c r="H63" t="b">
         <v>1</v>
       </c>
     </row>
     <row r="64">
       <c r="A64" t="inlineStr">
         <is>
+          <t>ENSG00000186310</t>
+        </is>
+      </c>
+      <c r="B64" t="inlineStr">
+        <is>
           <t>NAP1L3</t>
         </is>
       </c>
-      <c r="B64" t="b">
-        <v>0</v>
-      </c>
-      <c r="C64">
-        <v>1</v>
-      </c>
-      <c r="D64" t="inlineStr">
+      <c r="C64" t="b">
+        <v>0</v>
+      </c>
+      <c r="D64">
+        <v>1</v>
+      </c>
+      <c r="E64" t="inlineStr">
         <is>
           <t>DEG - mediation</t>
         </is>
       </c>
-      <c r="E64" t="inlineStr">
-        <is>
-          <t>Oligo.3</t>
-        </is>
-      </c>
       <c r="F64" t="inlineStr">
         <is>
+          <t>Oligo.3</t>
+        </is>
+      </c>
+      <c r="G64" t="inlineStr">
+        <is>
           <t>mediation gene: outcome Oligo.3</t>
         </is>
       </c>
-      <c r="G64" t="b">
+      <c r="H64" t="b">
         <v>1</v>
       </c>
     </row>
     <row r="65">
       <c r="A65" t="inlineStr">
         <is>
+          <t>ENSG00000166342</t>
+        </is>
+      </c>
+      <c r="B65" t="inlineStr">
+        <is>
           <t>NETO1</t>
         </is>
       </c>
-      <c r="B65" t="b">
-        <v>0</v>
-      </c>
-      <c r="C65">
-        <v>1</v>
-      </c>
-      <c r="D65" t="inlineStr">
+      <c r="C65" t="b">
+        <v>0</v>
+      </c>
+      <c r="D65">
+        <v>1</v>
+      </c>
+      <c r="E65" t="inlineStr">
         <is>
           <t>DEG - mediation</t>
         </is>
       </c>
-      <c r="E65" t="inlineStr">
+      <c r="F65" t="inlineStr">
         <is>
           <t>Astro.2</t>
         </is>
       </c>
-      <c r="F65" t="inlineStr">
+      <c r="G65" t="inlineStr">
         <is>
           <t>mediation gene: mediator Astro.2</t>
         </is>
       </c>
-      <c r="G65" t="b">
+      <c r="H65" t="b">
         <v>1</v>
       </c>
     </row>
     <row r="66">
       <c r="A66" t="inlineStr">
         <is>
+          <t>ENSG00000148826</t>
+        </is>
+      </c>
+      <c r="B66" t="inlineStr">
+        <is>
           <t>NKX6-2</t>
         </is>
       </c>
-      <c r="B66" t="b">
-        <v>0</v>
-      </c>
-      <c r="C66">
-        <v>1</v>
-      </c>
-      <c r="D66" t="inlineStr">
+      <c r="C66" t="b">
+        <v>0</v>
+      </c>
+      <c r="D66">
+        <v>1</v>
+      </c>
+      <c r="E66" t="inlineStr">
         <is>
           <t>MOFA - Factor3</t>
         </is>
       </c>
-      <c r="E66" t="inlineStr">
-        <is>
-          <t>Oligo.3</t>
-        </is>
-      </c>
       <c r="F66" t="inlineStr">
         <is>
+          <t>Oligo.3</t>
+        </is>
+      </c>
+      <c r="G66" t="inlineStr">
+        <is>
           <t>MOFA Oligo.3 Factor3-</t>
         </is>
       </c>
-      <c r="G66" t="b">
+      <c r="H66" t="b">
         <v>1</v>
       </c>
     </row>
     <row r="67">
       <c r="A67" t="inlineStr">
         <is>
+          <t>ENSG00000169760</t>
+        </is>
+      </c>
+      <c r="B67" t="inlineStr">
+        <is>
           <t>NLGN1</t>
         </is>
       </c>
-      <c r="B67" t="b">
-        <v>0</v>
-      </c>
-      <c r="C67">
-        <v>1</v>
-      </c>
-      <c r="D67" t="inlineStr">
+      <c r="C67" t="b">
+        <v>0</v>
+      </c>
+      <c r="D67">
+        <v>1</v>
+      </c>
+      <c r="E67" t="inlineStr">
         <is>
           <t>DEGs - LR</t>
         </is>
       </c>
-      <c r="E67" t="inlineStr">
-        <is>
-          <t>Oligo.3</t>
-        </is>
-      </c>
       <c r="F67" t="inlineStr">
         <is>
+          <t>Oligo.3</t>
+        </is>
+      </c>
+      <c r="G67" t="inlineStr">
+        <is>
           <t>DEG LR interactions: NLGN1 -&gt; NRXN1,NLGN1 -&gt; NRXN3,NRXN1 -&gt; NLGN1,NRXN3 -&gt; NLGN1</t>
         </is>
       </c>
-      <c r="G67" t="b">
+      <c r="H67" t="b">
         <v>1</v>
       </c>
     </row>
     <row r="68">
       <c r="A68" t="inlineStr">
         <is>
+          <t>ENSG00000221890</t>
+        </is>
+      </c>
+      <c r="B68" t="inlineStr">
+        <is>
           <t>NPTXR</t>
         </is>
       </c>
-      <c r="B68" t="b">
-        <v>0</v>
-      </c>
-      <c r="C68">
-        <v>1</v>
-      </c>
-      <c r="D68" t="inlineStr">
+      <c r="C68" t="b">
+        <v>0</v>
+      </c>
+      <c r="D68">
+        <v>1</v>
+      </c>
+      <c r="E68" t="inlineStr">
         <is>
           <t>DEG - mediation</t>
         </is>
       </c>
-      <c r="E68" t="inlineStr">
+      <c r="F68" t="inlineStr">
         <is>
           <t>Astro.1</t>
         </is>
       </c>
-      <c r="F68" t="inlineStr">
+      <c r="G68" t="inlineStr">
         <is>
           <t>mediation gene: mediator Astro.1</t>
         </is>
       </c>
-      <c r="G68" t="b">
+      <c r="H68" t="b">
         <v>1</v>
       </c>
     </row>
     <row r="69">
       <c r="A69" t="inlineStr">
         <is>
+          <t>ENSG00000185737</t>
+        </is>
+      </c>
+      <c r="B69" t="inlineStr">
+        <is>
           <t>NRG3</t>
         </is>
       </c>
-      <c r="B69" t="b">
-        <v>0</v>
-      </c>
-      <c r="C69">
-        <v>1</v>
-      </c>
-      <c r="D69" t="inlineStr">
+      <c r="C69" t="b">
+        <v>0</v>
+      </c>
+      <c r="D69">
+        <v>1</v>
+      </c>
+      <c r="E69" t="inlineStr">
         <is>
           <t>DEGs - LR</t>
         </is>
       </c>
-      <c r="E69" t="inlineStr">
-        <is>
-          <t>Oligo.3</t>
-        </is>
-      </c>
       <c r="F69" t="inlineStr">
         <is>
+          <t>Oligo.3</t>
+        </is>
+      </c>
+      <c r="G69" t="inlineStr">
+        <is>
           <t>DEG LR interactions: NRG3 -&gt; ERBB3</t>
         </is>
       </c>
-      <c r="G69" t="b">
+      <c r="H69" t="b">
         <v>1</v>
       </c>
     </row>
     <row r="70">
       <c r="A70" t="inlineStr">
         <is>
+          <t>ENSG00000179915</t>
+        </is>
+      </c>
+      <c r="B70" t="inlineStr">
+        <is>
           <t>NRXN1</t>
         </is>
       </c>
-      <c r="B70" t="b">
-        <v>0</v>
-      </c>
-      <c r="C70">
-        <v>1</v>
-      </c>
-      <c r="D70" t="inlineStr">
+      <c r="C70" t="b">
+        <v>0</v>
+      </c>
+      <c r="D70">
+        <v>1</v>
+      </c>
+      <c r="E70" t="inlineStr">
         <is>
           <t>DEGs - LR</t>
         </is>
       </c>
-      <c r="E70" t="inlineStr">
-        <is>
-          <t>Oligo.3</t>
-        </is>
-      </c>
       <c r="F70" t="inlineStr">
         <is>
+          <t>Oligo.3</t>
+        </is>
+      </c>
+      <c r="G70" t="inlineStr">
+        <is>
           <t>DEG LR interactions: NLGN1 -&gt; NRXN1,NLGN4X -&gt; NRXN1,NRXN1 -&gt; NLGN1,NXPH1 -&gt; NRXN1</t>
         </is>
       </c>
-      <c r="G70" t="b">
+      <c r="H70" t="b">
         <v>1</v>
       </c>
     </row>
     <row r="71">
       <c r="A71" t="inlineStr">
         <is>
+          <t>ENSG00000021645</t>
+        </is>
+      </c>
+      <c r="B71" t="inlineStr">
+        <is>
           <t>NRXN3</t>
         </is>
       </c>
-      <c r="B71" t="b">
-        <v>0</v>
-      </c>
-      <c r="C71">
-        <v>1</v>
-      </c>
-      <c r="D71" t="inlineStr">
+      <c r="C71" t="b">
+        <v>0</v>
+      </c>
+      <c r="D71">
+        <v>1</v>
+      </c>
+      <c r="E71" t="inlineStr">
         <is>
           <t>DEGs - LR</t>
         </is>
       </c>
-      <c r="E71" t="inlineStr">
-        <is>
-          <t>Oligo.3</t>
-        </is>
-      </c>
       <c r="F71" t="inlineStr">
         <is>
+          <t>Oligo.3</t>
+        </is>
+      </c>
+      <c r="G71" t="inlineStr">
+        <is>
           <t>DEG LR interactions: NLGN1 -&gt; NRXN3,NRXN3 -&gt; NLGN1,NXPH1 -&gt; NRXN3</t>
         </is>
       </c>
-      <c r="G71" t="b">
+      <c r="H71" t="b">
         <v>1</v>
       </c>
     </row>
     <row r="72">
       <c r="A72" t="inlineStr">
         <is>
+          <t>ENSG00000140538</t>
+        </is>
+      </c>
+      <c r="B72" t="inlineStr">
+        <is>
           <t>NTRK3</t>
         </is>
       </c>
-      <c r="B72" t="b">
-        <v>0</v>
-      </c>
-      <c r="C72">
+      <c r="C72" t="b">
+        <v>0</v>
+      </c>
+      <c r="D72">
         <v>2</v>
       </c>
-      <c r="D72" t="inlineStr">
+      <c r="E72" t="inlineStr">
         <is>
           <t>DEGs - LR, Marker - cell type specific</t>
         </is>
       </c>
-      <c r="E72" t="inlineStr">
-        <is>
-          <t>Oligo.3</t>
-        </is>
-      </c>
       <c r="F72" t="inlineStr">
         <is>
+          <t>Oligo.3</t>
+        </is>
+      </c>
+      <c r="G72" t="inlineStr">
+        <is>
           <t>Oligo.3 specific Enrich genes t= 9.07, DEG LR interactions: NTRK3 -&gt; PTPRD</t>
         </is>
       </c>
-      <c r="G72" t="b">
+      <c r="H72" t="b">
         <v>1</v>
       </c>
     </row>
     <row r="73">
       <c r="A73" t="inlineStr">
         <is>
+          <t>ENSG00000228474</t>
+        </is>
+      </c>
+      <c r="B73" t="inlineStr">
+        <is>
           <t>OST4</t>
         </is>
       </c>
-      <c r="B73" t="b">
-        <v>0</v>
-      </c>
-      <c r="C73">
-        <v>1</v>
-      </c>
-      <c r="D73" t="inlineStr">
+      <c r="C73" t="b">
+        <v>0</v>
+      </c>
+      <c r="D73">
+        <v>1</v>
+      </c>
+      <c r="E73" t="inlineStr">
         <is>
           <t>Marker - SpD</t>
         </is>
       </c>
-      <c r="E73" t="inlineStr">
+      <c r="F73" t="inlineStr">
         <is>
           <t>LD~Sp09D02</t>
         </is>
       </c>
-      <c r="F73" t="inlineStr">
+      <c r="G73" t="inlineStr">
         <is>
           <t>SpD MeanRatio gene: LD~Sp09D02/L2.3~Sp09D01: 1.109</t>
         </is>
       </c>
-      <c r="G73" t="b">
+      <c r="H73" t="b">
         <v>1</v>
       </c>
     </row>
     <row r="74">
       <c r="A74" t="inlineStr">
         <is>
+          <t>ENSG00000100836</t>
+        </is>
+      </c>
+      <c r="B74" t="inlineStr">
+        <is>
           <t>PABPN1</t>
         </is>
       </c>
-      <c r="B74" t="b">
-        <v>0</v>
-      </c>
-      <c r="C74">
+      <c r="C74" t="b">
+        <v>0</v>
+      </c>
+      <c r="D74">
         <v>2</v>
       </c>
-      <c r="D74" t="inlineStr">
+      <c r="E74" t="inlineStr">
         <is>
           <t>Marker - cell type specific</t>
         </is>
       </c>
-      <c r="E74" t="inlineStr">
+      <c r="F74" t="inlineStr">
         <is>
           <t>Astro.3, Excit.L2_5.1</t>
         </is>
       </c>
-      <c r="F74" t="inlineStr">
+      <c r="G74" t="inlineStr">
         <is>
           <t>Astro.3 specific MR genes - Astro.3/Astro.1: 1.046, Excit.L2_5.1 specific Enrich genes t= 9.16</t>
         </is>
       </c>
-      <c r="G74" t="b">
+      <c r="H74" t="b">
         <v>1</v>
       </c>
     </row>
     <row r="75">
       <c r="A75" t="inlineStr">
         <is>
+          <t>ENSG00000228842</t>
+        </is>
+      </c>
+      <c r="B75" t="inlineStr">
+        <is>
           <t>PCDH9-AS2</t>
         </is>
       </c>
-      <c r="B75" t="b">
-        <v>0</v>
-      </c>
-      <c r="C75">
-        <v>1</v>
-      </c>
-      <c r="D75" t="inlineStr">
+      <c r="C75" t="b">
+        <v>0</v>
+      </c>
+      <c r="D75">
+        <v>1</v>
+      </c>
+      <c r="E75" t="inlineStr">
         <is>
           <t>Marker - cell type specific</t>
         </is>
       </c>
-      <c r="E75" t="inlineStr">
+      <c r="F75" t="inlineStr">
         <is>
           <t>Astro.1</t>
         </is>
       </c>
-      <c r="F75" t="inlineStr">
+      <c r="G75" t="inlineStr">
         <is>
           <t>Astro.1 specific MR genes - Astro.1/Astro.3: 1.486</t>
         </is>
       </c>
-      <c r="G75" t="b">
+      <c r="H75" t="b">
         <v>1</v>
       </c>
     </row>
     <row r="76">
       <c r="A76" t="inlineStr">
         <is>
+          <t>ENSG00000123560</t>
+        </is>
+      </c>
+      <c r="B76" t="inlineStr">
+        <is>
           <t>PLP1</t>
         </is>
       </c>
-      <c r="B76" t="b">
-        <v>0</v>
-      </c>
-      <c r="C76">
+      <c r="C76" t="b">
+        <v>0</v>
+      </c>
+      <c r="D76">
         <v>2</v>
       </c>
-      <c r="D76" t="inlineStr">
+      <c r="E76" t="inlineStr">
         <is>
           <t>DEG - carrier, Marker - cell type specific</t>
         </is>
       </c>
-      <c r="E76" t="inlineStr">
+      <c r="F76" t="inlineStr">
         <is>
           <t>Excit.L2_5.1, Oligo.3</t>
         </is>
       </c>
-      <c r="F76" t="inlineStr">
+      <c r="G76" t="inlineStr">
         <is>
           <t>Excit.L2_5.1 specific Enrich genes t= 8.05, DEG of interest: Oligo.3 down</t>
         </is>
       </c>
-      <c r="G76" t="b">
+      <c r="H76" t="b">
         <v>1</v>
       </c>
     </row>
     <row r="77">
       <c r="A77" t="inlineStr">
         <is>
+          <t>ENSG00000117600</t>
+        </is>
+      </c>
+      <c r="B77" t="inlineStr">
+        <is>
           <t>PLPPR4</t>
         </is>
       </c>
-      <c r="B77" t="b">
-        <v>0</v>
-      </c>
-      <c r="C77">
-        <v>1</v>
-      </c>
-      <c r="D77" t="inlineStr">
+      <c r="C77" t="b">
+        <v>0</v>
+      </c>
+      <c r="D77">
+        <v>1</v>
+      </c>
+      <c r="E77" t="inlineStr">
         <is>
           <t>DEG - mediation</t>
         </is>
       </c>
-      <c r="E77" t="inlineStr">
+      <c r="F77" t="inlineStr">
         <is>
           <t>Astro.1</t>
         </is>
       </c>
-      <c r="F77" t="inlineStr">
+      <c r="G77" t="inlineStr">
         <is>
           <t>mediation gene: mediator Astro.1</t>
         </is>
       </c>
-      <c r="G77" t="b">
+      <c r="H77" t="b">
         <v>1</v>
       </c>
     </row>
     <row r="78">
       <c r="A78" t="inlineStr">
         <is>
+          <t>ENSG00000184304</t>
+        </is>
+      </c>
+      <c r="B78" t="inlineStr">
+        <is>
           <t>PRKD1</t>
         </is>
       </c>
-      <c r="B78" t="b">
-        <v>0</v>
-      </c>
-      <c r="C78">
-        <v>1</v>
-      </c>
-      <c r="D78" t="inlineStr">
+      <c r="C78" t="b">
+        <v>0</v>
+      </c>
+      <c r="D78">
+        <v>1</v>
+      </c>
+      <c r="E78" t="inlineStr">
         <is>
           <t>DEG - carrier</t>
         </is>
       </c>
-      <c r="E78" t="inlineStr">
+      <c r="F78" t="inlineStr">
         <is>
           <t>Excit.L5.2</t>
         </is>
       </c>
-      <c r="F78" t="inlineStr">
+      <c r="G78" t="inlineStr">
         <is>
           <t>DEG carrier top:  Excit.L5.2 down</t>
         </is>
       </c>
-      <c r="G78" t="b">
+      <c r="H78" t="b">
         <v>1</v>
       </c>
     </row>
     <row r="79">
       <c r="A79" t="inlineStr">
         <is>
+          <t>ENSG00000107317</t>
+        </is>
+      </c>
+      <c r="B79" t="inlineStr">
+        <is>
           <t>PTGDS</t>
         </is>
       </c>
-      <c r="B79" t="b">
-        <v>0</v>
-      </c>
-      <c r="C79">
-        <v>1</v>
-      </c>
-      <c r="D79" t="inlineStr">
+      <c r="C79" t="b">
+        <v>0</v>
+      </c>
+      <c r="D79">
+        <v>1</v>
+      </c>
+      <c r="E79" t="inlineStr">
         <is>
           <t>Marker - cell type specific</t>
         </is>
       </c>
-      <c r="E79" t="inlineStr">
+      <c r="F79" t="inlineStr">
         <is>
           <t>Astro.2</t>
         </is>
       </c>
-      <c r="F79" t="inlineStr">
+      <c r="G79" t="inlineStr">
         <is>
           <t>Astro.2 specific MR genes - Astro.2/Astro.5: 1.01, Astro.2 specific Enrich genes t= 4.92</t>
         </is>
       </c>
-      <c r="G79" t="b">
+      <c r="H79" t="b">
         <v>1</v>
       </c>
     </row>
     <row r="80">
       <c r="A80" t="inlineStr">
         <is>
+          <t>ENSG00000153707</t>
+        </is>
+      </c>
+      <c r="B80" t="inlineStr">
+        <is>
           <t>PTPRD</t>
         </is>
       </c>
-      <c r="B80" t="b">
-        <v>0</v>
-      </c>
-      <c r="C80">
-        <v>1</v>
-      </c>
-      <c r="D80" t="inlineStr">
+      <c r="C80" t="b">
+        <v>0</v>
+      </c>
+      <c r="D80">
+        <v>1</v>
+      </c>
+      <c r="E80" t="inlineStr">
         <is>
           <t>DEGs - LR</t>
         </is>
       </c>
-      <c r="E80" t="inlineStr">
-        <is>
-          <t>Oligo.3</t>
-        </is>
-      </c>
       <c r="F80" t="inlineStr">
         <is>
+          <t>Oligo.3</t>
+        </is>
+      </c>
+      <c r="G80" t="inlineStr">
+        <is>
           <t>DEG LR interactions: IL1RAPL1 -&gt; PTPRD,NTRK3 -&gt; PTPRD</t>
         </is>
       </c>
-      <c r="G80" t="b">
+      <c r="H80" t="b">
         <v>1</v>
       </c>
     </row>
     <row r="81">
       <c r="A81" t="inlineStr">
         <is>
+          <t>ENSG00000079974</t>
+        </is>
+      </c>
+      <c r="B81" t="inlineStr">
+        <is>
           <t>RABL2B</t>
         </is>
       </c>
-      <c r="B81" t="b">
-        <v>0</v>
-      </c>
-      <c r="C81">
-        <v>1</v>
-      </c>
-      <c r="D81" t="inlineStr">
+      <c r="C81" t="b">
+        <v>0</v>
+      </c>
+      <c r="D81">
+        <v>1</v>
+      </c>
+      <c r="E81" t="inlineStr">
         <is>
           <t>DEG - ancestry</t>
         </is>
       </c>
-      <c r="E81" t="inlineStr">
-        <is>
-          <t>Oligo.3</t>
-        </is>
-      </c>
       <c r="F81" t="inlineStr">
         <is>
+          <t>Oligo.3</t>
+        </is>
+      </c>
+      <c r="G81" t="inlineStr">
+        <is>
           <t>DEG Ancestry op: Oligo.3 AA_up-EA_down*</t>
         </is>
       </c>
-      <c r="G81" t="b">
+      <c r="H81" t="b">
         <v>1</v>
       </c>
     </row>
     <row r="82">
       <c r="A82" t="inlineStr">
         <is>
+          <t>ENSG00000177954</t>
+        </is>
+      </c>
+      <c r="B82" t="inlineStr">
+        <is>
           <t>RPS27</t>
         </is>
       </c>
-      <c r="B82" t="b">
-        <v>0</v>
-      </c>
-      <c r="C82">
-        <v>1</v>
-      </c>
-      <c r="D82" t="inlineStr">
+      <c r="C82" t="b">
+        <v>0</v>
+      </c>
+      <c r="D82">
+        <v>1</v>
+      </c>
+      <c r="E82" t="inlineStr">
         <is>
           <t>Marker - cell type specific</t>
         </is>
       </c>
-      <c r="E82" t="inlineStr">
+      <c r="F82" t="inlineStr">
         <is>
           <t>Astro.3</t>
         </is>
       </c>
-      <c r="F82" t="inlineStr">
+      <c r="G82" t="inlineStr">
         <is>
           <t>Astro.3 specific MR genes - Astro.3/Astro.2: 1.109</t>
         </is>
       </c>
-      <c r="G82" t="b">
+      <c r="H82" t="b">
         <v>1</v>
       </c>
     </row>
     <row r="83">
       <c r="A83" t="inlineStr">
         <is>
+          <t>ENSG00000250722</t>
+        </is>
+      </c>
+      <c r="B83" t="inlineStr">
+        <is>
           <t>SELENOP</t>
         </is>
       </c>
-      <c r="B83" t="b">
-        <v>0</v>
-      </c>
-      <c r="C83">
-        <v>1</v>
-      </c>
-      <c r="D83" t="inlineStr">
+      <c r="C83" t="b">
+        <v>0</v>
+      </c>
+      <c r="D83">
+        <v>1</v>
+      </c>
+      <c r="E83" t="inlineStr">
         <is>
           <t>MOFA - Factor3</t>
         </is>
       </c>
-      <c r="E83" t="inlineStr">
-        <is>
-          <t>Oligo.3</t>
-        </is>
-      </c>
       <c r="F83" t="inlineStr">
         <is>
+          <t>Oligo.3</t>
+        </is>
+      </c>
+      <c r="G83" t="inlineStr">
+        <is>
           <t>MOFA Oligo.3 Factor3-</t>
         </is>
       </c>
-      <c r="G83" t="b">
+      <c r="H83" t="b">
         <v>1</v>
       </c>
     </row>
     <row r="84">
       <c r="A84" t="inlineStr">
         <is>
+          <t>ENSG00000137872</t>
+        </is>
+      </c>
+      <c r="B84" t="inlineStr">
+        <is>
           <t>SEMA6D</t>
         </is>
       </c>
-      <c r="B84" t="b">
-        <v>0</v>
-      </c>
-      <c r="C84">
-        <v>1</v>
-      </c>
-      <c r="D84" t="inlineStr">
+      <c r="C84" t="b">
+        <v>0</v>
+      </c>
+      <c r="D84">
+        <v>1</v>
+      </c>
+      <c r="E84" t="inlineStr">
         <is>
           <t>Marker - cell type specific</t>
         </is>
       </c>
-      <c r="E84" t="inlineStr">
+      <c r="F84" t="inlineStr">
         <is>
           <t>Oligo.1</t>
         </is>
       </c>
-      <c r="F84" t="inlineStr">
+      <c r="G84" t="inlineStr">
         <is>
           <t>Oligo.1 specific MR genes - Oligo.1/Oligo.2: 1.179</t>
         </is>
       </c>
-      <c r="G84" t="b">
+      <c r="H84" t="b">
         <v>1</v>
       </c>
     </row>
     <row r="85">
       <c r="A85" t="inlineStr">
         <is>
+          <t>ENSG00000100359</t>
+        </is>
+      </c>
+      <c r="B85" t="inlineStr">
+        <is>
           <t>SGSM3</t>
         </is>
       </c>
-      <c r="B85" t="b">
-        <v>0</v>
-      </c>
-      <c r="C85">
-        <v>1</v>
-      </c>
-      <c r="D85" t="inlineStr">
+      <c r="C85" t="b">
+        <v>0</v>
+      </c>
+      <c r="D85">
+        <v>1</v>
+      </c>
+      <c r="E85" t="inlineStr">
         <is>
           <t>DEG - ancestry</t>
         </is>
       </c>
-      <c r="E85" t="inlineStr">
-        <is>
-          <t>Oligo.3</t>
-        </is>
-      </c>
       <c r="F85" t="inlineStr">
         <is>
+          <t>Oligo.3</t>
+        </is>
+      </c>
+      <c r="G85" t="inlineStr">
+        <is>
           <t>DEG Ancestry op: Oligo.3 AA_up*-EA_down</t>
         </is>
       </c>
-      <c r="G85" t="b">
+      <c r="H85" t="b">
         <v>1</v>
       </c>
     </row>
     <row r="86">
       <c r="A86" t="inlineStr">
         <is>
+          <t>ENSG00000155886</t>
+        </is>
+      </c>
+      <c r="B86" t="inlineStr">
+        <is>
           <t>SLC24A2</t>
         </is>
       </c>
-      <c r="B86" t="b">
-        <v>0</v>
-      </c>
-      <c r="C86">
-        <v>1</v>
-      </c>
-      <c r="D86" t="inlineStr">
+      <c r="C86" t="b">
+        <v>0</v>
+      </c>
+      <c r="D86">
+        <v>1</v>
+      </c>
+      <c r="E86" t="inlineStr">
         <is>
           <t>Marker - cell type specific</t>
         </is>
       </c>
-      <c r="E86" t="inlineStr">
+      <c r="F86" t="inlineStr">
         <is>
           <t>Astro.3</t>
         </is>
       </c>
-      <c r="F86" t="inlineStr">
+      <c r="G86" t="inlineStr">
         <is>
           <t>Astro.3 specific Enrich genes t= 8.18</t>
         </is>
       </c>
-      <c r="G86" t="b">
+      <c r="H86" t="b">
         <v>1</v>
       </c>
     </row>
     <row r="87">
       <c r="A87" t="inlineStr">
         <is>
+          <t>ENSG00000080493</t>
+        </is>
+      </c>
+      <c r="B87" t="inlineStr">
+        <is>
           <t>SLC4A4</t>
         </is>
       </c>
-      <c r="B87" t="b">
-        <v>0</v>
-      </c>
-      <c r="C87">
-        <v>1</v>
-      </c>
-      <c r="D87" t="inlineStr">
+      <c r="C87" t="b">
+        <v>0</v>
+      </c>
+      <c r="D87">
+        <v>1</v>
+      </c>
+      <c r="E87" t="inlineStr">
         <is>
           <t>MOFA - Factor3</t>
         </is>
       </c>
-      <c r="E87" t="inlineStr">
-        <is>
-          <t>Oligo.3</t>
-        </is>
-      </c>
       <c r="F87" t="inlineStr">
         <is>
+          <t>Oligo.3</t>
+        </is>
+      </c>
+      <c r="G87" t="inlineStr">
+        <is>
           <t>MOFA Oligo.3 Factor3+</t>
         </is>
       </c>
-      <c r="G87" t="b">
+      <c r="H87" t="b">
         <v>1</v>
       </c>
     </row>
     <row r="88">
       <c r="A88" t="inlineStr">
         <is>
+          <t>ENSG00000151012</t>
+        </is>
+      </c>
+      <c r="B88" t="inlineStr">
+        <is>
           <t>SLC7A11</t>
         </is>
       </c>
-      <c r="B88" t="b">
-        <v>0</v>
-      </c>
-      <c r="C88">
-        <v>1</v>
-      </c>
-      <c r="D88" t="inlineStr">
+      <c r="C88" t="b">
+        <v>0</v>
+      </c>
+      <c r="D88">
+        <v>1</v>
+      </c>
+      <c r="E88" t="inlineStr">
         <is>
           <t>DEG - carrier</t>
         </is>
       </c>
-      <c r="E88" t="inlineStr">
+      <c r="F88" t="inlineStr">
         <is>
           <t>Excit.L5.2</t>
         </is>
       </c>
-      <c r="F88" t="inlineStr">
+      <c r="G88" t="inlineStr">
         <is>
           <t>DEG carrier top:  Excit.L5.2 up</t>
         </is>
       </c>
-      <c r="G88" t="b">
+      <c r="H88" t="b">
         <v>1</v>
       </c>
     </row>
     <row r="89">
       <c r="A89" t="inlineStr">
         <is>
+          <t>ENSG00000104852</t>
+        </is>
+      </c>
+      <c r="B89" t="inlineStr">
+        <is>
           <t>SNRNP70</t>
         </is>
       </c>
-      <c r="B89" t="b">
-        <v>0</v>
-      </c>
-      <c r="C89">
-        <v>1</v>
-      </c>
-      <c r="D89" t="inlineStr">
+      <c r="C89" t="b">
+        <v>0</v>
+      </c>
+      <c r="D89">
+        <v>1</v>
+      </c>
+      <c r="E89" t="inlineStr">
         <is>
           <t>Marker - cell type specific</t>
         </is>
       </c>
-      <c r="E89" t="inlineStr">
+      <c r="F89" t="inlineStr">
         <is>
           <t>Astro.2</t>
         </is>
       </c>
-      <c r="F89" t="inlineStr">
+      <c r="G89" t="inlineStr">
         <is>
           <t>Astro.2 specific MR genes - Astro.2/Astro.3: 1.023</t>
         </is>
       </c>
-      <c r="G89" t="b">
+      <c r="H89" t="b">
         <v>1</v>
       </c>
     </row>
     <row r="90">
       <c r="A90" t="inlineStr">
         <is>
+          <t>ENSG00000101400</t>
+        </is>
+      </c>
+      <c r="B90" t="inlineStr">
+        <is>
           <t>SNTA1</t>
         </is>
       </c>
-      <c r="B90" t="b">
-        <v>0</v>
-      </c>
-      <c r="C90">
-        <v>1</v>
-      </c>
-      <c r="D90" t="inlineStr">
+      <c r="C90" t="b">
+        <v>0</v>
+      </c>
+      <c r="D90">
+        <v>1</v>
+      </c>
+      <c r="E90" t="inlineStr">
         <is>
           <t>Marker - cell type specific</t>
         </is>
       </c>
-      <c r="E90" t="inlineStr">
+      <c r="F90" t="inlineStr">
         <is>
           <t>Astro.2</t>
         </is>
       </c>
-      <c r="F90" t="inlineStr">
+      <c r="G90" t="inlineStr">
         <is>
           <t>Astro.2 specific Enrich genes t= 4.98</t>
         </is>
       </c>
-      <c r="G90" t="b">
+      <c r="H90" t="b">
         <v>1</v>
       </c>
     </row>
     <row r="91">
       <c r="A91" t="inlineStr">
         <is>
+          <t>ENSG00000120451</t>
+        </is>
+      </c>
+      <c r="B91" t="inlineStr">
+        <is>
           <t>SNX19</t>
         </is>
       </c>
-      <c r="B91" t="b">
-        <v>0</v>
-      </c>
-      <c r="C91">
-        <v>1</v>
-      </c>
-      <c r="D91" t="inlineStr">
+      <c r="C91" t="b">
+        <v>0</v>
+      </c>
+      <c r="D91">
+        <v>1</v>
+      </c>
+      <c r="E91" t="inlineStr">
         <is>
           <t>DEG - ancestry</t>
         </is>
       </c>
-      <c r="E91" t="inlineStr">
-        <is>
-          <t>Oligo.3</t>
-        </is>
-      </c>
       <c r="F91" t="inlineStr">
         <is>
+          <t>Oligo.3</t>
+        </is>
+      </c>
+      <c r="G91" t="inlineStr">
+        <is>
           <t>DEG Ancestry op: Oligo.3 AA_down*-EA_up</t>
         </is>
       </c>
-      <c r="G91" t="b">
+      <c r="H91" t="b">
         <v>1</v>
       </c>
     </row>
     <row r="92">
       <c r="A92" t="inlineStr">
         <is>
+          <t>ENSG00000095637</t>
+        </is>
+      </c>
+      <c r="B92" t="inlineStr">
+        <is>
           <t>SORBS1</t>
         </is>
       </c>
-      <c r="B92" t="b">
-        <v>0</v>
-      </c>
-      <c r="C92">
-        <v>1</v>
-      </c>
-      <c r="D92" t="inlineStr">
+      <c r="C92" t="b">
+        <v>0</v>
+      </c>
+      <c r="D92">
+        <v>1</v>
+      </c>
+      <c r="E92" t="inlineStr">
         <is>
           <t>DEG - mediation</t>
         </is>
       </c>
-      <c r="E92" t="inlineStr">
-        <is>
-          <t>Oligo.3</t>
-        </is>
-      </c>
       <c r="F92" t="inlineStr">
         <is>
+          <t>Oligo.3</t>
+        </is>
+      </c>
+      <c r="G92" t="inlineStr">
+        <is>
           <t>mediation gene: outcome Oligo.3</t>
         </is>
       </c>
-      <c r="G92" t="b">
+      <c r="H92" t="b">
         <v>1</v>
       </c>
     </row>
     <row r="93">
       <c r="A93" t="inlineStr">
         <is>
+          <t>ENSG00000110693</t>
+        </is>
+      </c>
+      <c r="B93" t="inlineStr">
+        <is>
           <t>SOX6</t>
         </is>
       </c>
-      <c r="B93" t="b">
-        <v>0</v>
-      </c>
-      <c r="C93">
-        <v>1</v>
-      </c>
-      <c r="D93" t="inlineStr">
+      <c r="C93" t="b">
+        <v>0</v>
+      </c>
+      <c r="D93">
+        <v>1</v>
+      </c>
+      <c r="E93" t="inlineStr">
         <is>
           <t>DEG - mediation</t>
         </is>
       </c>
-      <c r="E93" t="inlineStr">
-        <is>
-          <t>Oligo.3</t>
-        </is>
-      </c>
       <c r="F93" t="inlineStr">
         <is>
+          <t>Oligo.3</t>
+        </is>
+      </c>
+      <c r="G93" t="inlineStr">
+        <is>
           <t>mediation gene: outcome Oligo.3</t>
         </is>
       </c>
-      <c r="G93" t="b">
+      <c r="H93" t="b">
         <v>1</v>
       </c>
     </row>
     <row r="94">
       <c r="A94" t="inlineStr">
         <is>
+          <t>ENSG00000115415</t>
+        </is>
+      </c>
+      <c r="B94" t="inlineStr">
+        <is>
           <t>STAT1</t>
         </is>
       </c>
-      <c r="B94" t="b">
-        <v>0</v>
-      </c>
-      <c r="C94">
-        <v>1</v>
-      </c>
-      <c r="D94" t="inlineStr">
+      <c r="C94" t="b">
+        <v>0</v>
+      </c>
+      <c r="D94">
+        <v>1</v>
+      </c>
+      <c r="E94" t="inlineStr">
         <is>
           <t>DEG - carrier</t>
         </is>
       </c>
-      <c r="E94" t="inlineStr">
-        <is>
-          <t>Oligo.3</t>
-        </is>
-      </c>
       <c r="F94" t="inlineStr">
         <is>
+          <t>Oligo.3</t>
+        </is>
+      </c>
+      <c r="G94" t="inlineStr">
+        <is>
           <t>DEG of interest: Oligo.3 up</t>
         </is>
       </c>
-      <c r="G94" t="b">
+      <c r="H94" t="b">
         <v>1</v>
       </c>
     </row>
     <row r="95">
       <c r="A95" t="inlineStr">
         <is>
+          <t>ENSG00000138378</t>
+        </is>
+      </c>
+      <c r="B95" t="inlineStr">
+        <is>
           <t>STAT4</t>
         </is>
       </c>
-      <c r="B95" t="b">
-        <v>0</v>
-      </c>
-      <c r="C95">
-        <v>1</v>
-      </c>
-      <c r="D95" t="inlineStr">
+      <c r="C95" t="b">
+        <v>0</v>
+      </c>
+      <c r="D95">
+        <v>1</v>
+      </c>
+      <c r="E95" t="inlineStr">
         <is>
           <t>DEG - carrier</t>
         </is>
       </c>
-      <c r="E95" t="inlineStr">
-        <is>
-          <t>Oligo.3</t>
-        </is>
-      </c>
       <c r="F95" t="inlineStr">
         <is>
+          <t>Oligo.3</t>
+        </is>
+      </c>
+      <c r="G95" t="inlineStr">
+        <is>
           <t>DEG of interest: Oligo.3 up</t>
         </is>
       </c>
-      <c r="G95" t="b">
+      <c r="H95" t="b">
         <v>1</v>
       </c>
     </row>
     <row r="96">
       <c r="A96" t="inlineStr">
         <is>
+          <t>ENSG00000185518</t>
+        </is>
+      </c>
+      <c r="B96" t="inlineStr">
+        <is>
           <t>SV2B</t>
         </is>
       </c>
-      <c r="B96" t="b">
-        <v>0</v>
-      </c>
-      <c r="C96">
-        <v>1</v>
-      </c>
-      <c r="D96" t="inlineStr">
+      <c r="C96" t="b">
+        <v>0</v>
+      </c>
+      <c r="D96">
+        <v>1</v>
+      </c>
+      <c r="E96" t="inlineStr">
         <is>
           <t>DEG - mediation</t>
         </is>
       </c>
-      <c r="E96" t="inlineStr">
+      <c r="F96" t="inlineStr">
         <is>
           <t>Astro.2</t>
         </is>
       </c>
-      <c r="F96" t="inlineStr">
+      <c r="G96" t="inlineStr">
         <is>
           <t>mediation gene: mediator Astro.2</t>
         </is>
       </c>
-      <c r="G96" t="b">
+      <c r="H96" t="b">
         <v>1</v>
       </c>
     </row>
     <row r="97">
       <c r="A97" t="inlineStr">
         <is>
+          <t>ENSG00000136560</t>
+        </is>
+      </c>
+      <c r="B97" t="inlineStr">
+        <is>
           <t>TANK</t>
         </is>
       </c>
-      <c r="B97" t="b">
-        <v>0</v>
-      </c>
-      <c r="C97">
-        <v>1</v>
-      </c>
-      <c r="D97" t="inlineStr">
+      <c r="C97" t="b">
+        <v>0</v>
+      </c>
+      <c r="D97">
+        <v>1</v>
+      </c>
+      <c r="E97" t="inlineStr">
         <is>
           <t>Marker - cell type specific</t>
         </is>
       </c>
-      <c r="E97" t="inlineStr">
+      <c r="F97" t="inlineStr">
         <is>
           <t>Excit.L5.2</t>
         </is>
       </c>
-      <c r="F97" t="inlineStr">
+      <c r="G97" t="inlineStr">
         <is>
           <t>Excit.L5.2 specific Enrich genes t= 13.71</t>
         </is>
       </c>
-      <c r="G97" t="b">
+      <c r="H97" t="b">
         <v>1</v>
       </c>
     </row>
     <row r="98">
       <c r="A98" t="inlineStr">
         <is>
+          <t>ENSG00000137462</t>
+        </is>
+      </c>
+      <c r="B98" t="inlineStr">
+        <is>
           <t>TLR2</t>
         </is>
       </c>
-      <c r="B98" t="b">
-        <v>0</v>
-      </c>
-      <c r="C98">
-        <v>1</v>
-      </c>
-      <c r="D98" t="inlineStr">
+      <c r="C98" t="b">
+        <v>0</v>
+      </c>
+      <c r="D98">
+        <v>1</v>
+      </c>
+      <c r="E98" t="inlineStr">
         <is>
           <t>DEG - carrier</t>
         </is>
       </c>
-      <c r="E98" t="inlineStr">
-        <is>
-          <t>Oligo.3</t>
-        </is>
-      </c>
       <c r="F98" t="inlineStr">
         <is>
+          <t>Oligo.3</t>
+        </is>
+      </c>
+      <c r="G98" t="inlineStr">
+        <is>
           <t>DEG of interest: Oligo.3 up</t>
         </is>
       </c>
-      <c r="G98" t="b">
+      <c r="H98" t="b">
         <v>1</v>
       </c>
     </row>
     <row r="99">
       <c r="A99" t="inlineStr">
         <is>
+          <t>ENSG00000061938</t>
+        </is>
+      </c>
+      <c r="B99" t="inlineStr">
+        <is>
           <t>TNK2</t>
         </is>
       </c>
-      <c r="B99" t="b">
-        <v>0</v>
-      </c>
-      <c r="C99">
-        <v>1</v>
-      </c>
-      <c r="D99" t="inlineStr">
+      <c r="C99" t="b">
+        <v>0</v>
+      </c>
+      <c r="D99">
+        <v>1</v>
+      </c>
+      <c r="E99" t="inlineStr">
         <is>
           <t>Marker - cell type specific</t>
         </is>
       </c>
-      <c r="E99" t="inlineStr">
+      <c r="F99" t="inlineStr">
         <is>
           <t>OPC.5</t>
         </is>
       </c>
-      <c r="F99" t="inlineStr">
+      <c r="G99" t="inlineStr">
         <is>
           <t>OPC.5 specific MR genes - OPC.5/OPC.2: 1.04</t>
         </is>
       </c>
-      <c r="G99" t="b">
+      <c r="H99" t="b">
         <v>1</v>
       </c>
     </row>
     <row r="100">
       <c r="A100" t="inlineStr">
         <is>
+          <t>ENSG00000173960</t>
+        </is>
+      </c>
+      <c r="B100" t="inlineStr">
+        <is>
           <t>UBXN2A</t>
         </is>
       </c>
-      <c r="B100" t="b">
-        <v>0</v>
-      </c>
-      <c r="C100">
-        <v>1</v>
-      </c>
-      <c r="D100" t="inlineStr">
+      <c r="C100" t="b">
+        <v>0</v>
+      </c>
+      <c r="D100">
+        <v>1</v>
+      </c>
+      <c r="E100" t="inlineStr">
         <is>
           <t>DEG - ancestry</t>
         </is>
       </c>
-      <c r="E100" t="inlineStr">
-        <is>
-          <t>Oligo.3</t>
-        </is>
-      </c>
       <c r="F100" t="inlineStr">
         <is>
+          <t>Oligo.3</t>
+        </is>
+      </c>
+      <c r="G100" t="inlineStr">
+        <is>
           <t>DEG Ancestry op: Oligo.3 AA_down*-EA_up</t>
         </is>
       </c>
-      <c r="G100" t="b">
+      <c r="H100" t="b">
         <v>1</v>
       </c>
     </row>
     <row r="101">
       <c r="A101" t="inlineStr">
         <is>
+          <t>ENSG00000143952</t>
+        </is>
+      </c>
+      <c r="B101" t="inlineStr">
+        <is>
           <t>VPS54</t>
         </is>
       </c>
-      <c r="B101" t="b">
-        <v>0</v>
-      </c>
-      <c r="C101">
-        <v>1</v>
-      </c>
-      <c r="D101" t="inlineStr">
+      <c r="C101" t="b">
+        <v>0</v>
+      </c>
+      <c r="D101">
+        <v>1</v>
+      </c>
+      <c r="E101" t="inlineStr">
         <is>
           <t>DEG - ancestry</t>
         </is>
       </c>
-      <c r="E101" t="inlineStr">
-        <is>
-          <t>Oligo.3</t>
-        </is>
-      </c>
       <c r="F101" t="inlineStr">
         <is>
+          <t>Oligo.3</t>
+        </is>
+      </c>
+      <c r="G101" t="inlineStr">
+        <is>
           <t>DEG Ancestry op: Oligo.3 AA_down*-EA_up</t>
         </is>
       </c>
-      <c r="G101" t="b">
+      <c r="H101" t="b">
         <v>1</v>
       </c>
     </row>

</xml_diff>

<commit_message>
Update custom probe list based on Feb27 review - add review table + updated tables
</commit_message>
<xml_diff>
--- a/processed-data/21_Xenium/02_xenium_compile_custom/ERC_Xenium_select_custom_probes.xlsx
+++ b/processed-data/21_Xenium/02_xenium_compile_custom/ERC_Xenium_select_custom_probes.xlsx
@@ -351,7 +351,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:H101"/>
+  <dimension ref="A1:I101"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <sheetData>
     <row r="1" s="1" customFormat="1">
@@ -395,6 +395,11 @@
           <t>yesprobe</t>
         </is>
       </c>
+      <c r="I1" s="1" t="inlineStr">
+        <is>
+          <t>update</t>
+        </is>
+      </c>
     </row>
     <row r="2">
       <c r="A2" t="inlineStr">
@@ -431,6 +436,11 @@
       <c r="H2" t="b">
         <v>1</v>
       </c>
+      <c r="I2" t="inlineStr">
+        <is>
+          <t>Feb27</t>
+        </is>
+      </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
@@ -467,6 +477,11 @@
       <c r="H3" t="b">
         <v>1</v>
       </c>
+      <c r="I3" t="inlineStr">
+        <is>
+          <t>Feb27</t>
+        </is>
+      </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
@@ -503,6 +518,11 @@
       <c r="H4" t="b">
         <v>1</v>
       </c>
+      <c r="I4" t="inlineStr">
+        <is>
+          <t>Feb27</t>
+        </is>
+      </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
@@ -539,6 +559,11 @@
       <c r="H5" t="b">
         <v>1</v>
       </c>
+      <c r="I5" t="inlineStr">
+        <is>
+          <t>Feb27</t>
+        </is>
+      </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
@@ -575,6 +600,11 @@
       <c r="H6" t="b">
         <v>1</v>
       </c>
+      <c r="I6" t="inlineStr">
+        <is>
+          <t>Feb27</t>
+        </is>
+      </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
@@ -611,6 +641,11 @@
       <c r="H7" t="b">
         <v>1</v>
       </c>
+      <c r="I7" t="inlineStr">
+        <is>
+          <t>Feb27</t>
+        </is>
+      </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
@@ -647,6 +682,11 @@
       <c r="H8" t="b">
         <v>1</v>
       </c>
+      <c r="I8" t="inlineStr">
+        <is>
+          <t>Feb27</t>
+        </is>
+      </c>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
@@ -683,6 +723,11 @@
       <c r="H9" t="b">
         <v>1</v>
       </c>
+      <c r="I9" t="inlineStr">
+        <is>
+          <t>Feb27</t>
+        </is>
+      </c>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
@@ -719,6 +764,11 @@
       <c r="H10" t="b">
         <v>1</v>
       </c>
+      <c r="I10" t="inlineStr">
+        <is>
+          <t>Feb27</t>
+        </is>
+      </c>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
@@ -755,6 +805,11 @@
       <c r="H11" t="b">
         <v>1</v>
       </c>
+      <c r="I11" t="inlineStr">
+        <is>
+          <t>Feb27</t>
+        </is>
+      </c>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
@@ -791,16 +846,21 @@
       <c r="H12" t="b">
         <v>1</v>
       </c>
+      <c r="I12" t="inlineStr">
+        <is>
+          <t>Feb27</t>
+        </is>
+      </c>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>ENSG00000134389</t>
+          <t>ENSG00000133019</t>
         </is>
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>CFHR5</t>
+          <t>CHRM3</t>
         </is>
       </c>
       <c r="C13" t="b">
@@ -811,32 +871,37 @@
       </c>
       <c r="E13" t="inlineStr">
         <is>
-          <t>Marker - SpD</t>
+          <t>DEG - mediation</t>
         </is>
       </c>
       <c r="F13" t="inlineStr">
         <is>
-          <t>WM.uf_Sp09D07-WM_Sp09D06</t>
+          <t>Astro.3</t>
         </is>
       </c>
       <c r="G13" t="inlineStr">
         <is>
-          <t>SpD pw gene t=8.23</t>
+          <t>mediation gene: mediator Astro.3</t>
         </is>
       </c>
       <c r="H13" t="b">
         <v>1</v>
+      </c>
+      <c r="I13" t="inlineStr">
+        <is>
+          <t>Feb27</t>
+        </is>
       </c>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t>ENSG00000133019</t>
+          <t>ENSG00000171310</t>
         </is>
       </c>
       <c r="B14" t="inlineStr">
         <is>
-          <t>CHRM3</t>
+          <t>CHST11</t>
         </is>
       </c>
       <c r="C14" t="b">
@@ -847,32 +912,37 @@
       </c>
       <c r="E14" t="inlineStr">
         <is>
-          <t>DEG - mediation</t>
+          <t>DEG - carrier</t>
         </is>
       </c>
       <c r="F14" t="inlineStr">
         <is>
-          <t>Astro.3</t>
+          <t>Oligo.3</t>
         </is>
       </c>
       <c r="G14" t="inlineStr">
         <is>
-          <t>mediation gene: mediator Astro.3</t>
+          <t>DEG carrier top: Oligo.3 up logFC=2.82</t>
         </is>
       </c>
       <c r="H14" t="b">
         <v>1</v>
+      </c>
+      <c r="I14" t="inlineStr">
+        <is>
+          <t>Feb27</t>
+        </is>
       </c>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>ENSG00000171310</t>
+          <t>ENSG00000174469</t>
         </is>
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>CHST11</t>
+          <t>CNTNAP2</t>
         </is>
       </c>
       <c r="C15" t="b">
@@ -883,7 +953,7 @@
       </c>
       <c r="E15" t="inlineStr">
         <is>
-          <t>DEG - carrier</t>
+          <t>Marker - cell type specific</t>
         </is>
       </c>
       <c r="F15" t="inlineStr">
@@ -893,22 +963,27 @@
       </c>
       <c r="G15" t="inlineStr">
         <is>
-          <t>DEG carrier top: Oligo.3 up</t>
+          <t>Oligo.3 specific MR genes - Oligo.3/Oligo.2: 1.055</t>
         </is>
       </c>
       <c r="H15" t="b">
         <v>1</v>
+      </c>
+      <c r="I15" t="inlineStr">
+        <is>
+          <t>Feb27</t>
+        </is>
       </c>
     </row>
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t>ENSG00000174469</t>
+          <t>ENSG00000084636</t>
         </is>
       </c>
       <c r="B16" t="inlineStr">
         <is>
-          <t>CNTNAP2</t>
+          <t>COL16A1</t>
         </is>
       </c>
       <c r="C16" t="b">
@@ -924,27 +999,32 @@
       </c>
       <c r="F16" t="inlineStr">
         <is>
-          <t>Oligo.3</t>
+          <t>Astro.3</t>
         </is>
       </c>
       <c r="G16" t="inlineStr">
         <is>
-          <t>Oligo.3 specific MR genes - Oligo.3/Oligo.2: 1.055</t>
+          <t>Astro.3 specific MR genes - Astro.3/Astro.2: 1.061</t>
         </is>
       </c>
       <c r="H16" t="b">
         <v>1</v>
+      </c>
+      <c r="I16" t="inlineStr">
+        <is>
+          <t>Feb27</t>
+        </is>
       </c>
     </row>
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t>ENSG00000084636</t>
+          <t>ENSG00000124749</t>
         </is>
       </c>
       <c r="B17" t="inlineStr">
         <is>
-          <t>COL16A1</t>
+          <t>COL21A1</t>
         </is>
       </c>
       <c r="C17" t="b">
@@ -955,32 +1035,37 @@
       </c>
       <c r="E17" t="inlineStr">
         <is>
-          <t>Marker - cell type specific</t>
+          <t>DEG - carrier</t>
         </is>
       </c>
       <c r="F17" t="inlineStr">
         <is>
-          <t>Astro.3</t>
+          <t>Oligo.3</t>
         </is>
       </c>
       <c r="G17" t="inlineStr">
         <is>
-          <t>Astro.3 specific MR genes - Astro.3/Astro.2: 1.061</t>
+          <t>DEG carrier top: Oligo.3 up logFC=2.79</t>
         </is>
       </c>
       <c r="H17" t="b">
         <v>1</v>
+      </c>
+      <c r="I17" t="inlineStr">
+        <is>
+          <t>Feb27</t>
+        </is>
       </c>
     </row>
     <row r="18">
       <c r="A18" t="inlineStr">
         <is>
-          <t>ENSG00000124749</t>
+          <t>ENSG00000172428</t>
         </is>
       </c>
       <c r="B18" t="inlineStr">
         <is>
-          <t>COL21A1</t>
+          <t>COPS9</t>
         </is>
       </c>
       <c r="C18" t="b">
@@ -991,32 +1076,37 @@
       </c>
       <c r="E18" t="inlineStr">
         <is>
-          <t>DEG - carrier</t>
+          <t>Marker - SpD</t>
         </is>
       </c>
       <c r="F18" t="inlineStr">
         <is>
-          <t>Oligo.3</t>
+          <t>LD~Sp09D02</t>
         </is>
       </c>
       <c r="G18" t="inlineStr">
         <is>
-          <t>DEG carrier top: Oligo.3 up</t>
+          <t>SpD MeanRatio gene: LD~Sp09D02/Inhib~Sp09D09: 1.112</t>
         </is>
       </c>
       <c r="H18" t="b">
         <v>1</v>
+      </c>
+      <c r="I18" t="inlineStr">
+        <is>
+          <t>Feb27</t>
+        </is>
       </c>
     </row>
     <row r="19">
       <c r="A19" t="inlineStr">
         <is>
-          <t>ENSG00000172428</t>
+          <t>ENSG00000196353</t>
         </is>
       </c>
       <c r="B19" t="inlineStr">
         <is>
-          <t>COPS9</t>
+          <t>CPNE4</t>
         </is>
       </c>
       <c r="C19" t="b">
@@ -1027,32 +1117,37 @@
       </c>
       <c r="E19" t="inlineStr">
         <is>
-          <t>Marker - SpD</t>
+          <t>DEG - carrier</t>
         </is>
       </c>
       <c r="F19" t="inlineStr">
         <is>
-          <t>LD~Sp09D02</t>
+          <t>Oligo.3</t>
         </is>
       </c>
       <c r="G19" t="inlineStr">
         <is>
-          <t>SpD MeanRatio gene: LD~Sp09D02/Inhib~Sp09D09: 1.112</t>
+          <t>DEG of interest: Oligo.3 up logFC=1.87</t>
         </is>
       </c>
       <c r="H19" t="b">
         <v>1</v>
+      </c>
+      <c r="I19" t="inlineStr">
+        <is>
+          <t>Mar2</t>
+        </is>
       </c>
     </row>
     <row r="20">
       <c r="A20" t="inlineStr">
         <is>
-          <t>ENSG00000157851</t>
+          <t>ENSG00000004975</t>
         </is>
       </c>
       <c r="B20" t="inlineStr">
         <is>
-          <t>DPYSL5</t>
+          <t>DVL2</t>
         </is>
       </c>
       <c r="C20" t="b">
@@ -1063,32 +1158,37 @@
       </c>
       <c r="E20" t="inlineStr">
         <is>
-          <t>Marker - cell type global</t>
+          <t>DEG - ancestry</t>
         </is>
       </c>
       <c r="F20" t="inlineStr">
         <is>
-          <t>Oligo.2</t>
+          <t>Oligo.3</t>
         </is>
       </c>
       <c r="G20" t="inlineStr">
         <is>
-          <t>globl MR genes -  Oligo.2/Oligo.1: 1.557</t>
+          <t>DEG Ancestry op: Oligo.3 AA_up-EA_down*</t>
         </is>
       </c>
       <c r="H20" t="b">
         <v>1</v>
+      </c>
+      <c r="I20" t="inlineStr">
+        <is>
+          <t>Feb27</t>
+        </is>
       </c>
     </row>
     <row r="21">
       <c r="A21" t="inlineStr">
         <is>
-          <t>ENSG00000004975</t>
+          <t>ENSG00000171617</t>
         </is>
       </c>
       <c r="B21" t="inlineStr">
         <is>
-          <t>DVL2</t>
+          <t>ENC1</t>
         </is>
       </c>
       <c r="C21" t="b">
@@ -1099,7 +1199,7 @@
       </c>
       <c r="E21" t="inlineStr">
         <is>
-          <t>DEG - ancestry</t>
+          <t>DEG - mediation</t>
         </is>
       </c>
       <c r="F21" t="inlineStr">
@@ -1109,22 +1209,27 @@
       </c>
       <c r="G21" t="inlineStr">
         <is>
-          <t>DEG Ancestry op: Oligo.3 AA_up-EA_down*</t>
+          <t>mediation gene: outcome Oligo.3</t>
         </is>
       </c>
       <c r="H21" t="b">
         <v>1</v>
+      </c>
+      <c r="I21" t="inlineStr">
+        <is>
+          <t>Feb27</t>
+        </is>
       </c>
     </row>
     <row r="22">
       <c r="A22" t="inlineStr">
         <is>
-          <t>ENSG00000171617</t>
+          <t>ENSG00000178568</t>
         </is>
       </c>
       <c r="B22" t="inlineStr">
         <is>
-          <t>ENC1</t>
+          <t>ERBB4</t>
         </is>
       </c>
       <c r="C22" t="b">
@@ -1135,32 +1240,37 @@
       </c>
       <c r="E22" t="inlineStr">
         <is>
-          <t>DEG - mediation</t>
+          <t>Marker - cell type specific</t>
         </is>
       </c>
       <c r="F22" t="inlineStr">
         <is>
-          <t>Oligo.3</t>
+          <t>Oligo.1</t>
         </is>
       </c>
       <c r="G22" t="inlineStr">
         <is>
-          <t>mediation gene: outcome Oligo.3</t>
+          <t>Oligo.1 specific Enrich genes t= 5.58</t>
         </is>
       </c>
       <c r="H22" t="b">
         <v>1</v>
+      </c>
+      <c r="I22" t="inlineStr">
+        <is>
+          <t>Feb27</t>
+        </is>
       </c>
     </row>
     <row r="23">
       <c r="A23" t="inlineStr">
         <is>
-          <t>ENSG00000178568</t>
+          <t>ENSG00000182473</t>
         </is>
       </c>
       <c r="B23" t="inlineStr">
         <is>
-          <t>ERBB4</t>
+          <t>EXOC7</t>
         </is>
       </c>
       <c r="C23" t="b">
@@ -1176,27 +1286,32 @@
       </c>
       <c r="F23" t="inlineStr">
         <is>
-          <t>Oligo.1</t>
+          <t>OPC.5</t>
         </is>
       </c>
       <c r="G23" t="inlineStr">
         <is>
-          <t>Oligo.1 specific Enrich genes t= 5.58</t>
+          <t>OPC.5 specific Enrich genes t= 7.33</t>
         </is>
       </c>
       <c r="H23" t="b">
         <v>1</v>
+      </c>
+      <c r="I23" t="inlineStr">
+        <is>
+          <t>Feb27</t>
+        </is>
       </c>
     </row>
     <row r="24">
       <c r="A24" t="inlineStr">
         <is>
-          <t>ENSG00000182473</t>
+          <t>ENSG00000144369</t>
         </is>
       </c>
       <c r="B24" t="inlineStr">
         <is>
-          <t>EXOC7</t>
+          <t>FAM171B</t>
         </is>
       </c>
       <c r="C24" t="b">
@@ -1212,27 +1327,32 @@
       </c>
       <c r="F24" t="inlineStr">
         <is>
-          <t>OPC.5</t>
+          <t>Astro.1</t>
         </is>
       </c>
       <c r="G24" t="inlineStr">
         <is>
-          <t>OPC.5 specific Enrich genes t= 7.33</t>
+          <t>Astro.1 specific Enrich genes t= 8.3</t>
         </is>
       </c>
       <c r="H24" t="b">
         <v>1</v>
+      </c>
+      <c r="I24" t="inlineStr">
+        <is>
+          <t>Feb27</t>
+        </is>
       </c>
     </row>
     <row r="25">
       <c r="A25" t="inlineStr">
         <is>
-          <t>ENSG00000144369</t>
+          <t>ENSG00000182263</t>
         </is>
       </c>
       <c r="B25" t="inlineStr">
         <is>
-          <t>FAM171B</t>
+          <t>FIGN</t>
         </is>
       </c>
       <c r="C25" t="b">
@@ -1248,27 +1368,32 @@
       </c>
       <c r="F25" t="inlineStr">
         <is>
-          <t>Astro.1</t>
+          <t>Oligo.1</t>
         </is>
       </c>
       <c r="G25" t="inlineStr">
         <is>
-          <t>Astro.1 specific Enrich genes t= 8.3</t>
+          <t>Oligo.1 specific MR genes - Oligo.1/Oligo.4: 1.143</t>
         </is>
       </c>
       <c r="H25" t="b">
         <v>1</v>
+      </c>
+      <c r="I25" t="inlineStr">
+        <is>
+          <t>Feb27</t>
+        </is>
       </c>
     </row>
     <row r="26">
       <c r="A26" t="inlineStr">
         <is>
-          <t>ENSG00000182263</t>
+          <t>ENSG00000170345</t>
         </is>
       </c>
       <c r="B26" t="inlineStr">
         <is>
-          <t>FIGN</t>
+          <t>FOS</t>
         </is>
       </c>
       <c r="C26" t="b">
@@ -1279,32 +1404,37 @@
       </c>
       <c r="E26" t="inlineStr">
         <is>
-          <t>Marker - cell type specific</t>
+          <t>DEG - carrier</t>
         </is>
       </c>
       <c r="F26" t="inlineStr">
         <is>
-          <t>Oligo.1</t>
+          <t>Oligo.3</t>
         </is>
       </c>
       <c r="G26" t="inlineStr">
         <is>
-          <t>Oligo.1 specific MR genes - Oligo.1/Oligo.4: 1.143</t>
+          <t>DEG carrier top: Oligo.3 up logFC=2.77, DEG of interest: Oligo.3 up logFC=2.77</t>
         </is>
       </c>
       <c r="H26" t="b">
         <v>1</v>
+      </c>
+      <c r="I26" t="inlineStr">
+        <is>
+          <t>Feb27</t>
+        </is>
       </c>
     </row>
     <row r="27">
       <c r="A27" t="inlineStr">
         <is>
-          <t>ENSG00000170345</t>
+          <t>ENSG00000177283</t>
         </is>
       </c>
       <c r="B27" t="inlineStr">
         <is>
-          <t>FOS</t>
+          <t>FZD8</t>
         </is>
       </c>
       <c r="C27" t="b">
@@ -1315,32 +1445,37 @@
       </c>
       <c r="E27" t="inlineStr">
         <is>
-          <t>DEG - carrier</t>
+          <t>DEG - mediation</t>
         </is>
       </c>
       <c r="F27" t="inlineStr">
         <is>
-          <t>Oligo.3</t>
+          <t>Astro.2</t>
         </is>
       </c>
       <c r="G27" t="inlineStr">
         <is>
-          <t>DEG carrier top: Oligo.3 up, DEG of interest: Oligo.3 up</t>
+          <t>mediation gene: mediator Astro.2</t>
         </is>
       </c>
       <c r="H27" t="b">
         <v>1</v>
+      </c>
+      <c r="I27" t="inlineStr">
+        <is>
+          <t>Feb27</t>
+        </is>
       </c>
     </row>
     <row r="28">
       <c r="A28" t="inlineStr">
         <is>
-          <t>ENSG00000177283</t>
+          <t>ENSG00000147533</t>
         </is>
       </c>
       <c r="B28" t="inlineStr">
         <is>
-          <t>FZD8</t>
+          <t>GOLGA7</t>
         </is>
       </c>
       <c r="C28" t="b">
@@ -1351,32 +1486,37 @@
       </c>
       <c r="E28" t="inlineStr">
         <is>
-          <t>DEG - mediation</t>
+          <t>Marker - cell type specific</t>
         </is>
       </c>
       <c r="F28" t="inlineStr">
         <is>
-          <t>Astro.2</t>
+          <t>Oligo.1</t>
         </is>
       </c>
       <c r="G28" t="inlineStr">
         <is>
-          <t>mediation gene: mediator Astro.2</t>
+          <t>Oligo.1 specific Enrich genes t= 5.54</t>
         </is>
       </c>
       <c r="H28" t="b">
         <v>1</v>
+      </c>
+      <c r="I28" t="inlineStr">
+        <is>
+          <t>Feb27</t>
+        </is>
       </c>
     </row>
     <row r="29">
       <c r="A29" t="inlineStr">
         <is>
-          <t>ENSG00000147533</t>
+          <t>ENSG00000175265</t>
         </is>
       </c>
       <c r="B29" t="inlineStr">
         <is>
-          <t>GOLGA7</t>
+          <t>GOLGA8A</t>
         </is>
       </c>
       <c r="C29" t="b">
@@ -1387,21 +1527,26 @@
       </c>
       <c r="E29" t="inlineStr">
         <is>
-          <t>Marker - cell type specific</t>
+          <t>DEG - carrier</t>
         </is>
       </c>
       <c r="F29" t="inlineStr">
         <is>
-          <t>Oligo.1</t>
+          <t>Excit.L5.2</t>
         </is>
       </c>
       <c r="G29" t="inlineStr">
         <is>
-          <t>Oligo.1 specific Enrich genes t= 5.54</t>
+          <t>DEG carrier top:  Excit.L5.2 up</t>
         </is>
       </c>
       <c r="H29" t="b">
         <v>1</v>
+      </c>
+      <c r="I29" t="inlineStr">
+        <is>
+          <t>Mar2</t>
+        </is>
       </c>
     </row>
     <row r="30">
@@ -1439,6 +1584,11 @@
       <c r="H30" t="b">
         <v>1</v>
       </c>
+      <c r="I30" t="inlineStr">
+        <is>
+          <t>Feb27</t>
+        </is>
+      </c>
     </row>
     <row r="31">
       <c r="A31" t="inlineStr">
@@ -1475,6 +1625,11 @@
       <c r="H31" t="b">
         <v>1</v>
       </c>
+      <c r="I31" t="inlineStr">
+        <is>
+          <t>Feb27</t>
+        </is>
+      </c>
     </row>
     <row r="32">
       <c r="A32" t="inlineStr">
@@ -1511,16 +1666,21 @@
       <c r="H32" t="b">
         <v>1</v>
       </c>
+      <c r="I32" t="inlineStr">
+        <is>
+          <t>Feb27</t>
+        </is>
+      </c>
     </row>
     <row r="33">
       <c r="A33" t="inlineStr">
         <is>
-          <t>ENSG00000174948</t>
+          <t>ENSG00000244734</t>
         </is>
       </c>
       <c r="B33" t="inlineStr">
         <is>
-          <t>GPR149</t>
+          <t>HBB</t>
         </is>
       </c>
       <c r="C33" t="b">
@@ -1531,32 +1691,37 @@
       </c>
       <c r="E33" t="inlineStr">
         <is>
-          <t>DEG - carrier</t>
+          <t>DEG - ancestry</t>
         </is>
       </c>
       <c r="F33" t="inlineStr">
         <is>
-          <t>Excit.L2_5.1</t>
+          <t>Oligo.3</t>
         </is>
       </c>
       <c r="G33" t="inlineStr">
         <is>
-          <t>DEG carrier top:  Excit.L2_5.1 down</t>
+          <t>DEG carrier top: Oligo.3 AA_down</t>
         </is>
       </c>
       <c r="H33" t="b">
         <v>1</v>
+      </c>
+      <c r="I33" t="inlineStr">
+        <is>
+          <t>Feb27</t>
+        </is>
       </c>
     </row>
     <row r="34">
       <c r="A34" t="inlineStr">
         <is>
-          <t>ENSG00000244734</t>
+          <t>ENSG00000148357</t>
         </is>
       </c>
       <c r="B34" t="inlineStr">
         <is>
-          <t>HBB</t>
+          <t>HMCN2</t>
         </is>
       </c>
       <c r="C34" t="b">
@@ -1567,32 +1732,37 @@
       </c>
       <c r="E34" t="inlineStr">
         <is>
-          <t>DEG - ancestry</t>
+          <t>Marker - cell type specific</t>
         </is>
       </c>
       <c r="F34" t="inlineStr">
         <is>
-          <t>Oligo.3</t>
+          <t>Excit.L5.2</t>
         </is>
       </c>
       <c r="G34" t="inlineStr">
         <is>
-          <t>DEG carrier top: Oligo.3 AA_down</t>
+          <t>Excit.L5.2 specific MR genes - Excit.L5.2/Excit.L6b: 13.871</t>
         </is>
       </c>
       <c r="H34" t="b">
         <v>1</v>
+      </c>
+      <c r="I34" t="inlineStr">
+        <is>
+          <t>Feb27</t>
+        </is>
       </c>
     </row>
     <row r="35">
       <c r="A35" t="inlineStr">
         <is>
-          <t>ENSG00000148357</t>
+          <t>ENSG00000233429</t>
         </is>
       </c>
       <c r="B35" t="inlineStr">
         <is>
-          <t>HMCN2</t>
+          <t>HOTAIRM1</t>
         </is>
       </c>
       <c r="C35" t="b">
@@ -1613,22 +1783,27 @@
       </c>
       <c r="G35" t="inlineStr">
         <is>
-          <t>Excit.L5.2 specific MR genes - Excit.L5.2/Excit.L6b: 13.871</t>
+          <t>Excit.L5.2 specific Enrich genes t= 16.54</t>
         </is>
       </c>
       <c r="H35" t="b">
         <v>1</v>
+      </c>
+      <c r="I35" t="inlineStr">
+        <is>
+          <t>Feb27</t>
+        </is>
       </c>
     </row>
     <row r="36">
       <c r="A36" t="inlineStr">
         <is>
-          <t>ENSG00000233429</t>
+          <t>ENSG00000185811</t>
         </is>
       </c>
       <c r="B36" t="inlineStr">
         <is>
-          <t>HOTAIRM1</t>
+          <t>IKZF1</t>
         </is>
       </c>
       <c r="C36" t="b">
@@ -1639,32 +1814,37 @@
       </c>
       <c r="E36" t="inlineStr">
         <is>
-          <t>Marker - cell type specific</t>
+          <t>DEG - carrier</t>
         </is>
       </c>
       <c r="F36" t="inlineStr">
         <is>
-          <t>Excit.L5.2</t>
+          <t>Oligo.3</t>
         </is>
       </c>
       <c r="G36" t="inlineStr">
         <is>
-          <t>Excit.L5.2 specific Enrich genes t= 16.54</t>
+          <t>DEG carrier top: Oligo.3 up logFC=2.75</t>
         </is>
       </c>
       <c r="H36" t="b">
         <v>1</v>
+      </c>
+      <c r="I36" t="inlineStr">
+        <is>
+          <t>Feb27</t>
+        </is>
       </c>
     </row>
     <row r="37">
       <c r="A37" t="inlineStr">
         <is>
-          <t>ENSG00000185811</t>
+          <t>ENSG00000134352</t>
         </is>
       </c>
       <c r="B37" t="inlineStr">
         <is>
-          <t>IKZF1</t>
+          <t>IL6ST</t>
         </is>
       </c>
       <c r="C37" t="b">
@@ -1675,32 +1855,37 @@
       </c>
       <c r="E37" t="inlineStr">
         <is>
-          <t>DEG - carrier</t>
+          <t>DEG - mediation</t>
         </is>
       </c>
       <c r="F37" t="inlineStr">
         <is>
-          <t>Oligo.3</t>
+          <t>Astro.3</t>
         </is>
       </c>
       <c r="G37" t="inlineStr">
         <is>
-          <t>DEG carrier top: Oligo.3 up</t>
+          <t>mediation gene: mediator Astro.3</t>
         </is>
       </c>
       <c r="H37" t="b">
         <v>1</v>
+      </c>
+      <c r="I37" t="inlineStr">
+        <is>
+          <t>Feb27</t>
+        </is>
       </c>
     </row>
     <row r="38">
       <c r="A38" t="inlineStr">
         <is>
-          <t>ENSG00000134352</t>
+          <t>ENSG00000138448</t>
         </is>
       </c>
       <c r="B38" t="inlineStr">
         <is>
-          <t>IL6ST</t>
+          <t>ITGAV</t>
         </is>
       </c>
       <c r="C38" t="b">
@@ -1711,32 +1896,37 @@
       </c>
       <c r="E38" t="inlineStr">
         <is>
-          <t>DEG - mediation</t>
+          <t>Marker - cell type specific</t>
         </is>
       </c>
       <c r="F38" t="inlineStr">
         <is>
-          <t>Astro.3</t>
+          <t>Oligo.2</t>
         </is>
       </c>
       <c r="G38" t="inlineStr">
         <is>
-          <t>mediation gene: mediator Astro.3</t>
+          <t>Oligo.2 specific MR genes - Oligo.2/Oligo.1: 1.663</t>
         </is>
       </c>
       <c r="H38" t="b">
         <v>1</v>
+      </c>
+      <c r="I38" t="inlineStr">
+        <is>
+          <t>Feb27</t>
+        </is>
       </c>
     </row>
     <row r="39">
       <c r="A39" t="inlineStr">
         <is>
-          <t>ENSG00000138448</t>
+          <t>ENSG00000108773</t>
         </is>
       </c>
       <c r="B39" t="inlineStr">
         <is>
-          <t>ITGAV</t>
+          <t>KAT2A</t>
         </is>
       </c>
       <c r="C39" t="b">
@@ -1747,32 +1937,37 @@
       </c>
       <c r="E39" t="inlineStr">
         <is>
-          <t>Marker - cell type specific</t>
+          <t>DEG - ancestry</t>
         </is>
       </c>
       <c r="F39" t="inlineStr">
         <is>
-          <t>Oligo.2</t>
+          <t>Oligo.3</t>
         </is>
       </c>
       <c r="G39" t="inlineStr">
         <is>
-          <t>Oligo.2 specific MR genes - Oligo.2/Oligo.1: 1.663</t>
+          <t>DEG Ancestry op: Oligo.3 AA_up*-EA_down</t>
         </is>
       </c>
       <c r="H39" t="b">
         <v>1</v>
+      </c>
+      <c r="I39" t="inlineStr">
+        <is>
+          <t>Feb27</t>
+        </is>
       </c>
     </row>
     <row r="40">
       <c r="A40" t="inlineStr">
         <is>
-          <t>ENSG00000108773</t>
+          <t>ENSG00000184408</t>
         </is>
       </c>
       <c r="B40" t="inlineStr">
         <is>
-          <t>KAT2A</t>
+          <t>KCND2</t>
         </is>
       </c>
       <c r="C40" t="b">
@@ -1783,7 +1978,7 @@
       </c>
       <c r="E40" t="inlineStr">
         <is>
-          <t>DEG - ancestry</t>
+          <t>Marker - cell type specific</t>
         </is>
       </c>
       <c r="F40" t="inlineStr">
@@ -1793,22 +1988,27 @@
       </c>
       <c r="G40" t="inlineStr">
         <is>
-          <t>DEG Ancestry op: Oligo.3 AA_up*-EA_down</t>
+          <t>Oligo.3 specific Enrich genes t= 9.2</t>
         </is>
       </c>
       <c r="H40" t="b">
         <v>1</v>
+      </c>
+      <c r="I40" t="inlineStr">
+        <is>
+          <t>Feb27</t>
+        </is>
       </c>
     </row>
     <row r="41">
       <c r="A41" t="inlineStr">
         <is>
-          <t>ENSG00000184408</t>
+          <t>ENSG00000162989</t>
         </is>
       </c>
       <c r="B41" t="inlineStr">
         <is>
-          <t>KCND2</t>
+          <t>KCNJ3</t>
         </is>
       </c>
       <c r="C41" t="b">
@@ -1829,22 +2029,27 @@
       </c>
       <c r="G41" t="inlineStr">
         <is>
-          <t>Oligo.3 specific Enrich genes t= 9.2</t>
+          <t>Oligo.3 specific Enrich genes t= 9.5</t>
         </is>
       </c>
       <c r="H41" t="b">
         <v>1</v>
+      </c>
+      <c r="I41" t="inlineStr">
+        <is>
+          <t>Feb27</t>
+        </is>
       </c>
     </row>
     <row r="42">
       <c r="A42" t="inlineStr">
         <is>
-          <t>ENSG00000162989</t>
+          <t>ENSG00000234665</t>
         </is>
       </c>
       <c r="B42" t="inlineStr">
         <is>
-          <t>KCNJ3</t>
+          <t>LERFS</t>
         </is>
       </c>
       <c r="C42" t="b">
@@ -1855,7 +2060,7 @@
       </c>
       <c r="E42" t="inlineStr">
         <is>
-          <t>Marker - cell type specific</t>
+          <t>DEG - carrier</t>
         </is>
       </c>
       <c r="F42" t="inlineStr">
@@ -1865,22 +2070,27 @@
       </c>
       <c r="G42" t="inlineStr">
         <is>
-          <t>Oligo.3 specific Enrich genes t= 9.5</t>
+          <t>DEG carrier top: Oligo.3 down logFC=-1.39</t>
         </is>
       </c>
       <c r="H42" t="b">
         <v>1</v>
+      </c>
+      <c r="I42" t="inlineStr">
+        <is>
+          <t>Feb27</t>
+        </is>
       </c>
     </row>
     <row r="43">
       <c r="A43" t="inlineStr">
         <is>
-          <t>ENSG00000234665</t>
+          <t>ENSG00000233237</t>
         </is>
       </c>
       <c r="B43" t="inlineStr">
         <is>
-          <t>LERFS</t>
+          <t>LINC00472</t>
         </is>
       </c>
       <c r="C43" t="b">
@@ -1891,7 +2101,7 @@
       </c>
       <c r="E43" t="inlineStr">
         <is>
-          <t>DEG - carrier</t>
+          <t>DEG - ancestry</t>
         </is>
       </c>
       <c r="F43" t="inlineStr">
@@ -1901,22 +2111,27 @@
       </c>
       <c r="G43" t="inlineStr">
         <is>
-          <t>DEG carrier top: Oligo.3 down</t>
+          <t>DEG Ancestry op: Oligo.3 AA_down-EA_up*</t>
         </is>
       </c>
       <c r="H43" t="b">
         <v>1</v>
+      </c>
+      <c r="I43" t="inlineStr">
+        <is>
+          <t>Feb27</t>
+        </is>
       </c>
     </row>
     <row r="44">
       <c r="A44" t="inlineStr">
         <is>
-          <t>ENSG00000231023</t>
+          <t>ENSG00000230876</t>
         </is>
       </c>
       <c r="B44" t="inlineStr">
         <is>
-          <t>LINC00326</t>
+          <t>LINC00486</t>
         </is>
       </c>
       <c r="C44" t="b">
@@ -1932,27 +2147,32 @@
       </c>
       <c r="F44" t="inlineStr">
         <is>
-          <t>Excit.L2_5.1</t>
+          <t>Excit.L5.2</t>
         </is>
       </c>
       <c r="G44" t="inlineStr">
         <is>
-          <t>DEG carrier top:  Excit.L2_5.1 up</t>
+          <t>DEG carrier top:  Excit.L5.2 up</t>
         </is>
       </c>
       <c r="H44" t="b">
         <v>1</v>
+      </c>
+      <c r="I44" t="inlineStr">
+        <is>
+          <t>Mar2</t>
+        </is>
       </c>
     </row>
     <row r="45">
       <c r="A45" t="inlineStr">
         <is>
-          <t>ENSG00000233237</t>
+          <t>ENSG00000257585</t>
         </is>
       </c>
       <c r="B45" t="inlineStr">
         <is>
-          <t>LINC00472</t>
+          <t>LINC00609</t>
         </is>
       </c>
       <c r="C45" t="b">
@@ -1963,32 +2183,37 @@
       </c>
       <c r="E45" t="inlineStr">
         <is>
-          <t>DEG - ancestry</t>
+          <t>Marker - cell type specific</t>
         </is>
       </c>
       <c r="F45" t="inlineStr">
         <is>
-          <t>Oligo.3</t>
+          <t>Oligo.2</t>
         </is>
       </c>
       <c r="G45" t="inlineStr">
         <is>
-          <t>DEG Ancestry op: Oligo.3 AA_down-EA_up*</t>
+          <t>Oligo.2 specific Enrich genes t= 10.42</t>
         </is>
       </c>
       <c r="H45" t="b">
         <v>1</v>
+      </c>
+      <c r="I45" t="inlineStr">
+        <is>
+          <t>Feb27</t>
+        </is>
       </c>
     </row>
     <row r="46">
       <c r="A46" t="inlineStr">
         <is>
-          <t>ENSG00000257585</t>
+          <t>ENSG00000281186</t>
         </is>
       </c>
       <c r="B46" t="inlineStr">
         <is>
-          <t>LINC00609</t>
+          <t>LINC00706</t>
         </is>
       </c>
       <c r="C46" t="b">
@@ -1999,68 +2224,78 @@
       </c>
       <c r="E46" t="inlineStr">
         <is>
-          <t>Marker - cell type specific</t>
+          <t>DEG - ancestry</t>
         </is>
       </c>
       <c r="F46" t="inlineStr">
         <is>
-          <t>Oligo.2</t>
+          <t>Oligo.3</t>
         </is>
       </c>
       <c r="G46" t="inlineStr">
         <is>
-          <t>Oligo.2 specific Enrich genes t= 10.42</t>
+          <t>DEG carrier top: Oligo.3 AA_down</t>
         </is>
       </c>
       <c r="H46" t="b">
         <v>1</v>
+      </c>
+      <c r="I46" t="inlineStr">
+        <is>
+          <t>Feb27</t>
+        </is>
       </c>
     </row>
     <row r="47">
       <c r="A47" t="inlineStr">
         <is>
-          <t>ENSG00000281186</t>
+          <t>ENSG00000238217</t>
         </is>
       </c>
       <c r="B47" t="inlineStr">
         <is>
-          <t>LINC00706</t>
+          <t>LINC01877</t>
         </is>
       </c>
       <c r="C47" t="b">
         <v>0</v>
       </c>
       <c r="D47">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="E47" t="inlineStr">
         <is>
-          <t>DEG - ancestry</t>
+          <t>Marker - cell type global, Marker - cell type specific</t>
         </is>
       </c>
       <c r="F47" t="inlineStr">
         <is>
-          <t>Oligo.3</t>
+          <t>Oligo.2</t>
         </is>
       </c>
       <c r="G47" t="inlineStr">
         <is>
-          <t>DEG carrier top: Oligo.3 AA_down</t>
+          <t>globl MR genes -  Oligo.2/Oligo.1: 1.743, Oligo.2 specific MR genes - Oligo.2/Oligo.1: 1.743</t>
         </is>
       </c>
       <c r="H47" t="b">
         <v>1</v>
+      </c>
+      <c r="I47" t="inlineStr">
+        <is>
+          <t>Feb27</t>
+        </is>
       </c>
     </row>
     <row r="48">
       <c r="A48" t="inlineStr">
         <is>
-          <t>ENSG00000233973</t>
+          <t>ENSG00000254401</t>
         </is>
       </c>
       <c r="B48" t="inlineStr">
         <is>
-          <t>LINC01360</t>
+          <t>LINC02752</t>
         </is>
       </c>
       <c r="C48" t="b">
@@ -2071,7 +2306,7 @@
       </c>
       <c r="E48" t="inlineStr">
         <is>
-          <t>DEG - carrier</t>
+          <t>Marker - cell type global</t>
         </is>
       </c>
       <c r="F48" t="inlineStr">
@@ -2081,58 +2316,68 @@
       </c>
       <c r="G48" t="inlineStr">
         <is>
-          <t>DEG carrier top:  Excit.L5.2 up</t>
+          <t>globl MR genes -  Excit.L5.2/Excit.L2_5.2: 10.797</t>
         </is>
       </c>
       <c r="H48" t="b">
         <v>1</v>
+      </c>
+      <c r="I48" t="inlineStr">
+        <is>
+          <t>Feb27</t>
+        </is>
       </c>
     </row>
     <row r="49">
       <c r="A49" t="inlineStr">
         <is>
-          <t>ENSG00000238217</t>
+          <t>ENSG00000174482</t>
         </is>
       </c>
       <c r="B49" t="inlineStr">
         <is>
-          <t>LINC01877</t>
+          <t>LINGO2</t>
         </is>
       </c>
       <c r="C49" t="b">
         <v>0</v>
       </c>
       <c r="D49">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="E49" t="inlineStr">
         <is>
-          <t>Marker - cell type global, Marker - cell type specific</t>
+          <t>Marker - cell type specific</t>
         </is>
       </c>
       <c r="F49" t="inlineStr">
         <is>
-          <t>Oligo.2</t>
+          <t>Oligo.3</t>
         </is>
       </c>
       <c r="G49" t="inlineStr">
         <is>
-          <t>globl MR genes -  Oligo.2/Oligo.1: 1.743, Oligo.2 specific MR genes - Oligo.2/Oligo.1: 1.743</t>
+          <t>Oligo.3 specific Enrich genes t= 9.09</t>
         </is>
       </c>
       <c r="H49" t="b">
         <v>1</v>
+      </c>
+      <c r="I49" t="inlineStr">
+        <is>
+          <t>Feb27</t>
+        </is>
       </c>
     </row>
     <row r="50">
       <c r="A50" t="inlineStr">
         <is>
-          <t>ENSG00000254401</t>
+          <t>ENSG00000048540</t>
         </is>
       </c>
       <c r="B50" t="inlineStr">
         <is>
-          <t>LINC02752</t>
+          <t>LMO3</t>
         </is>
       </c>
       <c r="C50" t="b">
@@ -2143,32 +2388,37 @@
       </c>
       <c r="E50" t="inlineStr">
         <is>
-          <t>Marker - cell type global</t>
+          <t>Marker - cell type specific</t>
         </is>
       </c>
       <c r="F50" t="inlineStr">
         <is>
-          <t>Excit.L5.2</t>
+          <t>Astro.1</t>
         </is>
       </c>
       <c r="G50" t="inlineStr">
         <is>
-          <t>globl MR genes -  Excit.L5.2/Excit.L2_5.2: 10.797</t>
+          <t>Astro.1 specific Enrich genes t= 8.73</t>
         </is>
       </c>
       <c r="H50" t="b">
         <v>1</v>
+      </c>
+      <c r="I50" t="inlineStr">
+        <is>
+          <t>Feb27</t>
+        </is>
       </c>
     </row>
     <row r="51">
       <c r="A51" t="inlineStr">
         <is>
-          <t>ENSG00000174482</t>
+          <t>ENSG00000198121</t>
         </is>
       </c>
       <c r="B51" t="inlineStr">
         <is>
-          <t>LINGO2</t>
+          <t>LPAR1</t>
         </is>
       </c>
       <c r="C51" t="b">
@@ -2179,32 +2429,37 @@
       </c>
       <c r="E51" t="inlineStr">
         <is>
-          <t>Marker - cell type specific</t>
+          <t>DEG - carrier</t>
         </is>
       </c>
       <c r="F51" t="inlineStr">
         <is>
-          <t>Oligo.3</t>
+          <t>Excit.L2_5.1</t>
         </is>
       </c>
       <c r="G51" t="inlineStr">
         <is>
-          <t>Oligo.3 specific Enrich genes t= 9.09</t>
+          <t>DEG carrier top:  Excit.L2_5.1 down</t>
         </is>
       </c>
       <c r="H51" t="b">
         <v>1</v>
+      </c>
+      <c r="I51" t="inlineStr">
+        <is>
+          <t>Mar2</t>
+        </is>
       </c>
     </row>
     <row r="52">
       <c r="A52" t="inlineStr">
         <is>
-          <t>ENSG00000048540</t>
+          <t>ENSG00000235448</t>
         </is>
       </c>
       <c r="B52" t="inlineStr">
         <is>
-          <t>LMO3</t>
+          <t>LURAP1L-AS1</t>
         </is>
       </c>
       <c r="C52" t="b">
@@ -2215,32 +2470,37 @@
       </c>
       <c r="E52" t="inlineStr">
         <is>
-          <t>Marker - cell type specific</t>
+          <t>DEG - carrier</t>
         </is>
       </c>
       <c r="F52" t="inlineStr">
         <is>
-          <t>Astro.1</t>
+          <t>Oligo.3</t>
         </is>
       </c>
       <c r="G52" t="inlineStr">
         <is>
-          <t>Astro.1 specific Enrich genes t= 8.73</t>
+          <t>DEG carrier top: Oligo.3 down logFC=-1.48</t>
         </is>
       </c>
       <c r="H52" t="b">
         <v>1</v>
+      </c>
+      <c r="I52" t="inlineStr">
+        <is>
+          <t>Feb27</t>
+        </is>
       </c>
     </row>
     <row r="53">
       <c r="A53" t="inlineStr">
         <is>
-          <t>ENSG00000235448</t>
+          <t>ENSG00000102316</t>
         </is>
       </c>
       <c r="B53" t="inlineStr">
         <is>
-          <t>LURAP1L-AS1</t>
+          <t>MAGED2</t>
         </is>
       </c>
       <c r="C53" t="b">
@@ -2251,7 +2511,7 @@
       </c>
       <c r="E53" t="inlineStr">
         <is>
-          <t>DEG - carrier</t>
+          <t>DEG - ancestry</t>
         </is>
       </c>
       <c r="F53" t="inlineStr">
@@ -2261,22 +2521,27 @@
       </c>
       <c r="G53" t="inlineStr">
         <is>
-          <t>DEG carrier top: Oligo.3 down</t>
+          <t>DEG Ancestry op: Oligo.3 AA_up-EA_down*</t>
         </is>
       </c>
       <c r="H53" t="b">
         <v>1</v>
+      </c>
+      <c r="I53" t="inlineStr">
+        <is>
+          <t>Feb27</t>
+        </is>
       </c>
     </row>
     <row r="54">
       <c r="A54" t="inlineStr">
         <is>
-          <t>ENSG00000102316</t>
+          <t>ENSG00000186868</t>
         </is>
       </c>
       <c r="B54" t="inlineStr">
         <is>
-          <t>MAGED2</t>
+          <t>MAPT</t>
         </is>
       </c>
       <c r="C54" t="b">
@@ -2287,7 +2552,7 @@
       </c>
       <c r="E54" t="inlineStr">
         <is>
-          <t>DEG - ancestry</t>
+          <t>DEG - carrier</t>
         </is>
       </c>
       <c r="F54" t="inlineStr">
@@ -2297,94 +2562,109 @@
       </c>
       <c r="G54" t="inlineStr">
         <is>
-          <t>DEG Ancestry op: Oligo.3 AA_up-EA_down*</t>
+          <t>DEG of interest: Oligo.3 down logFC=-0.56</t>
         </is>
       </c>
       <c r="H54" t="b">
         <v>1</v>
+      </c>
+      <c r="I54" t="inlineStr">
+        <is>
+          <t>Feb27</t>
+        </is>
       </c>
     </row>
     <row r="55">
       <c r="A55" t="inlineStr">
         <is>
-          <t>ENSG00000186868</t>
+          <t>ENSG00000197971</t>
         </is>
       </c>
       <c r="B55" t="inlineStr">
         <is>
-          <t>MAPT</t>
+          <t>MBP</t>
         </is>
       </c>
       <c r="C55" t="b">
         <v>0</v>
       </c>
       <c r="D55">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="E55" t="inlineStr">
         <is>
-          <t>DEG - carrier</t>
+          <t>DEG - carrier, DEG - mediation, Marker - SpD</t>
         </is>
       </c>
       <c r="F55" t="inlineStr">
         <is>
-          <t>Oligo.3</t>
+          <t>Oligo.3, WM.uf~Sp09D07</t>
         </is>
       </c>
       <c r="G55" t="inlineStr">
         <is>
-          <t>DEG of interest: Oligo.3 down</t>
+          <t>SpD Enrich gene t=6.53, DEG of interest: Oligo.3 down logFC=-0.69, mediation gene: outcome Oligo.3</t>
         </is>
       </c>
       <c r="H55" t="b">
         <v>1</v>
+      </c>
+      <c r="I55" t="inlineStr">
+        <is>
+          <t>Feb27</t>
+        </is>
       </c>
     </row>
     <row r="56">
       <c r="A56" t="inlineStr">
         <is>
-          <t>ENSG00000197971</t>
+          <t>ENSG00000214548</t>
         </is>
       </c>
       <c r="B56" t="inlineStr">
         <is>
-          <t>MBP</t>
+          <t>MEG3</t>
         </is>
       </c>
       <c r="C56" t="b">
         <v>0</v>
       </c>
       <c r="D56">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="E56" t="inlineStr">
         <is>
-          <t>DEG - carrier, DEG - mediation, Marker - SpD</t>
+          <t>Marker - cell type specific</t>
         </is>
       </c>
       <c r="F56" t="inlineStr">
         <is>
-          <t>Oligo.3, WM.uf~Sp09D07</t>
+          <t>OPC.5</t>
         </is>
       </c>
       <c r="G56" t="inlineStr">
         <is>
-          <t>SpD Enrich gene t=6.53, DEG of interest: Oligo.3 down, mediation gene: outcome Oligo.3</t>
+          <t>OPC.5 specific MR genes - OPC.5/OPC.2: 1.019</t>
         </is>
       </c>
       <c r="H56" t="b">
         <v>1</v>
+      </c>
+      <c r="I56" t="inlineStr">
+        <is>
+          <t>Feb27</t>
+        </is>
       </c>
     </row>
     <row r="57">
       <c r="A57" t="inlineStr">
         <is>
-          <t>ENSG00000214548</t>
+          <t>ENSG00000225783</t>
         </is>
       </c>
       <c r="B57" t="inlineStr">
         <is>
-          <t>MEG3</t>
+          <t>MIAT</t>
         </is>
       </c>
       <c r="C57" t="b">
@@ -2395,32 +2675,37 @@
       </c>
       <c r="E57" t="inlineStr">
         <is>
-          <t>Marker - cell type specific</t>
+          <t>DEG - ancestry</t>
         </is>
       </c>
       <c r="F57" t="inlineStr">
         <is>
-          <t>OPC.5</t>
+          <t>Oligo.3</t>
         </is>
       </c>
       <c r="G57" t="inlineStr">
         <is>
-          <t>OPC.5 specific MR genes - OPC.5/OPC.2: 1.019</t>
+          <t>DEG carrier top: Oligo.3 AA_up</t>
         </is>
       </c>
       <c r="H57" t="b">
         <v>1</v>
+      </c>
+      <c r="I57" t="inlineStr">
+        <is>
+          <t>Feb27</t>
+        </is>
       </c>
     </row>
     <row r="58">
       <c r="A58" t="inlineStr">
         <is>
-          <t>ENSG00000225783</t>
+          <t>ENSG00000136297</t>
         </is>
       </c>
       <c r="B58" t="inlineStr">
         <is>
-          <t>MIAT</t>
+          <t>MMD2</t>
         </is>
       </c>
       <c r="C58" t="b">
@@ -2431,32 +2716,37 @@
       </c>
       <c r="E58" t="inlineStr">
         <is>
-          <t>DEG - ancestry</t>
+          <t>Marker - cell type specific</t>
         </is>
       </c>
       <c r="F58" t="inlineStr">
         <is>
-          <t>Oligo.3</t>
+          <t>Astro.2</t>
         </is>
       </c>
       <c r="G58" t="inlineStr">
         <is>
-          <t>DEG carrier top: Oligo.3 AA_up</t>
+          <t>Astro.2 specific MR genes - Astro.2/Astro.5: 1.004</t>
         </is>
       </c>
       <c r="H58" t="b">
         <v>1</v>
+      </c>
+      <c r="I58" t="inlineStr">
+        <is>
+          <t>Feb27</t>
+        </is>
       </c>
     </row>
     <row r="59">
       <c r="A59" t="inlineStr">
         <is>
-          <t>ENSG00000136297</t>
+          <t>ENSG00000198938</t>
         </is>
       </c>
       <c r="B59" t="inlineStr">
         <is>
-          <t>MMD2</t>
+          <t>MT-CO3</t>
         </is>
       </c>
       <c r="C59" t="b">
@@ -2472,27 +2762,32 @@
       </c>
       <c r="F59" t="inlineStr">
         <is>
-          <t>Astro.2</t>
+          <t>Oligo.3</t>
         </is>
       </c>
       <c r="G59" t="inlineStr">
         <is>
-          <t>Astro.2 specific MR genes - Astro.2/Astro.5: 1.004</t>
+          <t>Oligo.3 specific MR genes - Oligo.3/Oligo.4: 1.141</t>
         </is>
       </c>
       <c r="H59" t="b">
         <v>1</v>
+      </c>
+      <c r="I59" t="inlineStr">
+        <is>
+          <t>Feb27</t>
+        </is>
       </c>
     </row>
     <row r="60">
       <c r="A60" t="inlineStr">
         <is>
-          <t>ENSG00000198938</t>
+          <t>ENSG00000198727</t>
         </is>
       </c>
       <c r="B60" t="inlineStr">
         <is>
-          <t>MT-CO3</t>
+          <t>MT-CYB</t>
         </is>
       </c>
       <c r="C60" t="b">
@@ -2508,27 +2803,32 @@
       </c>
       <c r="F60" t="inlineStr">
         <is>
-          <t>Oligo.3</t>
+          <t>Excit.L2_5.1</t>
         </is>
       </c>
       <c r="G60" t="inlineStr">
         <is>
-          <t>Oligo.3 specific MR genes - Oligo.3/Oligo.4: 1.141</t>
+          <t>Excit.L2_5.1 specific MR genes - Excit.L2_5.1/Excit.L6b: 1.175</t>
         </is>
       </c>
       <c r="H60" t="b">
         <v>1</v>
+      </c>
+      <c r="I60" t="inlineStr">
+        <is>
+          <t>Feb27</t>
+        </is>
       </c>
     </row>
     <row r="61">
       <c r="A61" t="inlineStr">
         <is>
-          <t>ENSG00000198727</t>
+          <t>ENSG00000198888</t>
         </is>
       </c>
       <c r="B61" t="inlineStr">
         <is>
-          <t>MT-CYB</t>
+          <t>MT-ND1</t>
         </is>
       </c>
       <c r="C61" t="b">
@@ -2549,22 +2849,27 @@
       </c>
       <c r="G61" t="inlineStr">
         <is>
-          <t>Excit.L2_5.1 specific MR genes - Excit.L2_5.1/Excit.L6b: 1.175</t>
+          <t>Excit.L2_5.1 specific MR genes - Excit.L2_5.1/Excit.L6b: 1.201</t>
         </is>
       </c>
       <c r="H61" t="b">
         <v>1</v>
+      </c>
+      <c r="I61" t="inlineStr">
+        <is>
+          <t>Feb27</t>
+        </is>
       </c>
     </row>
     <row r="62">
       <c r="A62" t="inlineStr">
         <is>
-          <t>ENSG00000198888</t>
+          <t>ENSG00000198886</t>
         </is>
       </c>
       <c r="B62" t="inlineStr">
         <is>
-          <t>MT-ND1</t>
+          <t>MT-ND4</t>
         </is>
       </c>
       <c r="C62" t="b">
@@ -2575,21 +2880,26 @@
       </c>
       <c r="E62" t="inlineStr">
         <is>
-          <t>Marker - cell type specific</t>
+          <t>DEG - carrier</t>
         </is>
       </c>
       <c r="F62" t="inlineStr">
         <is>
-          <t>Excit.L2_5.1</t>
+          <t>Excit.L5.2</t>
         </is>
       </c>
       <c r="G62" t="inlineStr">
         <is>
-          <t>Excit.L2_5.1 specific MR genes - Excit.L2_5.1/Excit.L6b: 1.201</t>
+          <t>DEG carrier top:  Excit.L5.2 down</t>
         </is>
       </c>
       <c r="H62" t="b">
         <v>1</v>
+      </c>
+      <c r="I62" t="inlineStr">
+        <is>
+          <t>Mar2</t>
+        </is>
       </c>
     </row>
     <row r="63">
@@ -2627,6 +2937,11 @@
       <c r="H63" t="b">
         <v>1</v>
       </c>
+      <c r="I63" t="inlineStr">
+        <is>
+          <t>Feb27</t>
+        </is>
+      </c>
     </row>
     <row r="64">
       <c r="A64" t="inlineStr">
@@ -2663,6 +2978,11 @@
       <c r="H64" t="b">
         <v>1</v>
       </c>
+      <c r="I64" t="inlineStr">
+        <is>
+          <t>Feb27</t>
+        </is>
+      </c>
     </row>
     <row r="65">
       <c r="A65" t="inlineStr">
@@ -2699,16 +3019,21 @@
       <c r="H65" t="b">
         <v>1</v>
       </c>
+      <c r="I65" t="inlineStr">
+        <is>
+          <t>Feb27</t>
+        </is>
+      </c>
     </row>
     <row r="66">
       <c r="A66" t="inlineStr">
         <is>
-          <t>ENSG00000148826</t>
+          <t>ENSG00000169760</t>
         </is>
       </c>
       <c r="B66" t="inlineStr">
         <is>
-          <t>NKX6-2</t>
+          <t>NLGN1</t>
         </is>
       </c>
       <c r="C66" t="b">
@@ -2719,7 +3044,7 @@
       </c>
       <c r="E66" t="inlineStr">
         <is>
-          <t>MOFA - Factor3</t>
+          <t>DEGs - LR</t>
         </is>
       </c>
       <c r="F66" t="inlineStr">
@@ -2729,22 +3054,27 @@
       </c>
       <c r="G66" t="inlineStr">
         <is>
-          <t>MOFA Oligo.3 Factor3-</t>
+          <t>DEG LR interactions: NLGN1 -&gt; NRXN1,NLGN1 -&gt; NRXN3,NRXN1 -&gt; NLGN1,NRXN3 -&gt; NLGN1</t>
         </is>
       </c>
       <c r="H66" t="b">
         <v>1</v>
+      </c>
+      <c r="I66" t="inlineStr">
+        <is>
+          <t>Feb27</t>
+        </is>
       </c>
     </row>
     <row r="67">
       <c r="A67" t="inlineStr">
         <is>
-          <t>ENSG00000169760</t>
+          <t>ENSG00000221890</t>
         </is>
       </c>
       <c r="B67" t="inlineStr">
         <is>
-          <t>NLGN1</t>
+          <t>NPTXR</t>
         </is>
       </c>
       <c r="C67" t="b">
@@ -2755,32 +3085,37 @@
       </c>
       <c r="E67" t="inlineStr">
         <is>
-          <t>DEGs - LR</t>
+          <t>DEG - mediation</t>
         </is>
       </c>
       <c r="F67" t="inlineStr">
         <is>
-          <t>Oligo.3</t>
+          <t>Astro.1</t>
         </is>
       </c>
       <c r="G67" t="inlineStr">
         <is>
-          <t>DEG LR interactions: NLGN1 -&gt; NRXN1,NLGN1 -&gt; NRXN3,NRXN1 -&gt; NLGN1,NRXN3 -&gt; NLGN1</t>
+          <t>mediation gene: mediator Astro.1</t>
         </is>
       </c>
       <c r="H67" t="b">
         <v>1</v>
+      </c>
+      <c r="I67" t="inlineStr">
+        <is>
+          <t>Feb27</t>
+        </is>
       </c>
     </row>
     <row r="68">
       <c r="A68" t="inlineStr">
         <is>
-          <t>ENSG00000221890</t>
+          <t>ENSG00000185737</t>
         </is>
       </c>
       <c r="B68" t="inlineStr">
         <is>
-          <t>NPTXR</t>
+          <t>NRG3</t>
         </is>
       </c>
       <c r="C68" t="b">
@@ -2791,32 +3126,37 @@
       </c>
       <c r="E68" t="inlineStr">
         <is>
-          <t>DEG - mediation</t>
+          <t>DEGs - LR</t>
         </is>
       </c>
       <c r="F68" t="inlineStr">
         <is>
-          <t>Astro.1</t>
+          <t>Oligo.3</t>
         </is>
       </c>
       <c r="G68" t="inlineStr">
         <is>
-          <t>mediation gene: mediator Astro.1</t>
+          <t>DEG LR interactions: NRG3 -&gt; ERBB3</t>
         </is>
       </c>
       <c r="H68" t="b">
         <v>1</v>
+      </c>
+      <c r="I68" t="inlineStr">
+        <is>
+          <t>Feb27</t>
+        </is>
       </c>
     </row>
     <row r="69">
       <c r="A69" t="inlineStr">
         <is>
-          <t>ENSG00000185737</t>
+          <t>ENSG00000179915</t>
         </is>
       </c>
       <c r="B69" t="inlineStr">
         <is>
-          <t>NRG3</t>
+          <t>NRXN1</t>
         </is>
       </c>
       <c r="C69" t="b">
@@ -2837,22 +3177,27 @@
       </c>
       <c r="G69" t="inlineStr">
         <is>
-          <t>DEG LR interactions: NRG3 -&gt; ERBB3</t>
+          <t>DEG LR interactions: NLGN1 -&gt; NRXN1,NLGN4X -&gt; NRXN1,NRXN1 -&gt; NLGN1,NXPH1 -&gt; NRXN1</t>
         </is>
       </c>
       <c r="H69" t="b">
         <v>1</v>
+      </c>
+      <c r="I69" t="inlineStr">
+        <is>
+          <t>Feb27</t>
+        </is>
       </c>
     </row>
     <row r="70">
       <c r="A70" t="inlineStr">
         <is>
-          <t>ENSG00000179915</t>
+          <t>ENSG00000021645</t>
         </is>
       </c>
       <c r="B70" t="inlineStr">
         <is>
-          <t>NRXN1</t>
+          <t>NRXN3</t>
         </is>
       </c>
       <c r="C70" t="b">
@@ -2873,33 +3218,38 @@
       </c>
       <c r="G70" t="inlineStr">
         <is>
-          <t>DEG LR interactions: NLGN1 -&gt; NRXN1,NLGN4X -&gt; NRXN1,NRXN1 -&gt; NLGN1,NXPH1 -&gt; NRXN1</t>
+          <t>DEG LR interactions: NLGN1 -&gt; NRXN3,NRXN3 -&gt; NLGN1,NXPH1 -&gt; NRXN3</t>
         </is>
       </c>
       <c r="H70" t="b">
         <v>1</v>
+      </c>
+      <c r="I70" t="inlineStr">
+        <is>
+          <t>Feb27</t>
+        </is>
       </c>
     </row>
     <row r="71">
       <c r="A71" t="inlineStr">
         <is>
-          <t>ENSG00000021645</t>
+          <t>ENSG00000140538</t>
         </is>
       </c>
       <c r="B71" t="inlineStr">
         <is>
-          <t>NRXN3</t>
+          <t>NTRK3</t>
         </is>
       </c>
       <c r="C71" t="b">
         <v>0</v>
       </c>
       <c r="D71">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="E71" t="inlineStr">
         <is>
-          <t>DEGs - LR</t>
+          <t>DEGs - LR, Marker - cell type specific</t>
         </is>
       </c>
       <c r="F71" t="inlineStr">
@@ -2909,101 +3259,116 @@
       </c>
       <c r="G71" t="inlineStr">
         <is>
-          <t>DEG LR interactions: NLGN1 -&gt; NRXN3,NRXN3 -&gt; NLGN1,NXPH1 -&gt; NRXN3</t>
+          <t>Oligo.3 specific Enrich genes t= 9.07, DEG LR interactions: NTRK3 -&gt; PTPRD</t>
         </is>
       </c>
       <c r="H71" t="b">
         <v>1</v>
+      </c>
+      <c r="I71" t="inlineStr">
+        <is>
+          <t>Feb27</t>
+        </is>
       </c>
     </row>
     <row r="72">
       <c r="A72" t="inlineStr">
         <is>
-          <t>ENSG00000140538</t>
+          <t>ENSG00000228474</t>
         </is>
       </c>
       <c r="B72" t="inlineStr">
         <is>
-          <t>NTRK3</t>
+          <t>OST4</t>
         </is>
       </c>
       <c r="C72" t="b">
         <v>0</v>
       </c>
       <c r="D72">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="E72" t="inlineStr">
         <is>
-          <t>DEGs - LR, Marker - cell type specific</t>
+          <t>Marker - SpD</t>
         </is>
       </c>
       <c r="F72" t="inlineStr">
         <is>
-          <t>Oligo.3</t>
+          <t>LD~Sp09D02</t>
         </is>
       </c>
       <c r="G72" t="inlineStr">
         <is>
-          <t>Oligo.3 specific Enrich genes t= 9.07, DEG LR interactions: NTRK3 -&gt; PTPRD</t>
+          <t>SpD MeanRatio gene: LD~Sp09D02/L2.3~Sp09D01: 1.109</t>
         </is>
       </c>
       <c r="H72" t="b">
         <v>1</v>
+      </c>
+      <c r="I72" t="inlineStr">
+        <is>
+          <t>Feb27</t>
+        </is>
       </c>
     </row>
     <row r="73">
       <c r="A73" t="inlineStr">
         <is>
-          <t>ENSG00000228474</t>
+          <t>ENSG00000100836</t>
         </is>
       </c>
       <c r="B73" t="inlineStr">
         <is>
-          <t>OST4</t>
+          <t>PABPN1</t>
         </is>
       </c>
       <c r="C73" t="b">
         <v>0</v>
       </c>
       <c r="D73">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="E73" t="inlineStr">
         <is>
-          <t>Marker - SpD</t>
+          <t>Marker - cell type specific</t>
         </is>
       </c>
       <c r="F73" t="inlineStr">
         <is>
-          <t>LD~Sp09D02</t>
+          <t>Astro.3, Excit.L2_5.1</t>
         </is>
       </c>
       <c r="G73" t="inlineStr">
         <is>
-          <t>SpD MeanRatio gene: LD~Sp09D02/L2.3~Sp09D01: 1.109</t>
+          <t>Astro.3 specific MR genes - Astro.3/Astro.1: 1.046, Excit.L2_5.1 specific Enrich genes t= 9.16</t>
         </is>
       </c>
       <c r="H73" t="b">
         <v>1</v>
+      </c>
+      <c r="I73" t="inlineStr">
+        <is>
+          <t>Feb27</t>
+        </is>
       </c>
     </row>
     <row r="74">
       <c r="A74" t="inlineStr">
         <is>
-          <t>ENSG00000100836</t>
+          <t>ENSG00000228842</t>
         </is>
       </c>
       <c r="B74" t="inlineStr">
         <is>
-          <t>PABPN1</t>
+          <t>PCDH9-AS2</t>
         </is>
       </c>
       <c r="C74" t="b">
         <v>0</v>
       </c>
       <c r="D74">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="E74" t="inlineStr">
         <is>
@@ -3012,99 +3377,114 @@
       </c>
       <c r="F74" t="inlineStr">
         <is>
-          <t>Astro.3, Excit.L2_5.1</t>
+          <t>Astro.1</t>
         </is>
       </c>
       <c r="G74" t="inlineStr">
         <is>
-          <t>Astro.3 specific MR genes - Astro.3/Astro.1: 1.046, Excit.L2_5.1 specific Enrich genes t= 9.16</t>
+          <t>Astro.1 specific MR genes - Astro.1/Astro.3: 1.486</t>
         </is>
       </c>
       <c r="H74" t="b">
         <v>1</v>
+      </c>
+      <c r="I74" t="inlineStr">
+        <is>
+          <t>Feb27</t>
+        </is>
       </c>
     </row>
     <row r="75">
       <c r="A75" t="inlineStr">
         <is>
-          <t>ENSG00000228842</t>
+          <t>ENSG00000123560</t>
         </is>
       </c>
       <c r="B75" t="inlineStr">
         <is>
-          <t>PCDH9-AS2</t>
+          <t>PLP1</t>
         </is>
       </c>
       <c r="C75" t="b">
         <v>0</v>
       </c>
       <c r="D75">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="E75" t="inlineStr">
         <is>
-          <t>Marker - cell type specific</t>
+          <t>DEG - carrier, Marker - cell type specific</t>
         </is>
       </c>
       <c r="F75" t="inlineStr">
         <is>
-          <t>Astro.1</t>
+          <t>Excit.L2_5.1, Oligo.3</t>
         </is>
       </c>
       <c r="G75" t="inlineStr">
         <is>
-          <t>Astro.1 specific MR genes - Astro.1/Astro.3: 1.486</t>
+          <t>Excit.L2_5.1 specific Enrich genes t= 8.05, DEG of interest: Oligo.3 down logFC=-0.93</t>
         </is>
       </c>
       <c r="H75" t="b">
         <v>1</v>
+      </c>
+      <c r="I75" t="inlineStr">
+        <is>
+          <t>Feb27</t>
+        </is>
       </c>
     </row>
     <row r="76">
       <c r="A76" t="inlineStr">
         <is>
-          <t>ENSG00000123560</t>
+          <t>ENSG00000117600</t>
         </is>
       </c>
       <c r="B76" t="inlineStr">
         <is>
-          <t>PLP1</t>
+          <t>PLPPR4</t>
         </is>
       </c>
       <c r="C76" t="b">
         <v>0</v>
       </c>
       <c r="D76">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="E76" t="inlineStr">
         <is>
-          <t>DEG - carrier, Marker - cell type specific</t>
+          <t>DEG - mediation</t>
         </is>
       </c>
       <c r="F76" t="inlineStr">
         <is>
-          <t>Excit.L2_5.1, Oligo.3</t>
+          <t>Astro.1</t>
         </is>
       </c>
       <c r="G76" t="inlineStr">
         <is>
-          <t>Excit.L2_5.1 specific Enrich genes t= 8.05, DEG of interest: Oligo.3 down</t>
+          <t>mediation gene: mediator Astro.1</t>
         </is>
       </c>
       <c r="H76" t="b">
         <v>1</v>
+      </c>
+      <c r="I76" t="inlineStr">
+        <is>
+          <t>Feb27</t>
+        </is>
       </c>
     </row>
     <row r="77">
       <c r="A77" t="inlineStr">
         <is>
-          <t>ENSG00000117600</t>
+          <t>ENSG00000107317</t>
         </is>
       </c>
       <c r="B77" t="inlineStr">
         <is>
-          <t>PLPPR4</t>
+          <t>PTGDS</t>
         </is>
       </c>
       <c r="C77" t="b">
@@ -3115,32 +3495,37 @@
       </c>
       <c r="E77" t="inlineStr">
         <is>
-          <t>DEG - mediation</t>
+          <t>Marker - cell type specific</t>
         </is>
       </c>
       <c r="F77" t="inlineStr">
         <is>
-          <t>Astro.1</t>
+          <t>Astro.2</t>
         </is>
       </c>
       <c r="G77" t="inlineStr">
         <is>
-          <t>mediation gene: mediator Astro.1</t>
+          <t>Astro.2 specific MR genes - Astro.2/Astro.5: 1.01, Astro.2 specific Enrich genes t= 4.92</t>
         </is>
       </c>
       <c r="H77" t="b">
         <v>1</v>
+      </c>
+      <c r="I77" t="inlineStr">
+        <is>
+          <t>Feb27</t>
+        </is>
       </c>
     </row>
     <row r="78">
       <c r="A78" t="inlineStr">
         <is>
-          <t>ENSG00000184304</t>
+          <t>ENSG00000153707</t>
         </is>
       </c>
       <c r="B78" t="inlineStr">
         <is>
-          <t>PRKD1</t>
+          <t>PTPRD</t>
         </is>
       </c>
       <c r="C78" t="b">
@@ -3151,32 +3536,37 @@
       </c>
       <c r="E78" t="inlineStr">
         <is>
-          <t>DEG - carrier</t>
+          <t>DEGs - LR</t>
         </is>
       </c>
       <c r="F78" t="inlineStr">
         <is>
-          <t>Excit.L5.2</t>
+          <t>Oligo.3</t>
         </is>
       </c>
       <c r="G78" t="inlineStr">
         <is>
-          <t>DEG carrier top:  Excit.L5.2 down</t>
+          <t>DEG LR interactions: IL1RAPL1 -&gt; PTPRD,NTRK3 -&gt; PTPRD</t>
         </is>
       </c>
       <c r="H78" t="b">
         <v>1</v>
+      </c>
+      <c r="I78" t="inlineStr">
+        <is>
+          <t>Feb27</t>
+        </is>
       </c>
     </row>
     <row r="79">
       <c r="A79" t="inlineStr">
         <is>
-          <t>ENSG00000107317</t>
+          <t>ENSG00000079974</t>
         </is>
       </c>
       <c r="B79" t="inlineStr">
         <is>
-          <t>PTGDS</t>
+          <t>RABL2B</t>
         </is>
       </c>
       <c r="C79" t="b">
@@ -3187,32 +3577,37 @@
       </c>
       <c r="E79" t="inlineStr">
         <is>
-          <t>Marker - cell type specific</t>
+          <t>DEG - ancestry</t>
         </is>
       </c>
       <c r="F79" t="inlineStr">
         <is>
-          <t>Astro.2</t>
+          <t>Oligo.3</t>
         </is>
       </c>
       <c r="G79" t="inlineStr">
         <is>
-          <t>Astro.2 specific MR genes - Astro.2/Astro.5: 1.01, Astro.2 specific Enrich genes t= 4.92</t>
+          <t>DEG Ancestry op: Oligo.3 AA_up-EA_down*</t>
         </is>
       </c>
       <c r="H79" t="b">
         <v>1</v>
+      </c>
+      <c r="I79" t="inlineStr">
+        <is>
+          <t>Feb27</t>
+        </is>
       </c>
     </row>
     <row r="80">
       <c r="A80" t="inlineStr">
         <is>
-          <t>ENSG00000153707</t>
+          <t>ENSG00000129538</t>
         </is>
       </c>
       <c r="B80" t="inlineStr">
         <is>
-          <t>PTPRD</t>
+          <t>RNASE1</t>
         </is>
       </c>
       <c r="C80" t="b">
@@ -3223,7 +3618,7 @@
       </c>
       <c r="E80" t="inlineStr">
         <is>
-          <t>DEGs - LR</t>
+          <t>MOFA - Factor3</t>
         </is>
       </c>
       <c r="F80" t="inlineStr">
@@ -3233,22 +3628,27 @@
       </c>
       <c r="G80" t="inlineStr">
         <is>
-          <t>DEG LR interactions: IL1RAPL1 -&gt; PTPRD,NTRK3 -&gt; PTPRD</t>
+          <t>MOFA Oligo.3 Factor3-</t>
         </is>
       </c>
       <c r="H80" t="b">
         <v>1</v>
+      </c>
+      <c r="I80" t="inlineStr">
+        <is>
+          <t>Mar2</t>
+        </is>
       </c>
     </row>
     <row r="81">
       <c r="A81" t="inlineStr">
         <is>
-          <t>ENSG00000079974</t>
+          <t>ENSG00000177954</t>
         </is>
       </c>
       <c r="B81" t="inlineStr">
         <is>
-          <t>RABL2B</t>
+          <t>RPS27</t>
         </is>
       </c>
       <c r="C81" t="b">
@@ -3259,32 +3659,37 @@
       </c>
       <c r="E81" t="inlineStr">
         <is>
-          <t>DEG - ancestry</t>
+          <t>Marker - cell type specific</t>
         </is>
       </c>
       <c r="F81" t="inlineStr">
         <is>
-          <t>Oligo.3</t>
+          <t>Astro.3</t>
         </is>
       </c>
       <c r="G81" t="inlineStr">
         <is>
-          <t>DEG Ancestry op: Oligo.3 AA_up-EA_down*</t>
+          <t>Astro.3 specific MR genes - Astro.3/Astro.2: 1.109</t>
         </is>
       </c>
       <c r="H81" t="b">
         <v>1</v>
+      </c>
+      <c r="I81" t="inlineStr">
+        <is>
+          <t>Feb27</t>
+        </is>
       </c>
     </row>
     <row r="82">
       <c r="A82" t="inlineStr">
         <is>
-          <t>ENSG00000177954</t>
+          <t>ENSG00000250722</t>
         </is>
       </c>
       <c r="B82" t="inlineStr">
         <is>
-          <t>RPS27</t>
+          <t>SELENOP</t>
         </is>
       </c>
       <c r="C82" t="b">
@@ -3295,32 +3700,37 @@
       </c>
       <c r="E82" t="inlineStr">
         <is>
-          <t>Marker - cell type specific</t>
+          <t>MOFA - Factor3</t>
         </is>
       </c>
       <c r="F82" t="inlineStr">
         <is>
-          <t>Astro.3</t>
+          <t>Oligo.3</t>
         </is>
       </c>
       <c r="G82" t="inlineStr">
         <is>
-          <t>Astro.3 specific MR genes - Astro.3/Astro.2: 1.109</t>
+          <t>MOFA Oligo.3 Factor3-</t>
         </is>
       </c>
       <c r="H82" t="b">
         <v>1</v>
+      </c>
+      <c r="I82" t="inlineStr">
+        <is>
+          <t>Feb27</t>
+        </is>
       </c>
     </row>
     <row r="83">
       <c r="A83" t="inlineStr">
         <is>
-          <t>ENSG00000250722</t>
+          <t>ENSG00000137872</t>
         </is>
       </c>
       <c r="B83" t="inlineStr">
         <is>
-          <t>SELENOP</t>
+          <t>SEMA6D</t>
         </is>
       </c>
       <c r="C83" t="b">
@@ -3331,32 +3741,37 @@
       </c>
       <c r="E83" t="inlineStr">
         <is>
-          <t>MOFA - Factor3</t>
+          <t>Marker - cell type specific</t>
         </is>
       </c>
       <c r="F83" t="inlineStr">
         <is>
-          <t>Oligo.3</t>
+          <t>Oligo.1</t>
         </is>
       </c>
       <c r="G83" t="inlineStr">
         <is>
-          <t>MOFA Oligo.3 Factor3-</t>
+          <t>Oligo.1 specific MR genes - Oligo.1/Oligo.2: 1.179</t>
         </is>
       </c>
       <c r="H83" t="b">
         <v>1</v>
+      </c>
+      <c r="I83" t="inlineStr">
+        <is>
+          <t>Feb27</t>
+        </is>
       </c>
     </row>
     <row r="84">
       <c r="A84" t="inlineStr">
         <is>
-          <t>ENSG00000137872</t>
+          <t>ENSG00000100359</t>
         </is>
       </c>
       <c r="B84" t="inlineStr">
         <is>
-          <t>SEMA6D</t>
+          <t>SGSM3</t>
         </is>
       </c>
       <c r="C84" t="b">
@@ -3367,32 +3782,37 @@
       </c>
       <c r="E84" t="inlineStr">
         <is>
-          <t>Marker - cell type specific</t>
+          <t>DEG - ancestry</t>
         </is>
       </c>
       <c r="F84" t="inlineStr">
         <is>
-          <t>Oligo.1</t>
+          <t>Oligo.3</t>
         </is>
       </c>
       <c r="G84" t="inlineStr">
         <is>
-          <t>Oligo.1 specific MR genes - Oligo.1/Oligo.2: 1.179</t>
+          <t>DEG Ancestry op: Oligo.3 AA_up*-EA_down</t>
         </is>
       </c>
       <c r="H84" t="b">
         <v>1</v>
+      </c>
+      <c r="I84" t="inlineStr">
+        <is>
+          <t>Feb27</t>
+        </is>
       </c>
     </row>
     <row r="85">
       <c r="A85" t="inlineStr">
         <is>
-          <t>ENSG00000100359</t>
+          <t>ENSG00000155886</t>
         </is>
       </c>
       <c r="B85" t="inlineStr">
         <is>
-          <t>SGSM3</t>
+          <t>SLC24A2</t>
         </is>
       </c>
       <c r="C85" t="b">
@@ -3403,32 +3823,37 @@
       </c>
       <c r="E85" t="inlineStr">
         <is>
-          <t>DEG - ancestry</t>
+          <t>Marker - cell type specific</t>
         </is>
       </c>
       <c r="F85" t="inlineStr">
         <is>
-          <t>Oligo.3</t>
+          <t>Astro.3</t>
         </is>
       </c>
       <c r="G85" t="inlineStr">
         <is>
-          <t>DEG Ancestry op: Oligo.3 AA_up*-EA_down</t>
+          <t>Astro.3 specific Enrich genes t= 8.18</t>
         </is>
       </c>
       <c r="H85" t="b">
         <v>1</v>
+      </c>
+      <c r="I85" t="inlineStr">
+        <is>
+          <t>Feb27</t>
+        </is>
       </c>
     </row>
     <row r="86">
       <c r="A86" t="inlineStr">
         <is>
-          <t>ENSG00000155886</t>
+          <t>ENSG00000080493</t>
         </is>
       </c>
       <c r="B86" t="inlineStr">
         <is>
-          <t>SLC24A2</t>
+          <t>SLC4A4</t>
         </is>
       </c>
       <c r="C86" t="b">
@@ -3439,32 +3864,37 @@
       </c>
       <c r="E86" t="inlineStr">
         <is>
-          <t>Marker - cell type specific</t>
+          <t>MOFA - Factor3</t>
         </is>
       </c>
       <c r="F86" t="inlineStr">
         <is>
-          <t>Astro.3</t>
+          <t>Oligo.3</t>
         </is>
       </c>
       <c r="G86" t="inlineStr">
         <is>
-          <t>Astro.3 specific Enrich genes t= 8.18</t>
+          <t>MOFA Oligo.3 Factor3+</t>
         </is>
       </c>
       <c r="H86" t="b">
         <v>1</v>
+      </c>
+      <c r="I86" t="inlineStr">
+        <is>
+          <t>Feb27</t>
+        </is>
       </c>
     </row>
     <row r="87">
       <c r="A87" t="inlineStr">
         <is>
-          <t>ENSG00000080493</t>
+          <t>ENSG00000158865</t>
         </is>
       </c>
       <c r="B87" t="inlineStr">
         <is>
-          <t>SLC4A4</t>
+          <t>SLC5A11</t>
         </is>
       </c>
       <c r="C87" t="b">
@@ -3475,32 +3905,37 @@
       </c>
       <c r="E87" t="inlineStr">
         <is>
-          <t>MOFA - Factor3</t>
+          <t>Marker - cell type global</t>
         </is>
       </c>
       <c r="F87" t="inlineStr">
         <is>
-          <t>Oligo.3</t>
+          <t>Oligo.2</t>
         </is>
       </c>
       <c r="G87" t="inlineStr">
         <is>
-          <t>MOFA Oligo.3 Factor3+</t>
+          <t>globl MR genes -  Oligo.2/Oligo.5: 1.492</t>
         </is>
       </c>
       <c r="H87" t="b">
         <v>1</v>
+      </c>
+      <c r="I87" t="inlineStr">
+        <is>
+          <t>Mar2</t>
+        </is>
       </c>
     </row>
     <row r="88">
       <c r="A88" t="inlineStr">
         <is>
-          <t>ENSG00000151012</t>
+          <t>ENSG00000104852</t>
         </is>
       </c>
       <c r="B88" t="inlineStr">
         <is>
-          <t>SLC7A11</t>
+          <t>SNRNP70</t>
         </is>
       </c>
       <c r="C88" t="b">
@@ -3511,32 +3946,37 @@
       </c>
       <c r="E88" t="inlineStr">
         <is>
-          <t>DEG - carrier</t>
+          <t>Marker - cell type specific</t>
         </is>
       </c>
       <c r="F88" t="inlineStr">
         <is>
-          <t>Excit.L5.2</t>
+          <t>Astro.2</t>
         </is>
       </c>
       <c r="G88" t="inlineStr">
         <is>
-          <t>DEG carrier top:  Excit.L5.2 up</t>
+          <t>Astro.2 specific MR genes - Astro.2/Astro.3: 1.023</t>
         </is>
       </c>
       <c r="H88" t="b">
         <v>1</v>
+      </c>
+      <c r="I88" t="inlineStr">
+        <is>
+          <t>Feb27</t>
+        </is>
       </c>
     </row>
     <row r="89">
       <c r="A89" t="inlineStr">
         <is>
-          <t>ENSG00000104852</t>
+          <t>ENSG00000101400</t>
         </is>
       </c>
       <c r="B89" t="inlineStr">
         <is>
-          <t>SNRNP70</t>
+          <t>SNTA1</t>
         </is>
       </c>
       <c r="C89" t="b">
@@ -3557,22 +3997,27 @@
       </c>
       <c r="G89" t="inlineStr">
         <is>
-          <t>Astro.2 specific MR genes - Astro.2/Astro.3: 1.023</t>
+          <t>Astro.2 specific Enrich genes t= 4.98</t>
         </is>
       </c>
       <c r="H89" t="b">
         <v>1</v>
+      </c>
+      <c r="I89" t="inlineStr">
+        <is>
+          <t>Feb27</t>
+        </is>
       </c>
     </row>
     <row r="90">
       <c r="A90" t="inlineStr">
         <is>
-          <t>ENSG00000101400</t>
+          <t>ENSG00000120451</t>
         </is>
       </c>
       <c r="B90" t="inlineStr">
         <is>
-          <t>SNTA1</t>
+          <t>SNX19</t>
         </is>
       </c>
       <c r="C90" t="b">
@@ -3583,32 +4028,37 @@
       </c>
       <c r="E90" t="inlineStr">
         <is>
-          <t>Marker - cell type specific</t>
+          <t>DEG - ancestry</t>
         </is>
       </c>
       <c r="F90" t="inlineStr">
         <is>
-          <t>Astro.2</t>
+          <t>Oligo.3</t>
         </is>
       </c>
       <c r="G90" t="inlineStr">
         <is>
-          <t>Astro.2 specific Enrich genes t= 4.98</t>
+          <t>DEG Ancestry op: Oligo.3 AA_down*-EA_up</t>
         </is>
       </c>
       <c r="H90" t="b">
         <v>1</v>
+      </c>
+      <c r="I90" t="inlineStr">
+        <is>
+          <t>Feb27</t>
+        </is>
       </c>
     </row>
     <row r="91">
       <c r="A91" t="inlineStr">
         <is>
-          <t>ENSG00000120451</t>
+          <t>ENSG00000095637</t>
         </is>
       </c>
       <c r="B91" t="inlineStr">
         <is>
-          <t>SNX19</t>
+          <t>SORBS1</t>
         </is>
       </c>
       <c r="C91" t="b">
@@ -3619,7 +4069,7 @@
       </c>
       <c r="E91" t="inlineStr">
         <is>
-          <t>DEG - ancestry</t>
+          <t>DEG - mediation</t>
         </is>
       </c>
       <c r="F91" t="inlineStr">
@@ -3629,22 +4079,27 @@
       </c>
       <c r="G91" t="inlineStr">
         <is>
-          <t>DEG Ancestry op: Oligo.3 AA_down*-EA_up</t>
+          <t>mediation gene: outcome Oligo.3</t>
         </is>
       </c>
       <c r="H91" t="b">
         <v>1</v>
+      </c>
+      <c r="I91" t="inlineStr">
+        <is>
+          <t>Feb27</t>
+        </is>
       </c>
     </row>
     <row r="92">
       <c r="A92" t="inlineStr">
         <is>
-          <t>ENSG00000095637</t>
+          <t>ENSG00000115415</t>
         </is>
       </c>
       <c r="B92" t="inlineStr">
         <is>
-          <t>SORBS1</t>
+          <t>STAT1</t>
         </is>
       </c>
       <c r="C92" t="b">
@@ -3655,7 +4110,7 @@
       </c>
       <c r="E92" t="inlineStr">
         <is>
-          <t>DEG - mediation</t>
+          <t>DEG - carrier</t>
         </is>
       </c>
       <c r="F92" t="inlineStr">
@@ -3665,22 +4120,27 @@
       </c>
       <c r="G92" t="inlineStr">
         <is>
-          <t>mediation gene: outcome Oligo.3</t>
+          <t>DEG of interest: Oligo.3 up logFC=0.8</t>
         </is>
       </c>
       <c r="H92" t="b">
         <v>1</v>
+      </c>
+      <c r="I92" t="inlineStr">
+        <is>
+          <t>Feb27</t>
+        </is>
       </c>
     </row>
     <row r="93">
       <c r="A93" t="inlineStr">
         <is>
-          <t>ENSG00000110693</t>
+          <t>ENSG00000138378</t>
         </is>
       </c>
       <c r="B93" t="inlineStr">
         <is>
-          <t>SOX6</t>
+          <t>STAT4</t>
         </is>
       </c>
       <c r="C93" t="b">
@@ -3691,7 +4151,7 @@
       </c>
       <c r="E93" t="inlineStr">
         <is>
-          <t>DEG - mediation</t>
+          <t>DEG - carrier</t>
         </is>
       </c>
       <c r="F93" t="inlineStr">
@@ -3701,22 +4161,27 @@
       </c>
       <c r="G93" t="inlineStr">
         <is>
-          <t>mediation gene: outcome Oligo.3</t>
+          <t>DEG of interest: Oligo.3 up logFC=2.62</t>
         </is>
       </c>
       <c r="H93" t="b">
         <v>1</v>
+      </c>
+      <c r="I93" t="inlineStr">
+        <is>
+          <t>Feb27</t>
+        </is>
       </c>
     </row>
     <row r="94">
       <c r="A94" t="inlineStr">
         <is>
-          <t>ENSG00000115415</t>
+          <t>ENSG00000185518</t>
         </is>
       </c>
       <c r="B94" t="inlineStr">
         <is>
-          <t>STAT1</t>
+          <t>SV2B</t>
         </is>
       </c>
       <c r="C94" t="b">
@@ -3727,32 +4192,37 @@
       </c>
       <c r="E94" t="inlineStr">
         <is>
-          <t>DEG - carrier</t>
+          <t>DEG - mediation</t>
         </is>
       </c>
       <c r="F94" t="inlineStr">
         <is>
-          <t>Oligo.3</t>
+          <t>Astro.2</t>
         </is>
       </c>
       <c r="G94" t="inlineStr">
         <is>
-          <t>DEG of interest: Oligo.3 up</t>
+          <t>mediation gene: mediator Astro.2</t>
         </is>
       </c>
       <c r="H94" t="b">
         <v>1</v>
+      </c>
+      <c r="I94" t="inlineStr">
+        <is>
+          <t>Feb27</t>
+        </is>
       </c>
     </row>
     <row r="95">
       <c r="A95" t="inlineStr">
         <is>
-          <t>ENSG00000138378</t>
+          <t>ENSG00000136560</t>
         </is>
       </c>
       <c r="B95" t="inlineStr">
         <is>
-          <t>STAT4</t>
+          <t>TANK</t>
         </is>
       </c>
       <c r="C95" t="b">
@@ -3763,32 +4233,37 @@
       </c>
       <c r="E95" t="inlineStr">
         <is>
-          <t>DEG - carrier</t>
+          <t>Marker - cell type specific</t>
         </is>
       </c>
       <c r="F95" t="inlineStr">
         <is>
-          <t>Oligo.3</t>
+          <t>Excit.L5.2</t>
         </is>
       </c>
       <c r="G95" t="inlineStr">
         <is>
-          <t>DEG of interest: Oligo.3 up</t>
+          <t>Excit.L5.2 specific Enrich genes t= 13.71</t>
         </is>
       </c>
       <c r="H95" t="b">
         <v>1</v>
+      </c>
+      <c r="I95" t="inlineStr">
+        <is>
+          <t>Feb27</t>
+        </is>
       </c>
     </row>
     <row r="96">
       <c r="A96" t="inlineStr">
         <is>
-          <t>ENSG00000185518</t>
+          <t>ENSG00000137462</t>
         </is>
       </c>
       <c r="B96" t="inlineStr">
         <is>
-          <t>SV2B</t>
+          <t>TLR2</t>
         </is>
       </c>
       <c r="C96" t="b">
@@ -3799,32 +4274,37 @@
       </c>
       <c r="E96" t="inlineStr">
         <is>
-          <t>DEG - mediation</t>
+          <t>DEG - carrier</t>
         </is>
       </c>
       <c r="F96" t="inlineStr">
         <is>
-          <t>Astro.2</t>
+          <t>Oligo.3</t>
         </is>
       </c>
       <c r="G96" t="inlineStr">
         <is>
-          <t>mediation gene: mediator Astro.2</t>
+          <t>DEG of interest: Oligo.3 up logFC=1.56</t>
         </is>
       </c>
       <c r="H96" t="b">
         <v>1</v>
+      </c>
+      <c r="I96" t="inlineStr">
+        <is>
+          <t>Feb27</t>
+        </is>
       </c>
     </row>
     <row r="97">
       <c r="A97" t="inlineStr">
         <is>
-          <t>ENSG00000136560</t>
+          <t>ENSG00000061938</t>
         </is>
       </c>
       <c r="B97" t="inlineStr">
         <is>
-          <t>TANK</t>
+          <t>TNK2</t>
         </is>
       </c>
       <c r="C97" t="b">
@@ -3840,27 +4320,32 @@
       </c>
       <c r="F97" t="inlineStr">
         <is>
-          <t>Excit.L5.2</t>
+          <t>OPC.5</t>
         </is>
       </c>
       <c r="G97" t="inlineStr">
         <is>
-          <t>Excit.L5.2 specific Enrich genes t= 13.71</t>
+          <t>OPC.5 specific MR genes - OPC.5/OPC.2: 1.04</t>
         </is>
       </c>
       <c r="H97" t="b">
         <v>1</v>
+      </c>
+      <c r="I97" t="inlineStr">
+        <is>
+          <t>Feb27</t>
+        </is>
       </c>
     </row>
     <row r="98">
       <c r="A98" t="inlineStr">
         <is>
-          <t>ENSG00000137462</t>
+          <t>ENSG00000124900</t>
         </is>
       </c>
       <c r="B98" t="inlineStr">
         <is>
-          <t>TLR2</t>
+          <t>TRIM51</t>
         </is>
       </c>
       <c r="C98" t="b">
@@ -3871,32 +4356,37 @@
       </c>
       <c r="E98" t="inlineStr">
         <is>
-          <t>DEG - carrier</t>
+          <t>Marker - SpD</t>
         </is>
       </c>
       <c r="F98" t="inlineStr">
         <is>
-          <t>Oligo.3</t>
+          <t>WM.uf_Sp09D07-WM_Sp09D06</t>
         </is>
       </c>
       <c r="G98" t="inlineStr">
         <is>
-          <t>DEG of interest: Oligo.3 up</t>
+          <t>SpD pw gene t=7.53</t>
         </is>
       </c>
       <c r="H98" t="b">
         <v>1</v>
+      </c>
+      <c r="I98" t="inlineStr">
+        <is>
+          <t>Mar2</t>
+        </is>
       </c>
     </row>
     <row r="99">
       <c r="A99" t="inlineStr">
         <is>
-          <t>ENSG00000061938</t>
+          <t>ENSG00000173960</t>
         </is>
       </c>
       <c r="B99" t="inlineStr">
         <is>
-          <t>TNK2</t>
+          <t>UBXN2A</t>
         </is>
       </c>
       <c r="C99" t="b">
@@ -3907,32 +4397,37 @@
       </c>
       <c r="E99" t="inlineStr">
         <is>
-          <t>Marker - cell type specific</t>
+          <t>DEG - ancestry</t>
         </is>
       </c>
       <c r="F99" t="inlineStr">
         <is>
-          <t>OPC.5</t>
+          <t>Oligo.3</t>
         </is>
       </c>
       <c r="G99" t="inlineStr">
         <is>
-          <t>OPC.5 specific MR genes - OPC.5/OPC.2: 1.04</t>
+          <t>DEG Ancestry op: Oligo.3 AA_down*-EA_up</t>
         </is>
       </c>
       <c r="H99" t="b">
         <v>1</v>
+      </c>
+      <c r="I99" t="inlineStr">
+        <is>
+          <t>Feb27</t>
+        </is>
       </c>
     </row>
     <row r="100">
       <c r="A100" t="inlineStr">
         <is>
-          <t>ENSG00000173960</t>
+          <t>ENSG00000143952</t>
         </is>
       </c>
       <c r="B100" t="inlineStr">
         <is>
-          <t>UBXN2A</t>
+          <t>VPS54</t>
         </is>
       </c>
       <c r="C100" t="b">
@@ -3958,17 +4453,22 @@
       </c>
       <c r="H100" t="b">
         <v>1</v>
+      </c>
+      <c r="I100" t="inlineStr">
+        <is>
+          <t>Feb27</t>
+        </is>
       </c>
     </row>
     <row r="101">
       <c r="A101" t="inlineStr">
         <is>
-          <t>ENSG00000143952</t>
+          <t>ENSG00000188818</t>
         </is>
       </c>
       <c r="B101" t="inlineStr">
         <is>
-          <t>VPS54</t>
+          <t>ZDHHC11</t>
         </is>
       </c>
       <c r="C101" t="b">
@@ -3979,21 +4479,26 @@
       </c>
       <c r="E101" t="inlineStr">
         <is>
-          <t>DEG - ancestry</t>
+          <t>DEG - carrier</t>
         </is>
       </c>
       <c r="F101" t="inlineStr">
         <is>
-          <t>Oligo.3</t>
+          <t>Excit.L5.2</t>
         </is>
       </c>
       <c r="G101" t="inlineStr">
         <is>
-          <t>DEG Ancestry op: Oligo.3 AA_down*-EA_up</t>
+          <t>DEG carrier top:  Excit.L5.2 down</t>
         </is>
       </c>
       <c r="H101" t="b">
         <v>1</v>
+      </c>
+      <c r="I101" t="inlineStr">
+        <is>
+          <t>Mar2</t>
+        </is>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Update custom probes with new round of checks
</commit_message>
<xml_diff>
--- a/processed-data/21_Xenium/02_xenium_compile_custom/ERC_Xenium_select_custom_probes.xlsx
+++ b/processed-data/21_Xenium/02_xenium_compile_custom/ERC_Xenium_select_custom_probes.xlsx
@@ -580,11 +580,11 @@
         <v>0</v>
       </c>
       <c r="D6">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="E6" t="inlineStr">
         <is>
-          <t>Marker - cell type specific</t>
+          <t>Marker - cell type global, Marker - cell type specific</t>
         </is>
       </c>
       <c r="F6" t="inlineStr">
@@ -594,7 +594,7 @@
       </c>
       <c r="G6" t="inlineStr">
         <is>
-          <t>Oligo.5 specific MR genes - Oligo.5/Oligo.2: 2.851, Oligo.5 specific Enrich genes t= 12.26</t>
+          <t>globl MR genes -  Oligo.5/Excit.L2_5.2: 1.322, Oligo.5 specific MR genes - Oligo.5/Oligo.2: 2.851, Oligo.5 specific Enrich genes t= 12.26</t>
         </is>
       </c>
       <c r="H6" t="b">
@@ -855,12 +855,12 @@
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>ENSG00000133019</t>
+          <t>ENSG00000128656</t>
         </is>
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>CHRM3</t>
+          <t>CHN1</t>
         </is>
       </c>
       <c r="C13" t="b">
@@ -871,17 +871,17 @@
       </c>
       <c r="E13" t="inlineStr">
         <is>
-          <t>DEG - mediation</t>
+          <t>Marker - SpD</t>
         </is>
       </c>
       <c r="F13" t="inlineStr">
         <is>
-          <t>Astro.3</t>
+          <t>WM.uf_Sp09D07-WM_Sp09D06</t>
         </is>
       </c>
       <c r="G13" t="inlineStr">
         <is>
-          <t>mediation gene: mediator Astro.3</t>
+          <t>SpD pw gene t=8.2</t>
         </is>
       </c>
       <c r="H13" t="b">
@@ -889,19 +889,19 @@
       </c>
       <c r="I13" t="inlineStr">
         <is>
-          <t>Feb27</t>
+          <t>Mar6</t>
         </is>
       </c>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t>ENSG00000171310</t>
+          <t>ENSG00000133019</t>
         </is>
       </c>
       <c r="B14" t="inlineStr">
         <is>
-          <t>CHST11</t>
+          <t>CHRM3</t>
         </is>
       </c>
       <c r="C14" t="b">
@@ -912,17 +912,17 @@
       </c>
       <c r="E14" t="inlineStr">
         <is>
-          <t>DEG - carrier</t>
+          <t>DEG - mediation</t>
         </is>
       </c>
       <c r="F14" t="inlineStr">
         <is>
-          <t>Oligo.3</t>
+          <t>Astro.3</t>
         </is>
       </c>
       <c r="G14" t="inlineStr">
         <is>
-          <t>DEG carrier top: Oligo.3 up logFC=2.82</t>
+          <t>mediation gene: mediator Astro.3</t>
         </is>
       </c>
       <c r="H14" t="b">
@@ -937,12 +937,12 @@
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>ENSG00000174469</t>
+          <t>ENSG00000171310</t>
         </is>
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>CNTNAP2</t>
+          <t>CHST11</t>
         </is>
       </c>
       <c r="C15" t="b">
@@ -953,7 +953,7 @@
       </c>
       <c r="E15" t="inlineStr">
         <is>
-          <t>Marker - cell type specific</t>
+          <t>DEG - carrier</t>
         </is>
       </c>
       <c r="F15" t="inlineStr">
@@ -963,7 +963,7 @@
       </c>
       <c r="G15" t="inlineStr">
         <is>
-          <t>Oligo.3 specific MR genes - Oligo.3/Oligo.2: 1.055</t>
+          <t>DEG carrier top: Oligo.3 up logFC=2.82</t>
         </is>
       </c>
       <c r="H15" t="b">
@@ -978,12 +978,12 @@
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t>ENSG00000084636</t>
+          <t>ENSG00000174469</t>
         </is>
       </c>
       <c r="B16" t="inlineStr">
         <is>
-          <t>COL16A1</t>
+          <t>CNTNAP2</t>
         </is>
       </c>
       <c r="C16" t="b">
@@ -999,12 +999,12 @@
       </c>
       <c r="F16" t="inlineStr">
         <is>
-          <t>Astro.3</t>
+          <t>Oligo.3</t>
         </is>
       </c>
       <c r="G16" t="inlineStr">
         <is>
-          <t>Astro.3 specific MR genes - Astro.3/Astro.2: 1.061</t>
+          <t>Oligo.3 specific MR genes - Oligo.3/Oligo.2: 1.055</t>
         </is>
       </c>
       <c r="H16" t="b">
@@ -1019,12 +1019,12 @@
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t>ENSG00000124749</t>
+          <t>ENSG00000084636</t>
         </is>
       </c>
       <c r="B17" t="inlineStr">
         <is>
-          <t>COL21A1</t>
+          <t>COL16A1</t>
         </is>
       </c>
       <c r="C17" t="b">
@@ -1035,17 +1035,17 @@
       </c>
       <c r="E17" t="inlineStr">
         <is>
-          <t>DEG - carrier</t>
+          <t>Marker - cell type specific</t>
         </is>
       </c>
       <c r="F17" t="inlineStr">
         <is>
-          <t>Oligo.3</t>
+          <t>Astro.3</t>
         </is>
       </c>
       <c r="G17" t="inlineStr">
         <is>
-          <t>DEG carrier top: Oligo.3 up logFC=2.79</t>
+          <t>Astro.3 specific MR genes - Astro.3/Astro.2: 1.061</t>
         </is>
       </c>
       <c r="H17" t="b">
@@ -1060,12 +1060,12 @@
     <row r="18">
       <c r="A18" t="inlineStr">
         <is>
-          <t>ENSG00000172428</t>
+          <t>ENSG00000124749</t>
         </is>
       </c>
       <c r="B18" t="inlineStr">
         <is>
-          <t>COPS9</t>
+          <t>COL21A1</t>
         </is>
       </c>
       <c r="C18" t="b">
@@ -1076,17 +1076,17 @@
       </c>
       <c r="E18" t="inlineStr">
         <is>
-          <t>Marker - SpD</t>
+          <t>DEG - carrier</t>
         </is>
       </c>
       <c r="F18" t="inlineStr">
         <is>
-          <t>LD~Sp09D02</t>
+          <t>Oligo.3</t>
         </is>
       </c>
       <c r="G18" t="inlineStr">
         <is>
-          <t>SpD MeanRatio gene: LD~Sp09D02/Inhib~Sp09D09: 1.112</t>
+          <t>DEG carrier top: Oligo.3 up logFC=2.79</t>
         </is>
       </c>
       <c r="H18" t="b">
@@ -1101,12 +1101,12 @@
     <row r="19">
       <c r="A19" t="inlineStr">
         <is>
-          <t>ENSG00000196353</t>
+          <t>ENSG00000172428</t>
         </is>
       </c>
       <c r="B19" t="inlineStr">
         <is>
-          <t>CPNE4</t>
+          <t>COPS9</t>
         </is>
       </c>
       <c r="C19" t="b">
@@ -1117,17 +1117,17 @@
       </c>
       <c r="E19" t="inlineStr">
         <is>
-          <t>DEG - carrier</t>
+          <t>Marker - SpD</t>
         </is>
       </c>
       <c r="F19" t="inlineStr">
         <is>
-          <t>Oligo.3</t>
+          <t>LD~Sp09D02</t>
         </is>
       </c>
       <c r="G19" t="inlineStr">
         <is>
-          <t>DEG of interest: Oligo.3 up logFC=1.87</t>
+          <t>SpD MeanRatio gene: LD~Sp09D02/Inhib~Sp09D09: 1.112</t>
         </is>
       </c>
       <c r="H19" t="b">
@@ -1135,19 +1135,19 @@
       </c>
       <c r="I19" t="inlineStr">
         <is>
-          <t>Mar2</t>
+          <t>Feb27</t>
         </is>
       </c>
     </row>
     <row r="20">
       <c r="A20" t="inlineStr">
         <is>
-          <t>ENSG00000004975</t>
+          <t>ENSG00000196353</t>
         </is>
       </c>
       <c r="B20" t="inlineStr">
         <is>
-          <t>DVL2</t>
+          <t>CPNE4</t>
         </is>
       </c>
       <c r="C20" t="b">
@@ -1158,7 +1158,7 @@
       </c>
       <c r="E20" t="inlineStr">
         <is>
-          <t>DEG - ancestry</t>
+          <t>DEG - carrier</t>
         </is>
       </c>
       <c r="F20" t="inlineStr">
@@ -1168,7 +1168,7 @@
       </c>
       <c r="G20" t="inlineStr">
         <is>
-          <t>DEG Ancestry op: Oligo.3 AA_up-EA_down*</t>
+          <t>DEG of interest: Oligo.3 up logFC=1.87</t>
         </is>
       </c>
       <c r="H20" t="b">
@@ -1176,19 +1176,19 @@
       </c>
       <c r="I20" t="inlineStr">
         <is>
-          <t>Feb27</t>
+          <t>Mar2</t>
         </is>
       </c>
     </row>
     <row r="21">
       <c r="A21" t="inlineStr">
         <is>
-          <t>ENSG00000171617</t>
+          <t>ENSG00000004975</t>
         </is>
       </c>
       <c r="B21" t="inlineStr">
         <is>
-          <t>ENC1</t>
+          <t>DVL2</t>
         </is>
       </c>
       <c r="C21" t="b">
@@ -1199,7 +1199,7 @@
       </c>
       <c r="E21" t="inlineStr">
         <is>
-          <t>DEG - mediation</t>
+          <t>DEG - ancestry</t>
         </is>
       </c>
       <c r="F21" t="inlineStr">
@@ -1209,7 +1209,7 @@
       </c>
       <c r="G21" t="inlineStr">
         <is>
-          <t>mediation gene: outcome Oligo.3</t>
+          <t>DEG Ancestry op: Oligo.3 AA_up-EA_down*</t>
         </is>
       </c>
       <c r="H21" t="b">
@@ -1224,12 +1224,12 @@
     <row r="22">
       <c r="A22" t="inlineStr">
         <is>
-          <t>ENSG00000178568</t>
+          <t>ENSG00000171617</t>
         </is>
       </c>
       <c r="B22" t="inlineStr">
         <is>
-          <t>ERBB4</t>
+          <t>ENC1</t>
         </is>
       </c>
       <c r="C22" t="b">
@@ -1240,17 +1240,17 @@
       </c>
       <c r="E22" t="inlineStr">
         <is>
-          <t>Marker - cell type specific</t>
+          <t>DEG - mediation</t>
         </is>
       </c>
       <c r="F22" t="inlineStr">
         <is>
-          <t>Oligo.1</t>
+          <t>Oligo.3</t>
         </is>
       </c>
       <c r="G22" t="inlineStr">
         <is>
-          <t>Oligo.1 specific Enrich genes t= 5.58</t>
+          <t>mediation gene: outcome Oligo.3</t>
         </is>
       </c>
       <c r="H22" t="b">
@@ -1265,12 +1265,12 @@
     <row r="23">
       <c r="A23" t="inlineStr">
         <is>
-          <t>ENSG00000182473</t>
+          <t>ENSG00000178568</t>
         </is>
       </c>
       <c r="B23" t="inlineStr">
         <is>
-          <t>EXOC7</t>
+          <t>ERBB4</t>
         </is>
       </c>
       <c r="C23" t="b">
@@ -1286,12 +1286,12 @@
       </c>
       <c r="F23" t="inlineStr">
         <is>
-          <t>OPC.5</t>
+          <t>Oligo.1</t>
         </is>
       </c>
       <c r="G23" t="inlineStr">
         <is>
-          <t>OPC.5 specific Enrich genes t= 7.33</t>
+          <t>Oligo.1 specific Enrich genes t= 5.58</t>
         </is>
       </c>
       <c r="H23" t="b">
@@ -1306,12 +1306,12 @@
     <row r="24">
       <c r="A24" t="inlineStr">
         <is>
-          <t>ENSG00000144369</t>
+          <t>ENSG00000182473</t>
         </is>
       </c>
       <c r="B24" t="inlineStr">
         <is>
-          <t>FAM171B</t>
+          <t>EXOC7</t>
         </is>
       </c>
       <c r="C24" t="b">
@@ -1327,12 +1327,12 @@
       </c>
       <c r="F24" t="inlineStr">
         <is>
-          <t>Astro.1</t>
+          <t>OPC.5</t>
         </is>
       </c>
       <c r="G24" t="inlineStr">
         <is>
-          <t>Astro.1 specific Enrich genes t= 8.3</t>
+          <t>OPC.5 specific Enrich genes t= 7.33</t>
         </is>
       </c>
       <c r="H24" t="b">
@@ -1347,12 +1347,12 @@
     <row r="25">
       <c r="A25" t="inlineStr">
         <is>
-          <t>ENSG00000182263</t>
+          <t>ENSG00000144369</t>
         </is>
       </c>
       <c r="B25" t="inlineStr">
         <is>
-          <t>FIGN</t>
+          <t>FAM171B</t>
         </is>
       </c>
       <c r="C25" t="b">
@@ -1368,12 +1368,12 @@
       </c>
       <c r="F25" t="inlineStr">
         <is>
-          <t>Oligo.1</t>
+          <t>Astro.1</t>
         </is>
       </c>
       <c r="G25" t="inlineStr">
         <is>
-          <t>Oligo.1 specific MR genes - Oligo.1/Oligo.4: 1.143</t>
+          <t>Astro.1 specific Enrich genes t= 8.3</t>
         </is>
       </c>
       <c r="H25" t="b">
@@ -1388,12 +1388,12 @@
     <row r="26">
       <c r="A26" t="inlineStr">
         <is>
-          <t>ENSG00000170345</t>
+          <t>ENSG00000182263</t>
         </is>
       </c>
       <c r="B26" t="inlineStr">
         <is>
-          <t>FOS</t>
+          <t>FIGN</t>
         </is>
       </c>
       <c r="C26" t="b">
@@ -1404,17 +1404,17 @@
       </c>
       <c r="E26" t="inlineStr">
         <is>
-          <t>DEG - carrier</t>
+          <t>Marker - cell type specific</t>
         </is>
       </c>
       <c r="F26" t="inlineStr">
         <is>
-          <t>Oligo.3</t>
+          <t>Oligo.1</t>
         </is>
       </c>
       <c r="G26" t="inlineStr">
         <is>
-          <t>DEG carrier top: Oligo.3 up logFC=2.77, DEG of interest: Oligo.3 up logFC=2.77</t>
+          <t>Oligo.1 specific MR genes - Oligo.1/Oligo.4: 1.143</t>
         </is>
       </c>
       <c r="H26" t="b">
@@ -1429,12 +1429,12 @@
     <row r="27">
       <c r="A27" t="inlineStr">
         <is>
-          <t>ENSG00000177283</t>
+          <t>ENSG00000170345</t>
         </is>
       </c>
       <c r="B27" t="inlineStr">
         <is>
-          <t>FZD8</t>
+          <t>FOS</t>
         </is>
       </c>
       <c r="C27" t="b">
@@ -1445,17 +1445,17 @@
       </c>
       <c r="E27" t="inlineStr">
         <is>
-          <t>DEG - mediation</t>
+          <t>DEG - carrier</t>
         </is>
       </c>
       <c r="F27" t="inlineStr">
         <is>
-          <t>Astro.2</t>
+          <t>Oligo.3</t>
         </is>
       </c>
       <c r="G27" t="inlineStr">
         <is>
-          <t>mediation gene: mediator Astro.2</t>
+          <t>DEG carrier top: Oligo.3 up logFC=2.77, DEG of interest: Oligo.3 up logFC=2.77</t>
         </is>
       </c>
       <c r="H27" t="b">
@@ -1470,12 +1470,12 @@
     <row r="28">
       <c r="A28" t="inlineStr">
         <is>
-          <t>ENSG00000147533</t>
+          <t>ENSG00000177283</t>
         </is>
       </c>
       <c r="B28" t="inlineStr">
         <is>
-          <t>GOLGA7</t>
+          <t>FZD8</t>
         </is>
       </c>
       <c r="C28" t="b">
@@ -1486,17 +1486,17 @@
       </c>
       <c r="E28" t="inlineStr">
         <is>
-          <t>Marker - cell type specific</t>
+          <t>DEG - mediation</t>
         </is>
       </c>
       <c r="F28" t="inlineStr">
         <is>
-          <t>Oligo.1</t>
+          <t>Astro.2</t>
         </is>
       </c>
       <c r="G28" t="inlineStr">
         <is>
-          <t>Oligo.1 specific Enrich genes t= 5.54</t>
+          <t>mediation gene: mediator Astro.2</t>
         </is>
       </c>
       <c r="H28" t="b">
@@ -1511,12 +1511,12 @@
     <row r="29">
       <c r="A29" t="inlineStr">
         <is>
-          <t>ENSG00000175265</t>
+          <t>ENSG00000231373</t>
         </is>
       </c>
       <c r="B29" t="inlineStr">
         <is>
-          <t>GOLGA8A</t>
+          <t>GNA14-AS1</t>
         </is>
       </c>
       <c r="C29" t="b">
@@ -1527,17 +1527,17 @@
       </c>
       <c r="E29" t="inlineStr">
         <is>
-          <t>DEG - carrier</t>
+          <t>Marker - cell type global</t>
         </is>
       </c>
       <c r="F29" t="inlineStr">
         <is>
-          <t>Excit.L5.2</t>
+          <t>Astro.1</t>
         </is>
       </c>
       <c r="G29" t="inlineStr">
         <is>
-          <t>DEG carrier top:  Excit.L5.2 up</t>
+          <t>globl MR genes -  Astro.1/Astro.3: 1.372</t>
         </is>
       </c>
       <c r="H29" t="b">
@@ -1545,19 +1545,19 @@
       </c>
       <c r="I29" t="inlineStr">
         <is>
-          <t>Mar2</t>
+          <t>Mar6</t>
         </is>
       </c>
     </row>
     <row r="30">
       <c r="A30" t="inlineStr">
         <is>
-          <t>ENSG00000235984</t>
+          <t>ENSG00000147533</t>
         </is>
       </c>
       <c r="B30" t="inlineStr">
         <is>
-          <t>GPC5-AS1</t>
+          <t>GOLGA7</t>
         </is>
       </c>
       <c r="C30" t="b">
@@ -1573,12 +1573,12 @@
       </c>
       <c r="F30" t="inlineStr">
         <is>
-          <t>Excit.L5.2</t>
+          <t>Oligo.1</t>
         </is>
       </c>
       <c r="G30" t="inlineStr">
         <is>
-          <t>Excit.L5.2 specific MR genes - Excit.L5.2/Excit.L5.1: 13.028</t>
+          <t>Oligo.1 specific Enrich genes t= 5.54</t>
         </is>
       </c>
       <c r="H30" t="b">
@@ -1593,12 +1593,12 @@
     <row r="31">
       <c r="A31" t="inlineStr">
         <is>
-          <t>ENSG00000183098</t>
+          <t>ENSG00000175265</t>
         </is>
       </c>
       <c r="B31" t="inlineStr">
         <is>
-          <t>GPC6</t>
+          <t>GOLGA8A</t>
         </is>
       </c>
       <c r="C31" t="b">
@@ -1609,17 +1609,17 @@
       </c>
       <c r="E31" t="inlineStr">
         <is>
-          <t>MOFA - Factor3</t>
+          <t>DEG - carrier</t>
         </is>
       </c>
       <c r="F31" t="inlineStr">
         <is>
-          <t>Oligo.3</t>
+          <t>Excit.L5.2</t>
         </is>
       </c>
       <c r="G31" t="inlineStr">
         <is>
-          <t>MOFA Oligo.3 Factor3+</t>
+          <t>DEG carrier top: Excit.L5.2 up</t>
         </is>
       </c>
       <c r="H31" t="b">
@@ -1627,40 +1627,40 @@
       </c>
       <c r="I31" t="inlineStr">
         <is>
-          <t>Feb27</t>
+          <t>Mar2</t>
         </is>
       </c>
     </row>
     <row r="32">
       <c r="A32" t="inlineStr">
         <is>
-          <t>ENSG00000150625</t>
+          <t>ENSG00000235984</t>
         </is>
       </c>
       <c r="B32" t="inlineStr">
         <is>
-          <t>GPM6A</t>
+          <t>GPC5-AS1</t>
         </is>
       </c>
       <c r="C32" t="b">
         <v>0</v>
       </c>
       <c r="D32">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="E32" t="inlineStr">
         <is>
-          <t>DEG - mediation, Marker - cell type specific</t>
+          <t>Marker - cell type specific</t>
         </is>
       </c>
       <c r="F32" t="inlineStr">
         <is>
-          <t>Oligo.3</t>
+          <t>Excit.L5.2</t>
         </is>
       </c>
       <c r="G32" t="inlineStr">
         <is>
-          <t>Oligo.3 specific Enrich genes t= 9.66, mediation gene: outcome Oligo.3</t>
+          <t>Excit.L5.2 specific MR genes - Excit.L5.2/Excit.L5.1: 13.028</t>
         </is>
       </c>
       <c r="H32" t="b">
@@ -1675,12 +1675,12 @@
     <row r="33">
       <c r="A33" t="inlineStr">
         <is>
-          <t>ENSG00000244734</t>
+          <t>ENSG00000183098</t>
         </is>
       </c>
       <c r="B33" t="inlineStr">
         <is>
-          <t>HBB</t>
+          <t>GPC6</t>
         </is>
       </c>
       <c r="C33" t="b">
@@ -1691,7 +1691,7 @@
       </c>
       <c r="E33" t="inlineStr">
         <is>
-          <t>DEG - ancestry</t>
+          <t>MOFA - Factor3</t>
         </is>
       </c>
       <c r="F33" t="inlineStr">
@@ -1701,7 +1701,7 @@
       </c>
       <c r="G33" t="inlineStr">
         <is>
-          <t>DEG carrier top: Oligo.3 AA_down</t>
+          <t>MOFA Oligo.3 Factor3+</t>
         </is>
       </c>
       <c r="H33" t="b">
@@ -1716,33 +1716,33 @@
     <row r="34">
       <c r="A34" t="inlineStr">
         <is>
-          <t>ENSG00000148357</t>
+          <t>ENSG00000150625</t>
         </is>
       </c>
       <c r="B34" t="inlineStr">
         <is>
-          <t>HMCN2</t>
+          <t>GPM6A</t>
         </is>
       </c>
       <c r="C34" t="b">
         <v>0</v>
       </c>
       <c r="D34">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="E34" t="inlineStr">
         <is>
-          <t>Marker - cell type specific</t>
+          <t>DEG - mediation, Marker - cell type specific</t>
         </is>
       </c>
       <c r="F34" t="inlineStr">
         <is>
-          <t>Excit.L5.2</t>
+          <t>Oligo.3</t>
         </is>
       </c>
       <c r="G34" t="inlineStr">
         <is>
-          <t>Excit.L5.2 specific MR genes - Excit.L5.2/Excit.L6b: 13.871</t>
+          <t>Oligo.3 specific Enrich genes t= 9.66, mediation gene: outcome Oligo.3</t>
         </is>
       </c>
       <c r="H34" t="b">
@@ -1757,12 +1757,12 @@
     <row r="35">
       <c r="A35" t="inlineStr">
         <is>
-          <t>ENSG00000233429</t>
+          <t>ENSG00000244734</t>
         </is>
       </c>
       <c r="B35" t="inlineStr">
         <is>
-          <t>HOTAIRM1</t>
+          <t>HBB</t>
         </is>
       </c>
       <c r="C35" t="b">
@@ -1773,17 +1773,17 @@
       </c>
       <c r="E35" t="inlineStr">
         <is>
-          <t>Marker - cell type specific</t>
+          <t>DEG - ancestry</t>
         </is>
       </c>
       <c r="F35" t="inlineStr">
         <is>
-          <t>Excit.L5.2</t>
+          <t>Oligo.3</t>
         </is>
       </c>
       <c r="G35" t="inlineStr">
         <is>
-          <t>Excit.L5.2 specific Enrich genes t= 16.54</t>
+          <t>DEG carrier top: Oligo.3 AA_down</t>
         </is>
       </c>
       <c r="H35" t="b">
@@ -1798,12 +1798,12 @@
     <row r="36">
       <c r="A36" t="inlineStr">
         <is>
-          <t>ENSG00000185811</t>
+          <t>ENSG00000148357</t>
         </is>
       </c>
       <c r="B36" t="inlineStr">
         <is>
-          <t>IKZF1</t>
+          <t>HMCN2</t>
         </is>
       </c>
       <c r="C36" t="b">
@@ -1814,17 +1814,17 @@
       </c>
       <c r="E36" t="inlineStr">
         <is>
-          <t>DEG - carrier</t>
+          <t>Marker - cell type specific</t>
         </is>
       </c>
       <c r="F36" t="inlineStr">
         <is>
-          <t>Oligo.3</t>
+          <t>Excit.L5.2</t>
         </is>
       </c>
       <c r="G36" t="inlineStr">
         <is>
-          <t>DEG carrier top: Oligo.3 up logFC=2.75</t>
+          <t>Excit.L5.2 specific MR genes - Excit.L5.2/Excit.L6b: 13.871</t>
         </is>
       </c>
       <c r="H36" t="b">
@@ -1839,12 +1839,12 @@
     <row r="37">
       <c r="A37" t="inlineStr">
         <is>
-          <t>ENSG00000134352</t>
+          <t>ENSG00000233429</t>
         </is>
       </c>
       <c r="B37" t="inlineStr">
         <is>
-          <t>IL6ST</t>
+          <t>HOTAIRM1</t>
         </is>
       </c>
       <c r="C37" t="b">
@@ -1855,17 +1855,17 @@
       </c>
       <c r="E37" t="inlineStr">
         <is>
-          <t>DEG - mediation</t>
+          <t>Marker - cell type specific</t>
         </is>
       </c>
       <c r="F37" t="inlineStr">
         <is>
-          <t>Astro.3</t>
+          <t>Excit.L5.2</t>
         </is>
       </c>
       <c r="G37" t="inlineStr">
         <is>
-          <t>mediation gene: mediator Astro.3</t>
+          <t>Excit.L5.2 specific Enrich genes t= 16.54</t>
         </is>
       </c>
       <c r="H37" t="b">
@@ -1880,12 +1880,12 @@
     <row r="38">
       <c r="A38" t="inlineStr">
         <is>
-          <t>ENSG00000138448</t>
+          <t>ENSG00000185811</t>
         </is>
       </c>
       <c r="B38" t="inlineStr">
         <is>
-          <t>ITGAV</t>
+          <t>IKZF1</t>
         </is>
       </c>
       <c r="C38" t="b">
@@ -1896,17 +1896,17 @@
       </c>
       <c r="E38" t="inlineStr">
         <is>
-          <t>Marker - cell type specific</t>
+          <t>DEG - carrier</t>
         </is>
       </c>
       <c r="F38" t="inlineStr">
         <is>
-          <t>Oligo.2</t>
+          <t>Oligo.3</t>
         </is>
       </c>
       <c r="G38" t="inlineStr">
         <is>
-          <t>Oligo.2 specific MR genes - Oligo.2/Oligo.1: 1.663</t>
+          <t>DEG carrier top: Oligo.3 up logFC=2.75</t>
         </is>
       </c>
       <c r="H38" t="b">
@@ -1921,12 +1921,12 @@
     <row r="39">
       <c r="A39" t="inlineStr">
         <is>
-          <t>ENSG00000108773</t>
+          <t>ENSG00000134352</t>
         </is>
       </c>
       <c r="B39" t="inlineStr">
         <is>
-          <t>KAT2A</t>
+          <t>IL6ST</t>
         </is>
       </c>
       <c r="C39" t="b">
@@ -1937,17 +1937,17 @@
       </c>
       <c r="E39" t="inlineStr">
         <is>
-          <t>DEG - ancestry</t>
+          <t>DEG - mediation</t>
         </is>
       </c>
       <c r="F39" t="inlineStr">
         <is>
-          <t>Oligo.3</t>
+          <t>Astro.3</t>
         </is>
       </c>
       <c r="G39" t="inlineStr">
         <is>
-          <t>DEG Ancestry op: Oligo.3 AA_up*-EA_down</t>
+          <t>mediation gene: mediator Astro.3</t>
         </is>
       </c>
       <c r="H39" t="b">
@@ -1962,12 +1962,12 @@
     <row r="40">
       <c r="A40" t="inlineStr">
         <is>
-          <t>ENSG00000184408</t>
+          <t>ENSG00000138448</t>
         </is>
       </c>
       <c r="B40" t="inlineStr">
         <is>
-          <t>KCND2</t>
+          <t>ITGAV</t>
         </is>
       </c>
       <c r="C40" t="b">
@@ -1983,12 +1983,12 @@
       </c>
       <c r="F40" t="inlineStr">
         <is>
-          <t>Oligo.3</t>
+          <t>Oligo.2</t>
         </is>
       </c>
       <c r="G40" t="inlineStr">
         <is>
-          <t>Oligo.3 specific Enrich genes t= 9.2</t>
+          <t>Oligo.2 specific MR genes - Oligo.2/Oligo.1: 1.663</t>
         </is>
       </c>
       <c r="H40" t="b">
@@ -2003,12 +2003,12 @@
     <row r="41">
       <c r="A41" t="inlineStr">
         <is>
-          <t>ENSG00000162989</t>
+          <t>ENSG00000108773</t>
         </is>
       </c>
       <c r="B41" t="inlineStr">
         <is>
-          <t>KCNJ3</t>
+          <t>KAT2A</t>
         </is>
       </c>
       <c r="C41" t="b">
@@ -2019,7 +2019,7 @@
       </c>
       <c r="E41" t="inlineStr">
         <is>
-          <t>Marker - cell type specific</t>
+          <t>DEG - ancestry</t>
         </is>
       </c>
       <c r="F41" t="inlineStr">
@@ -2029,7 +2029,7 @@
       </c>
       <c r="G41" t="inlineStr">
         <is>
-          <t>Oligo.3 specific Enrich genes t= 9.5</t>
+          <t>DEG Ancestry op: Oligo.3 AA_up*-EA_down</t>
         </is>
       </c>
       <c r="H41" t="b">
@@ -2044,12 +2044,12 @@
     <row r="42">
       <c r="A42" t="inlineStr">
         <is>
-          <t>ENSG00000234665</t>
+          <t>ENSG00000184408</t>
         </is>
       </c>
       <c r="B42" t="inlineStr">
         <is>
-          <t>LERFS</t>
+          <t>KCND2</t>
         </is>
       </c>
       <c r="C42" t="b">
@@ -2060,7 +2060,7 @@
       </c>
       <c r="E42" t="inlineStr">
         <is>
-          <t>DEG - carrier</t>
+          <t>Marker - cell type specific</t>
         </is>
       </c>
       <c r="F42" t="inlineStr">
@@ -2070,7 +2070,7 @@
       </c>
       <c r="G42" t="inlineStr">
         <is>
-          <t>DEG carrier top: Oligo.3 down logFC=-1.39</t>
+          <t>Oligo.3 specific Enrich genes t= 9.2</t>
         </is>
       </c>
       <c r="H42" t="b">
@@ -2085,12 +2085,12 @@
     <row r="43">
       <c r="A43" t="inlineStr">
         <is>
-          <t>ENSG00000233237</t>
+          <t>ENSG00000162989</t>
         </is>
       </c>
       <c r="B43" t="inlineStr">
         <is>
-          <t>LINC00472</t>
+          <t>KCNJ3</t>
         </is>
       </c>
       <c r="C43" t="b">
@@ -2101,7 +2101,7 @@
       </c>
       <c r="E43" t="inlineStr">
         <is>
-          <t>DEG - ancestry</t>
+          <t>Marker - cell type specific</t>
         </is>
       </c>
       <c r="F43" t="inlineStr">
@@ -2111,7 +2111,7 @@
       </c>
       <c r="G43" t="inlineStr">
         <is>
-          <t>DEG Ancestry op: Oligo.3 AA_down-EA_up*</t>
+          <t>Oligo.3 specific Enrich genes t= 9.5</t>
         </is>
       </c>
       <c r="H43" t="b">
@@ -2126,12 +2126,12 @@
     <row r="44">
       <c r="A44" t="inlineStr">
         <is>
-          <t>ENSG00000230876</t>
+          <t>ENSG00000234665</t>
         </is>
       </c>
       <c r="B44" t="inlineStr">
         <is>
-          <t>LINC00486</t>
+          <t>LERFS</t>
         </is>
       </c>
       <c r="C44" t="b">
@@ -2147,12 +2147,12 @@
       </c>
       <c r="F44" t="inlineStr">
         <is>
-          <t>Excit.L5.2</t>
+          <t>Oligo.3</t>
         </is>
       </c>
       <c r="G44" t="inlineStr">
         <is>
-          <t>DEG carrier top:  Excit.L5.2 up</t>
+          <t>DEG carrier top: Oligo.3 down logFC=-1.39</t>
         </is>
       </c>
       <c r="H44" t="b">
@@ -2160,19 +2160,19 @@
       </c>
       <c r="I44" t="inlineStr">
         <is>
-          <t>Mar2</t>
+          <t>Feb27</t>
         </is>
       </c>
     </row>
     <row r="45">
       <c r="A45" t="inlineStr">
         <is>
-          <t>ENSG00000257585</t>
+          <t>ENSG00000233237</t>
         </is>
       </c>
       <c r="B45" t="inlineStr">
         <is>
-          <t>LINC00609</t>
+          <t>LINC00472</t>
         </is>
       </c>
       <c r="C45" t="b">
@@ -2183,17 +2183,17 @@
       </c>
       <c r="E45" t="inlineStr">
         <is>
-          <t>Marker - cell type specific</t>
+          <t>DEG - ancestry</t>
         </is>
       </c>
       <c r="F45" t="inlineStr">
         <is>
-          <t>Oligo.2</t>
+          <t>Oligo.3</t>
         </is>
       </c>
       <c r="G45" t="inlineStr">
         <is>
-          <t>Oligo.2 specific Enrich genes t= 10.42</t>
+          <t>DEG Ancestry op: Oligo.3 AA_down-EA_up*</t>
         </is>
       </c>
       <c r="H45" t="b">
@@ -2208,12 +2208,12 @@
     <row r="46">
       <c r="A46" t="inlineStr">
         <is>
-          <t>ENSG00000281186</t>
+          <t>ENSG00000230876</t>
         </is>
       </c>
       <c r="B46" t="inlineStr">
         <is>
-          <t>LINC00706</t>
+          <t>LINC00486</t>
         </is>
       </c>
       <c r="C46" t="b">
@@ -2224,17 +2224,17 @@
       </c>
       <c r="E46" t="inlineStr">
         <is>
-          <t>DEG - ancestry</t>
+          <t>DEG - carrier</t>
         </is>
       </c>
       <c r="F46" t="inlineStr">
         <is>
-          <t>Oligo.3</t>
+          <t>Excit.L5.2</t>
         </is>
       </c>
       <c r="G46" t="inlineStr">
         <is>
-          <t>DEG carrier top: Oligo.3 AA_down</t>
+          <t>DEG carrier top: Excit.L5.2 up</t>
         </is>
       </c>
       <c r="H46" t="b">
@@ -2242,30 +2242,30 @@
       </c>
       <c r="I46" t="inlineStr">
         <is>
-          <t>Feb27</t>
+          <t>Mar2</t>
         </is>
       </c>
     </row>
     <row r="47">
       <c r="A47" t="inlineStr">
         <is>
-          <t>ENSG00000238217</t>
+          <t>ENSG00000257585</t>
         </is>
       </c>
       <c r="B47" t="inlineStr">
         <is>
-          <t>LINC01877</t>
+          <t>LINC00609</t>
         </is>
       </c>
       <c r="C47" t="b">
         <v>0</v>
       </c>
       <c r="D47">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="E47" t="inlineStr">
         <is>
-          <t>Marker - cell type global, Marker - cell type specific</t>
+          <t>Marker - cell type specific</t>
         </is>
       </c>
       <c r="F47" t="inlineStr">
@@ -2275,7 +2275,7 @@
       </c>
       <c r="G47" t="inlineStr">
         <is>
-          <t>globl MR genes -  Oligo.2/Oligo.1: 1.743, Oligo.2 specific MR genes - Oligo.2/Oligo.1: 1.743</t>
+          <t>Oligo.2 specific Enrich genes t= 10.42</t>
         </is>
       </c>
       <c r="H47" t="b">
@@ -2290,12 +2290,12 @@
     <row r="48">
       <c r="A48" t="inlineStr">
         <is>
-          <t>ENSG00000254401</t>
+          <t>ENSG00000281186</t>
         </is>
       </c>
       <c r="B48" t="inlineStr">
         <is>
-          <t>LINC02752</t>
+          <t>LINC00706</t>
         </is>
       </c>
       <c r="C48" t="b">
@@ -2306,17 +2306,17 @@
       </c>
       <c r="E48" t="inlineStr">
         <is>
-          <t>Marker - cell type global</t>
+          <t>DEG - ancestry</t>
         </is>
       </c>
       <c r="F48" t="inlineStr">
         <is>
-          <t>Excit.L5.2</t>
+          <t>Oligo.3</t>
         </is>
       </c>
       <c r="G48" t="inlineStr">
         <is>
-          <t>globl MR genes -  Excit.L5.2/Excit.L2_5.2: 10.797</t>
+          <t>DEG carrier top: Oligo.3 AA_down</t>
         </is>
       </c>
       <c r="H48" t="b">
@@ -2331,33 +2331,33 @@
     <row r="49">
       <c r="A49" t="inlineStr">
         <is>
-          <t>ENSG00000174482</t>
+          <t>ENSG00000238217</t>
         </is>
       </c>
       <c r="B49" t="inlineStr">
         <is>
-          <t>LINGO2</t>
+          <t>LINC01877</t>
         </is>
       </c>
       <c r="C49" t="b">
         <v>0</v>
       </c>
       <c r="D49">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="E49" t="inlineStr">
         <is>
-          <t>Marker - cell type specific</t>
+          <t>Marker - cell type global, Marker - cell type specific</t>
         </is>
       </c>
       <c r="F49" t="inlineStr">
         <is>
-          <t>Oligo.3</t>
+          <t>Oligo.2</t>
         </is>
       </c>
       <c r="G49" t="inlineStr">
         <is>
-          <t>Oligo.3 specific Enrich genes t= 9.09</t>
+          <t>globl MR genes -  Oligo.2/Oligo.1: 1.743, Oligo.2 specific MR genes - Oligo.2/Oligo.1: 1.743</t>
         </is>
       </c>
       <c r="H49" t="b">
@@ -2372,12 +2372,12 @@
     <row r="50">
       <c r="A50" t="inlineStr">
         <is>
-          <t>ENSG00000048540</t>
+          <t>ENSG00000254401</t>
         </is>
       </c>
       <c r="B50" t="inlineStr">
         <is>
-          <t>LMO3</t>
+          <t>LINC02752</t>
         </is>
       </c>
       <c r="C50" t="b">
@@ -2388,17 +2388,17 @@
       </c>
       <c r="E50" t="inlineStr">
         <is>
-          <t>Marker - cell type specific</t>
+          <t>Marker - cell type global</t>
         </is>
       </c>
       <c r="F50" t="inlineStr">
         <is>
-          <t>Astro.1</t>
+          <t>Excit.L5.2</t>
         </is>
       </c>
       <c r="G50" t="inlineStr">
         <is>
-          <t>Astro.1 specific Enrich genes t= 8.73</t>
+          <t>globl MR genes -  Excit.L5.2/Excit.L2_5.2: 10.797</t>
         </is>
       </c>
       <c r="H50" t="b">
@@ -2413,12 +2413,12 @@
     <row r="51">
       <c r="A51" t="inlineStr">
         <is>
-          <t>ENSG00000198121</t>
+          <t>ENSG00000174482</t>
         </is>
       </c>
       <c r="B51" t="inlineStr">
         <is>
-          <t>LPAR1</t>
+          <t>LINGO2</t>
         </is>
       </c>
       <c r="C51" t="b">
@@ -2429,17 +2429,17 @@
       </c>
       <c r="E51" t="inlineStr">
         <is>
-          <t>DEG - carrier</t>
+          <t>Marker - cell type specific</t>
         </is>
       </c>
       <c r="F51" t="inlineStr">
         <is>
-          <t>Excit.L2_5.1</t>
+          <t>Oligo.3</t>
         </is>
       </c>
       <c r="G51" t="inlineStr">
         <is>
-          <t>DEG carrier top:  Excit.L2_5.1 down</t>
+          <t>Oligo.3 specific Enrich genes t= 9.09</t>
         </is>
       </c>
       <c r="H51" t="b">
@@ -2447,19 +2447,19 @@
       </c>
       <c r="I51" t="inlineStr">
         <is>
-          <t>Mar2</t>
+          <t>Feb27</t>
         </is>
       </c>
     </row>
     <row r="52">
       <c r="A52" t="inlineStr">
         <is>
-          <t>ENSG00000235448</t>
+          <t>ENSG00000048540</t>
         </is>
       </c>
       <c r="B52" t="inlineStr">
         <is>
-          <t>LURAP1L-AS1</t>
+          <t>LMO3</t>
         </is>
       </c>
       <c r="C52" t="b">
@@ -2470,17 +2470,17 @@
       </c>
       <c r="E52" t="inlineStr">
         <is>
-          <t>DEG - carrier</t>
+          <t>Marker - cell type specific</t>
         </is>
       </c>
       <c r="F52" t="inlineStr">
         <is>
-          <t>Oligo.3</t>
+          <t>Astro.1</t>
         </is>
       </c>
       <c r="G52" t="inlineStr">
         <is>
-          <t>DEG carrier top: Oligo.3 down logFC=-1.48</t>
+          <t>Astro.1 specific Enrich genes t= 8.73</t>
         </is>
       </c>
       <c r="H52" t="b">
@@ -2495,12 +2495,12 @@
     <row r="53">
       <c r="A53" t="inlineStr">
         <is>
-          <t>ENSG00000102316</t>
+          <t>ENSG00000198121</t>
         </is>
       </c>
       <c r="B53" t="inlineStr">
         <is>
-          <t>MAGED2</t>
+          <t>LPAR1</t>
         </is>
       </c>
       <c r="C53" t="b">
@@ -2511,17 +2511,17 @@
       </c>
       <c r="E53" t="inlineStr">
         <is>
-          <t>DEG - ancestry</t>
+          <t>DEG - carrier</t>
         </is>
       </c>
       <c r="F53" t="inlineStr">
         <is>
-          <t>Oligo.3</t>
+          <t>Excit.L2_5.1</t>
         </is>
       </c>
       <c r="G53" t="inlineStr">
         <is>
-          <t>DEG Ancestry op: Oligo.3 AA_up-EA_down*</t>
+          <t>DEG carrier top: Excit.L2_5.1 down</t>
         </is>
       </c>
       <c r="H53" t="b">
@@ -2529,19 +2529,19 @@
       </c>
       <c r="I53" t="inlineStr">
         <is>
-          <t>Feb27</t>
+          <t>Mar2</t>
         </is>
       </c>
     </row>
     <row r="54">
       <c r="A54" t="inlineStr">
         <is>
-          <t>ENSG00000186868</t>
+          <t>ENSG00000173988</t>
         </is>
       </c>
       <c r="B54" t="inlineStr">
         <is>
-          <t>MAPT</t>
+          <t>LRRC63</t>
         </is>
       </c>
       <c r="C54" t="b">
@@ -2552,17 +2552,17 @@
       </c>
       <c r="E54" t="inlineStr">
         <is>
-          <t>DEG - carrier</t>
+          <t>Marker - cell type global</t>
         </is>
       </c>
       <c r="F54" t="inlineStr">
         <is>
-          <t>Oligo.3</t>
+          <t>Oligo.2</t>
         </is>
       </c>
       <c r="G54" t="inlineStr">
         <is>
-          <t>DEG of interest: Oligo.3 down logFC=-0.56</t>
+          <t>globl MR genes -  Oligo.2/Oligo.1: 1.457</t>
         </is>
       </c>
       <c r="H54" t="b">
@@ -2570,40 +2570,40 @@
       </c>
       <c r="I54" t="inlineStr">
         <is>
-          <t>Feb27</t>
+          <t>Mar6</t>
         </is>
       </c>
     </row>
     <row r="55">
       <c r="A55" t="inlineStr">
         <is>
-          <t>ENSG00000197971</t>
+          <t>ENSG00000235448</t>
         </is>
       </c>
       <c r="B55" t="inlineStr">
         <is>
-          <t>MBP</t>
+          <t>LURAP1L-AS1</t>
         </is>
       </c>
       <c r="C55" t="b">
         <v>0</v>
       </c>
       <c r="D55">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="E55" t="inlineStr">
         <is>
-          <t>DEG - carrier, DEG - mediation, Marker - SpD</t>
+          <t>DEG - carrier</t>
         </is>
       </c>
       <c r="F55" t="inlineStr">
         <is>
-          <t>Oligo.3, WM.uf~Sp09D07</t>
+          <t>Oligo.3</t>
         </is>
       </c>
       <c r="G55" t="inlineStr">
         <is>
-          <t>SpD Enrich gene t=6.53, DEG of interest: Oligo.3 down logFC=-0.69, mediation gene: outcome Oligo.3</t>
+          <t>DEG carrier top: Oligo.3 down logFC=-1.48</t>
         </is>
       </c>
       <c r="H55" t="b">
@@ -2618,12 +2618,12 @@
     <row r="56">
       <c r="A56" t="inlineStr">
         <is>
-          <t>ENSG00000214548</t>
+          <t>ENSG00000102316</t>
         </is>
       </c>
       <c r="B56" t="inlineStr">
         <is>
-          <t>MEG3</t>
+          <t>MAGED2</t>
         </is>
       </c>
       <c r="C56" t="b">
@@ -2634,17 +2634,17 @@
       </c>
       <c r="E56" t="inlineStr">
         <is>
-          <t>Marker - cell type specific</t>
+          <t>DEG - ancestry</t>
         </is>
       </c>
       <c r="F56" t="inlineStr">
         <is>
-          <t>OPC.5</t>
+          <t>Oligo.3</t>
         </is>
       </c>
       <c r="G56" t="inlineStr">
         <is>
-          <t>OPC.5 specific MR genes - OPC.5/OPC.2: 1.019</t>
+          <t>DEG Ancestry op: Oligo.3 AA_up-EA_down*</t>
         </is>
       </c>
       <c r="H56" t="b">
@@ -2659,12 +2659,12 @@
     <row r="57">
       <c r="A57" t="inlineStr">
         <is>
-          <t>ENSG00000225783</t>
+          <t>ENSG00000186868</t>
         </is>
       </c>
       <c r="B57" t="inlineStr">
         <is>
-          <t>MIAT</t>
+          <t>MAPT</t>
         </is>
       </c>
       <c r="C57" t="b">
@@ -2675,7 +2675,7 @@
       </c>
       <c r="E57" t="inlineStr">
         <is>
-          <t>DEG - ancestry</t>
+          <t>DEG - carrier</t>
         </is>
       </c>
       <c r="F57" t="inlineStr">
@@ -2685,7 +2685,7 @@
       </c>
       <c r="G57" t="inlineStr">
         <is>
-          <t>DEG carrier top: Oligo.3 AA_up</t>
+          <t>DEG of interest: Oligo.3 down logFC=-0.56</t>
         </is>
       </c>
       <c r="H57" t="b">
@@ -2700,33 +2700,33 @@
     <row r="58">
       <c r="A58" t="inlineStr">
         <is>
-          <t>ENSG00000136297</t>
+          <t>ENSG00000197971</t>
         </is>
       </c>
       <c r="B58" t="inlineStr">
         <is>
-          <t>MMD2</t>
+          <t>MBP</t>
         </is>
       </c>
       <c r="C58" t="b">
         <v>0</v>
       </c>
       <c r="D58">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="E58" t="inlineStr">
         <is>
-          <t>Marker - cell type specific</t>
+          <t>DEG - carrier, DEG - mediation, Marker - SpD</t>
         </is>
       </c>
       <c r="F58" t="inlineStr">
         <is>
-          <t>Astro.2</t>
+          <t>Oligo.3, WM.uf~Sp09D07</t>
         </is>
       </c>
       <c r="G58" t="inlineStr">
         <is>
-          <t>Astro.2 specific MR genes - Astro.2/Astro.5: 1.004</t>
+          <t>SpD Enrich gene t=6.53, DEG of interest: Oligo.3 down logFC=-0.69, mediation gene: outcome Oligo.3</t>
         </is>
       </c>
       <c r="H58" t="b">
@@ -2741,12 +2741,12 @@
     <row r="59">
       <c r="A59" t="inlineStr">
         <is>
-          <t>ENSG00000198938</t>
+          <t>ENSG00000214548</t>
         </is>
       </c>
       <c r="B59" t="inlineStr">
         <is>
-          <t>MT-CO3</t>
+          <t>MEG3</t>
         </is>
       </c>
       <c r="C59" t="b">
@@ -2762,12 +2762,12 @@
       </c>
       <c r="F59" t="inlineStr">
         <is>
-          <t>Oligo.3</t>
+          <t>OPC.5</t>
         </is>
       </c>
       <c r="G59" t="inlineStr">
         <is>
-          <t>Oligo.3 specific MR genes - Oligo.3/Oligo.4: 1.141</t>
+          <t>OPC.5 specific MR genes - OPC.5/OPC.2: 1.019</t>
         </is>
       </c>
       <c r="H59" t="b">
@@ -2782,12 +2782,12 @@
     <row r="60">
       <c r="A60" t="inlineStr">
         <is>
-          <t>ENSG00000198727</t>
+          <t>ENSG00000225783</t>
         </is>
       </c>
       <c r="B60" t="inlineStr">
         <is>
-          <t>MT-CYB</t>
+          <t>MIAT</t>
         </is>
       </c>
       <c r="C60" t="b">
@@ -2798,17 +2798,17 @@
       </c>
       <c r="E60" t="inlineStr">
         <is>
-          <t>Marker - cell type specific</t>
+          <t>DEG - ancestry</t>
         </is>
       </c>
       <c r="F60" t="inlineStr">
         <is>
-          <t>Excit.L2_5.1</t>
+          <t>Oligo.3</t>
         </is>
       </c>
       <c r="G60" t="inlineStr">
         <is>
-          <t>Excit.L2_5.1 specific MR genes - Excit.L2_5.1/Excit.L6b: 1.175</t>
+          <t>DEG carrier top: Oligo.3 AA_up</t>
         </is>
       </c>
       <c r="H60" t="b">
@@ -2823,12 +2823,12 @@
     <row r="61">
       <c r="A61" t="inlineStr">
         <is>
-          <t>ENSG00000198888</t>
+          <t>ENSG00000136297</t>
         </is>
       </c>
       <c r="B61" t="inlineStr">
         <is>
-          <t>MT-ND1</t>
+          <t>MMD2</t>
         </is>
       </c>
       <c r="C61" t="b">
@@ -2844,12 +2844,12 @@
       </c>
       <c r="F61" t="inlineStr">
         <is>
-          <t>Excit.L2_5.1</t>
+          <t>Astro.2</t>
         </is>
       </c>
       <c r="G61" t="inlineStr">
         <is>
-          <t>Excit.L2_5.1 specific MR genes - Excit.L2_5.1/Excit.L6b: 1.201</t>
+          <t>Astro.2 specific MR genes - Astro.2/Astro.5: 1.004</t>
         </is>
       </c>
       <c r="H61" t="b">
@@ -2864,33 +2864,33 @@
     <row r="62">
       <c r="A62" t="inlineStr">
         <is>
-          <t>ENSG00000198886</t>
+          <t>ENSG00000198938</t>
         </is>
       </c>
       <c r="B62" t="inlineStr">
         <is>
-          <t>MT-ND4</t>
+          <t>MT-CO3</t>
         </is>
       </c>
       <c r="C62" t="b">
         <v>0</v>
       </c>
       <c r="D62">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="E62" t="inlineStr">
         <is>
-          <t>DEG - carrier</t>
+          <t>DEG - carrier, Marker - cell type specific</t>
         </is>
       </c>
       <c r="F62" t="inlineStr">
         <is>
-          <t>Excit.L5.2</t>
+          <t>Excit.L5.2, Oligo.3</t>
         </is>
       </c>
       <c r="G62" t="inlineStr">
         <is>
-          <t>DEG carrier top:  Excit.L5.2 down</t>
+          <t>Oligo.3 specific MR genes - Oligo.3/Oligo.4: 1.141, DEG carrier top: Excit.L5.2 down</t>
         </is>
       </c>
       <c r="H62" t="b">
@@ -2898,19 +2898,19 @@
       </c>
       <c r="I62" t="inlineStr">
         <is>
-          <t>Mar2</t>
+          <t>Feb27</t>
         </is>
       </c>
     </row>
     <row r="63">
       <c r="A63" t="inlineStr">
         <is>
-          <t>ENSG00000128654</t>
+          <t>ENSG00000198727</t>
         </is>
       </c>
       <c r="B63" t="inlineStr">
         <is>
-          <t>MTX2</t>
+          <t>MT-CYB</t>
         </is>
       </c>
       <c r="C63" t="b">
@@ -2926,12 +2926,12 @@
       </c>
       <c r="F63" t="inlineStr">
         <is>
-          <t>Oligo.2</t>
+          <t>Excit.L2_5.1</t>
         </is>
       </c>
       <c r="G63" t="inlineStr">
         <is>
-          <t>Oligo.2 specific Enrich genes t= 11.38</t>
+          <t>Excit.L2_5.1 specific MR genes - Excit.L2_5.1/Excit.L6b: 1.175</t>
         </is>
       </c>
       <c r="H63" t="b">
@@ -2946,12 +2946,12 @@
     <row r="64">
       <c r="A64" t="inlineStr">
         <is>
-          <t>ENSG00000186310</t>
+          <t>ENSG00000198888</t>
         </is>
       </c>
       <c r="B64" t="inlineStr">
         <is>
-          <t>NAP1L3</t>
+          <t>MT-ND1</t>
         </is>
       </c>
       <c r="C64" t="b">
@@ -2962,17 +2962,17 @@
       </c>
       <c r="E64" t="inlineStr">
         <is>
-          <t>DEG - mediation</t>
+          <t>Marker - cell type specific</t>
         </is>
       </c>
       <c r="F64" t="inlineStr">
         <is>
-          <t>Oligo.3</t>
+          <t>Excit.L2_5.1</t>
         </is>
       </c>
       <c r="G64" t="inlineStr">
         <is>
-          <t>mediation gene: outcome Oligo.3</t>
+          <t>Excit.L2_5.1 specific MR genes - Excit.L2_5.1/Excit.L6b: 1.201</t>
         </is>
       </c>
       <c r="H64" t="b">
@@ -2987,12 +2987,12 @@
     <row r="65">
       <c r="A65" t="inlineStr">
         <is>
-          <t>ENSG00000166342</t>
+          <t>ENSG00000128654</t>
         </is>
       </c>
       <c r="B65" t="inlineStr">
         <is>
-          <t>NETO1</t>
+          <t>MTX2</t>
         </is>
       </c>
       <c r="C65" t="b">
@@ -3003,17 +3003,17 @@
       </c>
       <c r="E65" t="inlineStr">
         <is>
-          <t>DEG - mediation</t>
+          <t>Marker - cell type specific</t>
         </is>
       </c>
       <c r="F65" t="inlineStr">
         <is>
-          <t>Astro.2</t>
+          <t>Oligo.2</t>
         </is>
       </c>
       <c r="G65" t="inlineStr">
         <is>
-          <t>mediation gene: mediator Astro.2</t>
+          <t>Oligo.2 specific Enrich genes t= 11.38</t>
         </is>
       </c>
       <c r="H65" t="b">
@@ -3028,12 +3028,12 @@
     <row r="66">
       <c r="A66" t="inlineStr">
         <is>
-          <t>ENSG00000169760</t>
+          <t>ENSG00000186310</t>
         </is>
       </c>
       <c r="B66" t="inlineStr">
         <is>
-          <t>NLGN1</t>
+          <t>NAP1L3</t>
         </is>
       </c>
       <c r="C66" t="b">
@@ -3044,7 +3044,7 @@
       </c>
       <c r="E66" t="inlineStr">
         <is>
-          <t>DEGs - LR</t>
+          <t>DEG - mediation</t>
         </is>
       </c>
       <c r="F66" t="inlineStr">
@@ -3054,7 +3054,7 @@
       </c>
       <c r="G66" t="inlineStr">
         <is>
-          <t>DEG LR interactions: NLGN1 -&gt; NRXN1,NLGN1 -&gt; NRXN3,NRXN1 -&gt; NLGN1,NRXN3 -&gt; NLGN1</t>
+          <t>mediation gene: outcome Oligo.3</t>
         </is>
       </c>
       <c r="H66" t="b">
@@ -3069,12 +3069,12 @@
     <row r="67">
       <c r="A67" t="inlineStr">
         <is>
-          <t>ENSG00000221890</t>
+          <t>ENSG00000166342</t>
         </is>
       </c>
       <c r="B67" t="inlineStr">
         <is>
-          <t>NPTXR</t>
+          <t>NETO1</t>
         </is>
       </c>
       <c r="C67" t="b">
@@ -3090,12 +3090,12 @@
       </c>
       <c r="F67" t="inlineStr">
         <is>
-          <t>Astro.1</t>
+          <t>Astro.2</t>
         </is>
       </c>
       <c r="G67" t="inlineStr">
         <is>
-          <t>mediation gene: mediator Astro.1</t>
+          <t>mediation gene: mediator Astro.2</t>
         </is>
       </c>
       <c r="H67" t="b">
@@ -3110,12 +3110,12 @@
     <row r="68">
       <c r="A68" t="inlineStr">
         <is>
-          <t>ENSG00000185737</t>
+          <t>ENSG00000169760</t>
         </is>
       </c>
       <c r="B68" t="inlineStr">
         <is>
-          <t>NRG3</t>
+          <t>NLGN1</t>
         </is>
       </c>
       <c r="C68" t="b">
@@ -3136,7 +3136,7 @@
       </c>
       <c r="G68" t="inlineStr">
         <is>
-          <t>DEG LR interactions: NRG3 -&gt; ERBB3</t>
+          <t>DEG LR interactions: NLGN1 -&gt; NRXN1,NLGN1 -&gt; NRXN3,NRXN1 -&gt; NLGN1,NRXN3 -&gt; NLGN1</t>
         </is>
       </c>
       <c r="H68" t="b">
@@ -3151,12 +3151,12 @@
     <row r="69">
       <c r="A69" t="inlineStr">
         <is>
-          <t>ENSG00000179915</t>
+          <t>ENSG00000221890</t>
         </is>
       </c>
       <c r="B69" t="inlineStr">
         <is>
-          <t>NRXN1</t>
+          <t>NPTXR</t>
         </is>
       </c>
       <c r="C69" t="b">
@@ -3167,17 +3167,17 @@
       </c>
       <c r="E69" t="inlineStr">
         <is>
-          <t>DEGs - LR</t>
+          <t>DEG - mediation</t>
         </is>
       </c>
       <c r="F69" t="inlineStr">
         <is>
-          <t>Oligo.3</t>
+          <t>Astro.1</t>
         </is>
       </c>
       <c r="G69" t="inlineStr">
         <is>
-          <t>DEG LR interactions: NLGN1 -&gt; NRXN1,NLGN4X -&gt; NRXN1,NRXN1 -&gt; NLGN1,NXPH1 -&gt; NRXN1</t>
+          <t>mediation gene: mediator Astro.1</t>
         </is>
       </c>
       <c r="H69" t="b">
@@ -3192,12 +3192,12 @@
     <row r="70">
       <c r="A70" t="inlineStr">
         <is>
-          <t>ENSG00000021645</t>
+          <t>ENSG00000185737</t>
         </is>
       </c>
       <c r="B70" t="inlineStr">
         <is>
-          <t>NRXN3</t>
+          <t>NRG3</t>
         </is>
       </c>
       <c r="C70" t="b">
@@ -3218,7 +3218,7 @@
       </c>
       <c r="G70" t="inlineStr">
         <is>
-          <t>DEG LR interactions: NLGN1 -&gt; NRXN3,NRXN3 -&gt; NLGN1,NXPH1 -&gt; NRXN3</t>
+          <t>DEG LR interactions: NRG3 -&gt; ERBB3</t>
         </is>
       </c>
       <c r="H70" t="b">
@@ -3233,23 +3233,23 @@
     <row r="71">
       <c r="A71" t="inlineStr">
         <is>
-          <t>ENSG00000140538</t>
+          <t>ENSG00000179915</t>
         </is>
       </c>
       <c r="B71" t="inlineStr">
         <is>
-          <t>NTRK3</t>
+          <t>NRXN1</t>
         </is>
       </c>
       <c r="C71" t="b">
         <v>0</v>
       </c>
       <c r="D71">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="E71" t="inlineStr">
         <is>
-          <t>DEGs - LR, Marker - cell type specific</t>
+          <t>DEGs - LR</t>
         </is>
       </c>
       <c r="F71" t="inlineStr">
@@ -3259,7 +3259,7 @@
       </c>
       <c r="G71" t="inlineStr">
         <is>
-          <t>Oligo.3 specific Enrich genes t= 9.07, DEG LR interactions: NTRK3 -&gt; PTPRD</t>
+          <t>DEG LR interactions: NLGN1 -&gt; NRXN1,NLGN4X -&gt; NRXN1,NRXN1 -&gt; NLGN1,NXPH1 -&gt; NRXN1</t>
         </is>
       </c>
       <c r="H71" t="b">
@@ -3274,12 +3274,12 @@
     <row r="72">
       <c r="A72" t="inlineStr">
         <is>
-          <t>ENSG00000228474</t>
+          <t>ENSG00000021645</t>
         </is>
       </c>
       <c r="B72" t="inlineStr">
         <is>
-          <t>OST4</t>
+          <t>NRXN3</t>
         </is>
       </c>
       <c r="C72" t="b">
@@ -3290,17 +3290,17 @@
       </c>
       <c r="E72" t="inlineStr">
         <is>
-          <t>Marker - SpD</t>
+          <t>DEGs - LR</t>
         </is>
       </c>
       <c r="F72" t="inlineStr">
         <is>
-          <t>LD~Sp09D02</t>
+          <t>Oligo.3</t>
         </is>
       </c>
       <c r="G72" t="inlineStr">
         <is>
-          <t>SpD MeanRatio gene: LD~Sp09D02/L2.3~Sp09D01: 1.109</t>
+          <t>DEG LR interactions: NLGN1 -&gt; NRXN3,NRXN3 -&gt; NLGN1,NXPH1 -&gt; NRXN3</t>
         </is>
       </c>
       <c r="H72" t="b">
@@ -3315,12 +3315,12 @@
     <row r="73">
       <c r="A73" t="inlineStr">
         <is>
-          <t>ENSG00000100836</t>
+          <t>ENSG00000140538</t>
         </is>
       </c>
       <c r="B73" t="inlineStr">
         <is>
-          <t>PABPN1</t>
+          <t>NTRK3</t>
         </is>
       </c>
       <c r="C73" t="b">
@@ -3331,17 +3331,17 @@
       </c>
       <c r="E73" t="inlineStr">
         <is>
-          <t>Marker - cell type specific</t>
+          <t>DEGs - LR, Marker - cell type specific</t>
         </is>
       </c>
       <c r="F73" t="inlineStr">
         <is>
-          <t>Astro.3, Excit.L2_5.1</t>
+          <t>Oligo.3</t>
         </is>
       </c>
       <c r="G73" t="inlineStr">
         <is>
-          <t>Astro.3 specific MR genes - Astro.3/Astro.1: 1.046, Excit.L2_5.1 specific Enrich genes t= 9.16</t>
+          <t>Oligo.3 specific Enrich genes t= 9.07, DEG LR interactions: NTRK3 -&gt; PTPRD</t>
         </is>
       </c>
       <c r="H73" t="b">
@@ -3356,12 +3356,12 @@
     <row r="74">
       <c r="A74" t="inlineStr">
         <is>
-          <t>ENSG00000228842</t>
+          <t>ENSG00000228474</t>
         </is>
       </c>
       <c r="B74" t="inlineStr">
         <is>
-          <t>PCDH9-AS2</t>
+          <t>OST4</t>
         </is>
       </c>
       <c r="C74" t="b">
@@ -3372,17 +3372,17 @@
       </c>
       <c r="E74" t="inlineStr">
         <is>
-          <t>Marker - cell type specific</t>
+          <t>Marker - SpD</t>
         </is>
       </c>
       <c r="F74" t="inlineStr">
         <is>
-          <t>Astro.1</t>
+          <t>LD~Sp09D02</t>
         </is>
       </c>
       <c r="G74" t="inlineStr">
         <is>
-          <t>Astro.1 specific MR genes - Astro.1/Astro.3: 1.486</t>
+          <t>SpD MeanRatio gene: LD~Sp09D02/L2.3~Sp09D01: 1.109</t>
         </is>
       </c>
       <c r="H74" t="b">
@@ -3397,12 +3397,12 @@
     <row r="75">
       <c r="A75" t="inlineStr">
         <is>
-          <t>ENSG00000123560</t>
+          <t>ENSG00000100836</t>
         </is>
       </c>
       <c r="B75" t="inlineStr">
         <is>
-          <t>PLP1</t>
+          <t>PABPN1</t>
         </is>
       </c>
       <c r="C75" t="b">
@@ -3413,17 +3413,17 @@
       </c>
       <c r="E75" t="inlineStr">
         <is>
-          <t>DEG - carrier, Marker - cell type specific</t>
+          <t>Marker - cell type specific</t>
         </is>
       </c>
       <c r="F75" t="inlineStr">
         <is>
-          <t>Excit.L2_5.1, Oligo.3</t>
+          <t>Astro.3, Excit.L2_5.1</t>
         </is>
       </c>
       <c r="G75" t="inlineStr">
         <is>
-          <t>Excit.L2_5.1 specific Enrich genes t= 8.05, DEG of interest: Oligo.3 down logFC=-0.93</t>
+          <t>Astro.3 specific MR genes - Astro.3/Astro.1: 1.046, Excit.L2_5.1 specific Enrich genes t= 9.16</t>
         </is>
       </c>
       <c r="H75" t="b">
@@ -3438,12 +3438,12 @@
     <row r="76">
       <c r="A76" t="inlineStr">
         <is>
-          <t>ENSG00000117600</t>
+          <t>ENSG00000228842</t>
         </is>
       </c>
       <c r="B76" t="inlineStr">
         <is>
-          <t>PLPPR4</t>
+          <t>PCDH9-AS2</t>
         </is>
       </c>
       <c r="C76" t="b">
@@ -3454,7 +3454,7 @@
       </c>
       <c r="E76" t="inlineStr">
         <is>
-          <t>DEG - mediation</t>
+          <t>Marker - cell type specific</t>
         </is>
       </c>
       <c r="F76" t="inlineStr">
@@ -3464,7 +3464,7 @@
       </c>
       <c r="G76" t="inlineStr">
         <is>
-          <t>mediation gene: mediator Astro.1</t>
+          <t>Astro.1 specific MR genes - Astro.1/Astro.3: 1.486</t>
         </is>
       </c>
       <c r="H76" t="b">
@@ -3479,33 +3479,33 @@
     <row r="77">
       <c r="A77" t="inlineStr">
         <is>
-          <t>ENSG00000107317</t>
+          <t>ENSG00000123560</t>
         </is>
       </c>
       <c r="B77" t="inlineStr">
         <is>
-          <t>PTGDS</t>
+          <t>PLP1</t>
         </is>
       </c>
       <c r="C77" t="b">
         <v>0</v>
       </c>
       <c r="D77">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="E77" t="inlineStr">
         <is>
-          <t>Marker - cell type specific</t>
+          <t>DEG - carrier, Marker - cell type specific</t>
         </is>
       </c>
       <c r="F77" t="inlineStr">
         <is>
-          <t>Astro.2</t>
+          <t>Excit.L2_5.1, Oligo.3</t>
         </is>
       </c>
       <c r="G77" t="inlineStr">
         <is>
-          <t>Astro.2 specific MR genes - Astro.2/Astro.5: 1.01, Astro.2 specific Enrich genes t= 4.92</t>
+          <t>Excit.L2_5.1 specific Enrich genes t= 8.05, DEG of interest: Oligo.3 down logFC=-0.93</t>
         </is>
       </c>
       <c r="H77" t="b">
@@ -3520,12 +3520,12 @@
     <row r="78">
       <c r="A78" t="inlineStr">
         <is>
-          <t>ENSG00000153707</t>
+          <t>ENSG00000117600</t>
         </is>
       </c>
       <c r="B78" t="inlineStr">
         <is>
-          <t>PTPRD</t>
+          <t>PLPPR4</t>
         </is>
       </c>
       <c r="C78" t="b">
@@ -3536,17 +3536,17 @@
       </c>
       <c r="E78" t="inlineStr">
         <is>
-          <t>DEGs - LR</t>
+          <t>DEG - mediation</t>
         </is>
       </c>
       <c r="F78" t="inlineStr">
         <is>
-          <t>Oligo.3</t>
+          <t>Astro.1</t>
         </is>
       </c>
       <c r="G78" t="inlineStr">
         <is>
-          <t>DEG LR interactions: IL1RAPL1 -&gt; PTPRD,NTRK3 -&gt; PTPRD</t>
+          <t>mediation gene: mediator Astro.1</t>
         </is>
       </c>
       <c r="H78" t="b">
@@ -3561,12 +3561,12 @@
     <row r="79">
       <c r="A79" t="inlineStr">
         <is>
-          <t>ENSG00000079974</t>
+          <t>ENSG00000107317</t>
         </is>
       </c>
       <c r="B79" t="inlineStr">
         <is>
-          <t>RABL2B</t>
+          <t>PTGDS</t>
         </is>
       </c>
       <c r="C79" t="b">
@@ -3577,17 +3577,17 @@
       </c>
       <c r="E79" t="inlineStr">
         <is>
-          <t>DEG - ancestry</t>
+          <t>Marker - cell type specific</t>
         </is>
       </c>
       <c r="F79" t="inlineStr">
         <is>
-          <t>Oligo.3</t>
+          <t>Astro.2</t>
         </is>
       </c>
       <c r="G79" t="inlineStr">
         <is>
-          <t>DEG Ancestry op: Oligo.3 AA_up-EA_down*</t>
+          <t>Astro.2 specific MR genes - Astro.2/Astro.5: 1.01, Astro.2 specific Enrich genes t= 4.92</t>
         </is>
       </c>
       <c r="H79" t="b">
@@ -3602,12 +3602,12 @@
     <row r="80">
       <c r="A80" t="inlineStr">
         <is>
-          <t>ENSG00000129538</t>
+          <t>ENSG00000153707</t>
         </is>
       </c>
       <c r="B80" t="inlineStr">
         <is>
-          <t>RNASE1</t>
+          <t>PTPRD</t>
         </is>
       </c>
       <c r="C80" t="b">
@@ -3618,7 +3618,7 @@
       </c>
       <c r="E80" t="inlineStr">
         <is>
-          <t>MOFA - Factor3</t>
+          <t>DEGs - LR</t>
         </is>
       </c>
       <c r="F80" t="inlineStr">
@@ -3628,7 +3628,7 @@
       </c>
       <c r="G80" t="inlineStr">
         <is>
-          <t>MOFA Oligo.3 Factor3-</t>
+          <t>DEG LR interactions: IL1RAPL1 -&gt; PTPRD,NTRK3 -&gt; PTPRD</t>
         </is>
       </c>
       <c r="H80" t="b">
@@ -3636,19 +3636,19 @@
       </c>
       <c r="I80" t="inlineStr">
         <is>
-          <t>Mar2</t>
+          <t>Feb27</t>
         </is>
       </c>
     </row>
     <row r="81">
       <c r="A81" t="inlineStr">
         <is>
-          <t>ENSG00000177954</t>
+          <t>ENSG00000079974</t>
         </is>
       </c>
       <c r="B81" t="inlineStr">
         <is>
-          <t>RPS27</t>
+          <t>RABL2B</t>
         </is>
       </c>
       <c r="C81" t="b">
@@ -3659,17 +3659,17 @@
       </c>
       <c r="E81" t="inlineStr">
         <is>
-          <t>Marker - cell type specific</t>
+          <t>DEG - ancestry</t>
         </is>
       </c>
       <c r="F81" t="inlineStr">
         <is>
-          <t>Astro.3</t>
+          <t>Oligo.3</t>
         </is>
       </c>
       <c r="G81" t="inlineStr">
         <is>
-          <t>Astro.3 specific MR genes - Astro.3/Astro.2: 1.109</t>
+          <t>DEG Ancestry op: Oligo.3 AA_up-EA_down*</t>
         </is>
       </c>
       <c r="H81" t="b">
@@ -3684,12 +3684,12 @@
     <row r="82">
       <c r="A82" t="inlineStr">
         <is>
-          <t>ENSG00000250722</t>
+          <t>ENSG00000129538</t>
         </is>
       </c>
       <c r="B82" t="inlineStr">
         <is>
-          <t>SELENOP</t>
+          <t>RNASE1</t>
         </is>
       </c>
       <c r="C82" t="b">
@@ -3718,19 +3718,19 @@
       </c>
       <c r="I82" t="inlineStr">
         <is>
-          <t>Feb27</t>
+          <t>Mar2</t>
         </is>
       </c>
     </row>
     <row r="83">
       <c r="A83" t="inlineStr">
         <is>
-          <t>ENSG00000137872</t>
+          <t>ENSG00000177954</t>
         </is>
       </c>
       <c r="B83" t="inlineStr">
         <is>
-          <t>SEMA6D</t>
+          <t>RPS27</t>
         </is>
       </c>
       <c r="C83" t="b">
@@ -3746,12 +3746,12 @@
       </c>
       <c r="F83" t="inlineStr">
         <is>
-          <t>Oligo.1</t>
+          <t>Astro.3</t>
         </is>
       </c>
       <c r="G83" t="inlineStr">
         <is>
-          <t>Oligo.1 specific MR genes - Oligo.1/Oligo.2: 1.179</t>
+          <t>Astro.3 specific MR genes - Astro.3/Astro.2: 1.109</t>
         </is>
       </c>
       <c r="H83" t="b">
@@ -3766,12 +3766,12 @@
     <row r="84">
       <c r="A84" t="inlineStr">
         <is>
-          <t>ENSG00000100359</t>
+          <t>ENSG00000250722</t>
         </is>
       </c>
       <c r="B84" t="inlineStr">
         <is>
-          <t>SGSM3</t>
+          <t>SELENOP</t>
         </is>
       </c>
       <c r="C84" t="b">
@@ -3782,7 +3782,7 @@
       </c>
       <c r="E84" t="inlineStr">
         <is>
-          <t>DEG - ancestry</t>
+          <t>MOFA - Factor3</t>
         </is>
       </c>
       <c r="F84" t="inlineStr">
@@ -3792,7 +3792,7 @@
       </c>
       <c r="G84" t="inlineStr">
         <is>
-          <t>DEG Ancestry op: Oligo.3 AA_up*-EA_down</t>
+          <t>MOFA Oligo.3 Factor3-</t>
         </is>
       </c>
       <c r="H84" t="b">
@@ -3807,12 +3807,12 @@
     <row r="85">
       <c r="A85" t="inlineStr">
         <is>
-          <t>ENSG00000155886</t>
+          <t>ENSG00000137872</t>
         </is>
       </c>
       <c r="B85" t="inlineStr">
         <is>
-          <t>SLC24A2</t>
+          <t>SEMA6D</t>
         </is>
       </c>
       <c r="C85" t="b">
@@ -3828,12 +3828,12 @@
       </c>
       <c r="F85" t="inlineStr">
         <is>
-          <t>Astro.3</t>
+          <t>Oligo.1</t>
         </is>
       </c>
       <c r="G85" t="inlineStr">
         <is>
-          <t>Astro.3 specific Enrich genes t= 8.18</t>
+          <t>Oligo.1 specific MR genes - Oligo.1/Oligo.2: 1.179</t>
         </is>
       </c>
       <c r="H85" t="b">
@@ -3848,12 +3848,12 @@
     <row r="86">
       <c r="A86" t="inlineStr">
         <is>
-          <t>ENSG00000080493</t>
+          <t>ENSG00000100359</t>
         </is>
       </c>
       <c r="B86" t="inlineStr">
         <is>
-          <t>SLC4A4</t>
+          <t>SGSM3</t>
         </is>
       </c>
       <c r="C86" t="b">
@@ -3864,7 +3864,7 @@
       </c>
       <c r="E86" t="inlineStr">
         <is>
-          <t>MOFA - Factor3</t>
+          <t>DEG - ancestry</t>
         </is>
       </c>
       <c r="F86" t="inlineStr">
@@ -3874,7 +3874,7 @@
       </c>
       <c r="G86" t="inlineStr">
         <is>
-          <t>MOFA Oligo.3 Factor3+</t>
+          <t>DEG Ancestry op: Oligo.3 AA_up*-EA_down</t>
         </is>
       </c>
       <c r="H86" t="b">
@@ -3889,12 +3889,12 @@
     <row r="87">
       <c r="A87" t="inlineStr">
         <is>
-          <t>ENSG00000158865</t>
+          <t>ENSG00000155886</t>
         </is>
       </c>
       <c r="B87" t="inlineStr">
         <is>
-          <t>SLC5A11</t>
+          <t>SLC24A2</t>
         </is>
       </c>
       <c r="C87" t="b">
@@ -3905,17 +3905,17 @@
       </c>
       <c r="E87" t="inlineStr">
         <is>
-          <t>Marker - cell type global</t>
+          <t>Marker - cell type specific</t>
         </is>
       </c>
       <c r="F87" t="inlineStr">
         <is>
-          <t>Oligo.2</t>
+          <t>Astro.3</t>
         </is>
       </c>
       <c r="G87" t="inlineStr">
         <is>
-          <t>globl MR genes -  Oligo.2/Oligo.5: 1.492</t>
+          <t>Astro.3 specific Enrich genes t= 8.18</t>
         </is>
       </c>
       <c r="H87" t="b">
@@ -3923,19 +3923,19 @@
       </c>
       <c r="I87" t="inlineStr">
         <is>
-          <t>Mar2</t>
+          <t>Feb27</t>
         </is>
       </c>
     </row>
     <row r="88">
       <c r="A88" t="inlineStr">
         <is>
-          <t>ENSG00000104852</t>
+          <t>ENSG00000080493</t>
         </is>
       </c>
       <c r="B88" t="inlineStr">
         <is>
-          <t>SNRNP70</t>
+          <t>SLC4A4</t>
         </is>
       </c>
       <c r="C88" t="b">
@@ -3946,17 +3946,17 @@
       </c>
       <c r="E88" t="inlineStr">
         <is>
-          <t>Marker - cell type specific</t>
+          <t>MOFA - Factor3</t>
         </is>
       </c>
       <c r="F88" t="inlineStr">
         <is>
-          <t>Astro.2</t>
+          <t>Oligo.3</t>
         </is>
       </c>
       <c r="G88" t="inlineStr">
         <is>
-          <t>Astro.2 specific MR genes - Astro.2/Astro.3: 1.023</t>
+          <t>MOFA Oligo.3 Factor3+</t>
         </is>
       </c>
       <c r="H88" t="b">
@@ -3971,12 +3971,12 @@
     <row r="89">
       <c r="A89" t="inlineStr">
         <is>
-          <t>ENSG00000101400</t>
+          <t>ENSG00000104852</t>
         </is>
       </c>
       <c r="B89" t="inlineStr">
         <is>
-          <t>SNTA1</t>
+          <t>SNRNP70</t>
         </is>
       </c>
       <c r="C89" t="b">
@@ -3997,7 +3997,7 @@
       </c>
       <c r="G89" t="inlineStr">
         <is>
-          <t>Astro.2 specific Enrich genes t= 4.98</t>
+          <t>Astro.2 specific MR genes - Astro.2/Astro.3: 1.023</t>
         </is>
       </c>
       <c r="H89" t="b">
@@ -4012,12 +4012,12 @@
     <row r="90">
       <c r="A90" t="inlineStr">
         <is>
-          <t>ENSG00000120451</t>
+          <t>ENSG00000101400</t>
         </is>
       </c>
       <c r="B90" t="inlineStr">
         <is>
-          <t>SNX19</t>
+          <t>SNTA1</t>
         </is>
       </c>
       <c r="C90" t="b">
@@ -4028,17 +4028,17 @@
       </c>
       <c r="E90" t="inlineStr">
         <is>
-          <t>DEG - ancestry</t>
+          <t>Marker - cell type specific</t>
         </is>
       </c>
       <c r="F90" t="inlineStr">
         <is>
-          <t>Oligo.3</t>
+          <t>Astro.2</t>
         </is>
       </c>
       <c r="G90" t="inlineStr">
         <is>
-          <t>DEG Ancestry op: Oligo.3 AA_down*-EA_up</t>
+          <t>Astro.2 specific Enrich genes t= 4.98</t>
         </is>
       </c>
       <c r="H90" t="b">
@@ -4053,12 +4053,12 @@
     <row r="91">
       <c r="A91" t="inlineStr">
         <is>
-          <t>ENSG00000095637</t>
+          <t>ENSG00000120451</t>
         </is>
       </c>
       <c r="B91" t="inlineStr">
         <is>
-          <t>SORBS1</t>
+          <t>SNX19</t>
         </is>
       </c>
       <c r="C91" t="b">
@@ -4069,7 +4069,7 @@
       </c>
       <c r="E91" t="inlineStr">
         <is>
-          <t>DEG - mediation</t>
+          <t>DEG - ancestry</t>
         </is>
       </c>
       <c r="F91" t="inlineStr">
@@ -4079,7 +4079,7 @@
       </c>
       <c r="G91" t="inlineStr">
         <is>
-          <t>mediation gene: outcome Oligo.3</t>
+          <t>DEG Ancestry op: Oligo.3 AA_down*-EA_up</t>
         </is>
       </c>
       <c r="H91" t="b">
@@ -4094,12 +4094,12 @@
     <row r="92">
       <c r="A92" t="inlineStr">
         <is>
-          <t>ENSG00000115415</t>
+          <t>ENSG00000095637</t>
         </is>
       </c>
       <c r="B92" t="inlineStr">
         <is>
-          <t>STAT1</t>
+          <t>SORBS1</t>
         </is>
       </c>
       <c r="C92" t="b">
@@ -4110,7 +4110,7 @@
       </c>
       <c r="E92" t="inlineStr">
         <is>
-          <t>DEG - carrier</t>
+          <t>DEG - mediation</t>
         </is>
       </c>
       <c r="F92" t="inlineStr">
@@ -4120,7 +4120,7 @@
       </c>
       <c r="G92" t="inlineStr">
         <is>
-          <t>DEG of interest: Oligo.3 up logFC=0.8</t>
+          <t>mediation gene: outcome Oligo.3</t>
         </is>
       </c>
       <c r="H92" t="b">
@@ -4135,12 +4135,12 @@
     <row r="93">
       <c r="A93" t="inlineStr">
         <is>
-          <t>ENSG00000138378</t>
+          <t>ENSG00000115415</t>
         </is>
       </c>
       <c r="B93" t="inlineStr">
         <is>
-          <t>STAT4</t>
+          <t>STAT1</t>
         </is>
       </c>
       <c r="C93" t="b">
@@ -4161,7 +4161,7 @@
       </c>
       <c r="G93" t="inlineStr">
         <is>
-          <t>DEG of interest: Oligo.3 up logFC=2.62</t>
+          <t>DEG of interest: Oligo.3 up logFC=0.8</t>
         </is>
       </c>
       <c r="H93" t="b">
@@ -4176,12 +4176,12 @@
     <row r="94">
       <c r="A94" t="inlineStr">
         <is>
-          <t>ENSG00000185518</t>
+          <t>ENSG00000138378</t>
         </is>
       </c>
       <c r="B94" t="inlineStr">
         <is>
-          <t>SV2B</t>
+          <t>STAT4</t>
         </is>
       </c>
       <c r="C94" t="b">
@@ -4192,17 +4192,17 @@
       </c>
       <c r="E94" t="inlineStr">
         <is>
-          <t>DEG - mediation</t>
+          <t>DEG - carrier</t>
         </is>
       </c>
       <c r="F94" t="inlineStr">
         <is>
-          <t>Astro.2</t>
+          <t>Oligo.3</t>
         </is>
       </c>
       <c r="G94" t="inlineStr">
         <is>
-          <t>mediation gene: mediator Astro.2</t>
+          <t>DEG of interest: Oligo.3 up logFC=2.62</t>
         </is>
       </c>
       <c r="H94" t="b">
@@ -4217,12 +4217,12 @@
     <row r="95">
       <c r="A95" t="inlineStr">
         <is>
-          <t>ENSG00000136560</t>
+          <t>ENSG00000185518</t>
         </is>
       </c>
       <c r="B95" t="inlineStr">
         <is>
-          <t>TANK</t>
+          <t>SV2B</t>
         </is>
       </c>
       <c r="C95" t="b">
@@ -4233,17 +4233,17 @@
       </c>
       <c r="E95" t="inlineStr">
         <is>
-          <t>Marker - cell type specific</t>
+          <t>DEG - mediation</t>
         </is>
       </c>
       <c r="F95" t="inlineStr">
         <is>
-          <t>Excit.L5.2</t>
+          <t>Astro.2</t>
         </is>
       </c>
       <c r="G95" t="inlineStr">
         <is>
-          <t>Excit.L5.2 specific Enrich genes t= 13.71</t>
+          <t>mediation gene: mediator Astro.2</t>
         </is>
       </c>
       <c r="H95" t="b">
@@ -4258,12 +4258,12 @@
     <row r="96">
       <c r="A96" t="inlineStr">
         <is>
-          <t>ENSG00000137462</t>
+          <t>ENSG00000136560</t>
         </is>
       </c>
       <c r="B96" t="inlineStr">
         <is>
-          <t>TLR2</t>
+          <t>TANK</t>
         </is>
       </c>
       <c r="C96" t="b">
@@ -4274,17 +4274,17 @@
       </c>
       <c r="E96" t="inlineStr">
         <is>
-          <t>DEG - carrier</t>
+          <t>Marker - cell type specific</t>
         </is>
       </c>
       <c r="F96" t="inlineStr">
         <is>
-          <t>Oligo.3</t>
+          <t>Excit.L5.2</t>
         </is>
       </c>
       <c r="G96" t="inlineStr">
         <is>
-          <t>DEG of interest: Oligo.3 up logFC=1.56</t>
+          <t>Excit.L5.2 specific Enrich genes t= 13.71</t>
         </is>
       </c>
       <c r="H96" t="b">
@@ -4299,12 +4299,12 @@
     <row r="97">
       <c r="A97" t="inlineStr">
         <is>
-          <t>ENSG00000061938</t>
+          <t>ENSG00000137462</t>
         </is>
       </c>
       <c r="B97" t="inlineStr">
         <is>
-          <t>TNK2</t>
+          <t>TLR2</t>
         </is>
       </c>
       <c r="C97" t="b">
@@ -4315,17 +4315,17 @@
       </c>
       <c r="E97" t="inlineStr">
         <is>
-          <t>Marker - cell type specific</t>
+          <t>DEG - carrier</t>
         </is>
       </c>
       <c r="F97" t="inlineStr">
         <is>
-          <t>OPC.5</t>
+          <t>Oligo.3</t>
         </is>
       </c>
       <c r="G97" t="inlineStr">
         <is>
-          <t>OPC.5 specific MR genes - OPC.5/OPC.2: 1.04</t>
+          <t>DEG of interest: Oligo.3 up logFC=1.56</t>
         </is>
       </c>
       <c r="H97" t="b">
@@ -4340,12 +4340,12 @@
     <row r="98">
       <c r="A98" t="inlineStr">
         <is>
-          <t>ENSG00000124900</t>
+          <t>ENSG00000061938</t>
         </is>
       </c>
       <c r="B98" t="inlineStr">
         <is>
-          <t>TRIM51</t>
+          <t>TNK2</t>
         </is>
       </c>
       <c r="C98" t="b">
@@ -4356,17 +4356,17 @@
       </c>
       <c r="E98" t="inlineStr">
         <is>
-          <t>Marker - SpD</t>
+          <t>Marker - cell type specific</t>
         </is>
       </c>
       <c r="F98" t="inlineStr">
         <is>
-          <t>WM.uf_Sp09D07-WM_Sp09D06</t>
+          <t>OPC.5</t>
         </is>
       </c>
       <c r="G98" t="inlineStr">
         <is>
-          <t>SpD pw gene t=7.53</t>
+          <t>OPC.5 specific MR genes - OPC.5/OPC.2: 1.04</t>
         </is>
       </c>
       <c r="H98" t="b">
@@ -4374,7 +4374,7 @@
       </c>
       <c r="I98" t="inlineStr">
         <is>
-          <t>Mar2</t>
+          <t>Feb27</t>
         </is>
       </c>
     </row>
@@ -4489,7 +4489,7 @@
       </c>
       <c r="G101" t="inlineStr">
         <is>
-          <t>DEG carrier top:  Excit.L5.2 down</t>
+          <t>DEG carrier top: Excit.L5.2 down</t>
         </is>
       </c>
       <c r="H101" t="b">

</xml_diff>